<commit_message>
Remove a data da conversa de carreira de toda a aplicação
Sai do modelo de dados, da planilha de coleta (coluna, Leia-me e
importação), do detalhe do candidato e das páginas de metodologia.
Planilha de exemplo regerada sem a coluna, com o mesmo cenário.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E5WdJkUTyiNFgco3uhd6x7
</commit_message>
<xml_diff>
--- a/exemplos/Gazin_Mapa_Sucessorio_EXEMPLO_FICTICIO.xlsx
+++ b/exemplos/Gazin_Mapa_Sucessorio_EXEMPLO_FICTICIO.xlsx
@@ -401,7 +401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:A23"/>
   <cols>
     <col min="1" max="1" width="120.83203125" customWidth="1"/>
   </cols>
@@ -513,22 +513,17 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Interesse, prontidão e mobilidade mudam com o tempo: registre a Data da conversa de carreira (dia/mês/ano, por exemplo 15/09/2026).</v>
+        <v>e-NPS da área 2026: número de -100 a 100, só para quem lidera equipe.</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>e-NPS da área 2026: número de -100 a 100, só para quem lidera equipe.</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="str">
         <v>Corte de aderência: 60 pontos.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A23"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5806,7 +5801,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S219"/>
+  <dimension ref="A1:R219"/>
   <cols>
     <col min="1" max="1" width="40.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -5823,10 +5818,9 @@
     <col min="13" max="13" width="30.83203125" customWidth="1"/>
     <col min="14" max="14" width="29.83203125" customWidth="1"/>
     <col min="15" max="15" width="50.83203125" customWidth="1"/>
-    <col min="16" max="16" width="30.83203125" customWidth="1"/>
-    <col min="17" max="17" width="39.83203125" customWidth="1"/>
-    <col min="18" max="18" width="15.83203125" customWidth="1"/>
-    <col min="19" max="19" width="20.83203125" customWidth="1"/>
+    <col min="16" max="16" width="39.83203125" customWidth="1"/>
+    <col min="17" max="17" width="15.83203125" customWidth="1"/>
+    <col min="18" max="18" width="20.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5876,15 +5870,12 @@
         <v>Possível sucessor da sua posição (nome)</v>
       </c>
       <c r="P1" t="str">
-        <v>Data da conversa de carreira</v>
+        <v>Avaliação de desempenho (ciclo atual)</v>
       </c>
       <c r="Q1" t="str">
-        <v>Avaliação de desempenho (ciclo atual)</v>
+        <v>Lidera equipe</v>
       </c>
       <c r="R1" t="str">
-        <v>Lidera equipe</v>
-      </c>
-      <c r="S1" t="str">
         <v>e-NPS da área 2026</v>
       </c>
     </row>
@@ -5935,15 +5926,12 @@
         <v>João Pedro Cardoso Jardim</v>
       </c>
       <c r="P2" t="str">
-        <v>18/06/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q2" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R2" t="str">
         <v>Sim</v>
       </c>
-      <c r="S2">
+      <c r="R2">
         <v>50</v>
       </c>
     </row>
@@ -5994,15 +5982,12 @@
         <v/>
       </c>
       <c r="P3" t="str">
-        <v>10/08/2026</v>
+        <v>Risco / Baixo Desempenho</v>
       </c>
       <c r="Q3" t="str">
-        <v>Risco / Baixo Desempenho</v>
-      </c>
-      <c r="R3" t="str">
         <v>Sim</v>
       </c>
-      <c r="S3">
+      <c r="R3">
         <v>70</v>
       </c>
     </row>
@@ -6053,15 +6038,12 @@
         <v/>
       </c>
       <c r="P4" t="str">
-        <v>30/07/2026</v>
+        <v>Estrela</v>
       </c>
       <c r="Q4" t="str">
-        <v>Estrela</v>
-      </c>
-      <c r="R4" t="str">
         <v>Sim</v>
       </c>
-      <c r="S4">
+      <c r="R4">
         <v>78</v>
       </c>
     </row>
@@ -6112,15 +6094,12 @@
         <v/>
       </c>
       <c r="P5" t="str">
-        <v>24/08/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q5" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R5" t="str">
         <v>Sim</v>
       </c>
-      <c r="S5">
+      <c r="R5">
         <v>64</v>
       </c>
     </row>
@@ -6171,15 +6150,12 @@
         <v/>
       </c>
       <c r="P6" t="str">
-        <v>08/07/2026</v>
+        <v>Enigma / Questionável</v>
       </c>
       <c r="Q6" t="str">
-        <v>Enigma / Questionável</v>
-      </c>
-      <c r="R6" t="str">
         <v>Sim</v>
       </c>
-      <c r="S6">
+      <c r="R6">
         <v>65</v>
       </c>
     </row>
@@ -6230,15 +6206,12 @@
         <v/>
       </c>
       <c r="P7" t="str">
-        <v>05/08/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q7" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R7" t="str">
         <v>Sim</v>
       </c>
-      <c r="S7">
+      <c r="R7">
         <v>42</v>
       </c>
     </row>
@@ -6289,15 +6262,12 @@
         <v/>
       </c>
       <c r="P8" t="str">
-        <v>04/06/2026</v>
+        <v/>
       </c>
       <c r="Q8" t="str">
-        <v/>
-      </c>
-      <c r="R8" t="str">
         <v>Sim</v>
       </c>
-      <c r="S8">
+      <c r="R8">
         <v>66</v>
       </c>
     </row>
@@ -6348,15 +6318,12 @@
         <v>Bruna Guimarães Queiroz</v>
       </c>
       <c r="P9" t="str">
-        <v>14/07/2026</v>
+        <v>Empregado Sólido / Responsável</v>
       </c>
       <c r="Q9" t="str">
-        <v>Empregado Sólido / Responsável</v>
-      </c>
-      <c r="R9" t="str">
         <v>Sim</v>
       </c>
-      <c r="S9">
+      <c r="R9">
         <v>45</v>
       </c>
     </row>
@@ -6407,15 +6374,12 @@
         <v>Thomas Jefesson Soares de Souza</v>
       </c>
       <c r="P10" t="str">
-        <v>26/07/2026</v>
+        <v>Alto Potencial</v>
       </c>
       <c r="Q10" t="str">
-        <v>Alto Potencial</v>
-      </c>
-      <c r="R10" t="str">
         <v>Sim</v>
       </c>
-      <c r="S10">
+      <c r="R10">
         <v>55</v>
       </c>
     </row>
@@ -6466,15 +6430,12 @@
         <v/>
       </c>
       <c r="P11" t="str">
-        <v>04/07/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q11" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R11" t="str">
         <v>Sim</v>
       </c>
-      <c r="S11">
+      <c r="R11">
         <v>41</v>
       </c>
     </row>
@@ -6525,15 +6486,12 @@
         <v>Joel Borato</v>
       </c>
       <c r="P12" t="str">
-        <v>12/08/2026</v>
+        <v>Estrela</v>
       </c>
       <c r="Q12" t="str">
-        <v>Estrela</v>
-      </c>
-      <c r="R12" t="str">
         <v>Sim</v>
       </c>
-      <c r="S12">
+      <c r="R12">
         <v>69</v>
       </c>
     </row>
@@ -6584,15 +6542,12 @@
         <v>Nicareli Neves</v>
       </c>
       <c r="P13" t="str">
-        <v>06/08/2026</v>
+        <v>Empregado Sólido / Responsável</v>
       </c>
       <c r="Q13" t="str">
-        <v>Empregado Sólido / Responsável</v>
-      </c>
-      <c r="R13" t="str">
         <v>Sim</v>
       </c>
-      <c r="S13">
+      <c r="R13">
         <v>86</v>
       </c>
     </row>
@@ -6643,15 +6598,12 @@
         <v/>
       </c>
       <c r="P14" t="str">
-        <v>06/06/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q14" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R14" t="str">
         <v>Sim</v>
       </c>
-      <c r="S14">
+      <c r="R14">
         <v>29</v>
       </c>
     </row>
@@ -6702,15 +6654,12 @@
         <v/>
       </c>
       <c r="P15" t="str">
-        <v>17/07/2026</v>
+        <v>Empregado Sólido / Responsável</v>
       </c>
       <c r="Q15" t="str">
-        <v>Empregado Sólido / Responsável</v>
-      </c>
-      <c r="R15" t="str">
         <v>Sim</v>
       </c>
-      <c r="S15">
+      <c r="R15">
         <v>74</v>
       </c>
     </row>
@@ -6761,15 +6710,12 @@
         <v>Juliana Rodriguez Ferro</v>
       </c>
       <c r="P16" t="str">
-        <v>05/06/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q16" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R16" t="str">
         <v>Sim</v>
       </c>
-      <c r="S16">
+      <c r="R16">
         <v>26</v>
       </c>
     </row>
@@ -6820,15 +6766,12 @@
         <v/>
       </c>
       <c r="P17" t="str">
-        <v>04/08/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q17" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R17" t="str">
         <v>Sim</v>
       </c>
-      <c r="S17">
+      <c r="R17">
         <v>55</v>
       </c>
     </row>
@@ -6879,15 +6822,12 @@
         <v>Daiane Domingues dos Santos</v>
       </c>
       <c r="P18" t="str">
-        <v>12/07/2026</v>
+        <v>Alto Potencial</v>
       </c>
       <c r="Q18" t="str">
-        <v>Alto Potencial</v>
-      </c>
-      <c r="R18" t="str">
         <v>Sim</v>
       </c>
-      <c r="S18">
+      <c r="R18">
         <v>23</v>
       </c>
     </row>
@@ -6938,15 +6878,12 @@
         <v>Daiane Domingues dos Santos</v>
       </c>
       <c r="P19" t="str">
-        <v>17/09/2026</v>
+        <v>Alto Potencial</v>
       </c>
       <c r="Q19" t="str">
-        <v>Alto Potencial</v>
-      </c>
-      <c r="R19" t="str">
         <v>Sim</v>
       </c>
-      <c r="S19">
+      <c r="R19">
         <v>46</v>
       </c>
     </row>
@@ -6997,15 +6934,12 @@
         <v/>
       </c>
       <c r="P20" t="str">
-        <v>06/06/2026</v>
+        <v>Bom Executor / Especialista</v>
       </c>
       <c r="Q20" t="str">
-        <v>Bom Executor / Especialista</v>
-      </c>
-      <c r="R20" t="str">
         <v>Sim</v>
       </c>
-      <c r="S20">
+      <c r="R20">
         <v>81</v>
       </c>
     </row>
@@ -7056,15 +6990,12 @@
         <v/>
       </c>
       <c r="P21" t="str">
-        <v>27/07/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q21" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R21" t="str">
         <v>Sim</v>
       </c>
-      <c r="S21">
+      <c r="R21">
         <v>91</v>
       </c>
     </row>
@@ -7115,15 +7046,12 @@
         <v/>
       </c>
       <c r="P22" t="str">
-        <v>31/07/2026</v>
+        <v>Enigma / Questionável</v>
       </c>
       <c r="Q22" t="str">
-        <v>Enigma / Questionável</v>
-      </c>
-      <c r="R22" t="str">
         <v>Sim</v>
       </c>
-      <c r="S22">
+      <c r="R22">
         <v>41</v>
       </c>
     </row>
@@ -7174,15 +7102,12 @@
         <v/>
       </c>
       <c r="P23" t="str">
-        <v>15/06/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q23" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R23" t="str">
         <v>Sim</v>
       </c>
-      <c r="S23">
+      <c r="R23">
         <v>58</v>
       </c>
     </row>
@@ -7233,15 +7158,12 @@
         <v>Jeovanir Castro de Souza</v>
       </c>
       <c r="P24" t="str">
-        <v>03/07/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q24" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R24" t="str">
         <v>Sim</v>
       </c>
-      <c r="S24">
+      <c r="R24">
         <v>59</v>
       </c>
     </row>
@@ -7292,15 +7214,12 @@
         <v>Daiane Domingues dos Santos, Raquel Cristina Vidotto Ramos</v>
       </c>
       <c r="P25" t="str">
-        <v>07/07/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q25" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R25" t="str">
         <v>Sim</v>
       </c>
-      <c r="S25">
+      <c r="R25">
         <v>27</v>
       </c>
     </row>
@@ -7351,15 +7270,12 @@
         <v/>
       </c>
       <c r="P26" t="str">
-        <v>10/08/2026</v>
+        <v>Empregado Sólido / Responsável</v>
       </c>
       <c r="Q26" t="str">
-        <v>Empregado Sólido / Responsável</v>
-      </c>
-      <c r="R26" t="str">
         <v>Sim</v>
       </c>
-      <c r="S26">
+      <c r="R26">
         <v>49</v>
       </c>
     </row>
@@ -7410,15 +7326,12 @@
         <v>Lincoln Eduardo Nunes, Eduarda Meireles</v>
       </c>
       <c r="P27" t="str">
-        <v>19/07/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q27" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R27" t="str">
         <v>Sim</v>
       </c>
-      <c r="S27">
+      <c r="R27">
         <v>64</v>
       </c>
     </row>
@@ -7469,15 +7382,12 @@
         <v/>
       </c>
       <c r="P28" t="str">
-        <v>08/08/2026</v>
+        <v>Estrela</v>
       </c>
       <c r="Q28" t="str">
-        <v>Estrela</v>
-      </c>
-      <c r="R28" t="str">
         <v>Sim</v>
       </c>
-      <c r="S28">
+      <c r="R28">
         <v>43</v>
       </c>
     </row>
@@ -7528,15 +7438,12 @@
         <v/>
       </c>
       <c r="P29" t="str">
-        <v>10/09/2026</v>
+        <v>Empregado Eficaz</v>
       </c>
       <c r="Q29" t="str">
-        <v>Empregado Eficaz</v>
-      </c>
-      <c r="R29" t="str">
         <v>Sim</v>
       </c>
-      <c r="S29">
+      <c r="R29">
         <v>59</v>
       </c>
     </row>
@@ -7587,15 +7494,12 @@
         <v/>
       </c>
       <c r="P30" t="str">
-        <v>21/06/2026</v>
+        <v>Empregado Eficaz</v>
       </c>
       <c r="Q30" t="str">
-        <v>Empregado Eficaz</v>
-      </c>
-      <c r="R30" t="str">
         <v>Sim</v>
       </c>
-      <c r="S30">
+      <c r="R30">
         <v>62</v>
       </c>
     </row>
@@ -7646,15 +7550,12 @@
         <v>Andreza Miranda da Silva</v>
       </c>
       <c r="P31" t="str">
-        <v>16/06/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q31" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R31" t="str">
         <v>Sim</v>
       </c>
-      <c r="S31">
+      <c r="R31">
         <v>15</v>
       </c>
     </row>
@@ -7705,15 +7606,12 @@
         <v/>
       </c>
       <c r="P32" t="str">
-        <v>01/08/2026</v>
+        <v>Enigma / Questionável</v>
       </c>
       <c r="Q32" t="str">
-        <v>Enigma / Questionável</v>
-      </c>
-      <c r="R32" t="str">
         <v>Sim</v>
       </c>
-      <c r="S32">
+      <c r="R32">
         <v>-10</v>
       </c>
     </row>
@@ -7764,15 +7662,12 @@
         <v>Elton Fernando Hoshino</v>
       </c>
       <c r="P33" t="str">
-        <v>12/08/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q33" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R33" t="str">
         <v>Sim</v>
       </c>
-      <c r="S33">
+      <c r="R33">
         <v>51</v>
       </c>
     </row>
@@ -7823,15 +7718,12 @@
         <v/>
       </c>
       <c r="P34" t="str">
-        <v>14/09/2026</v>
+        <v>Empregado Eficaz</v>
       </c>
       <c r="Q34" t="str">
-        <v>Empregado Eficaz</v>
-      </c>
-      <c r="R34" t="str">
         <v>Sim</v>
       </c>
-      <c r="S34">
+      <c r="R34">
         <v>38</v>
       </c>
     </row>
@@ -7882,15 +7774,12 @@
         <v/>
       </c>
       <c r="P35" t="str">
-        <v>11/06/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q35" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R35" t="str">
         <v>Sim</v>
       </c>
-      <c r="S35">
+      <c r="R35">
         <v>79</v>
       </c>
     </row>
@@ -7941,15 +7830,12 @@
         <v>Nicareli Neves</v>
       </c>
       <c r="P36" t="str">
-        <v>23/08/2026</v>
+        <v>Risco / Baixo Desempenho</v>
       </c>
       <c r="Q36" t="str">
-        <v>Risco / Baixo Desempenho</v>
-      </c>
-      <c r="R36" t="str">
         <v>Sim</v>
       </c>
-      <c r="S36">
+      <c r="R36">
         <v>23</v>
       </c>
     </row>
@@ -8000,15 +7886,12 @@
         <v/>
       </c>
       <c r="P37" t="str">
-        <v>13/08/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q37" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R37" t="str">
         <v>Sim</v>
       </c>
-      <c r="S37">
+      <c r="R37">
         <v>90</v>
       </c>
     </row>
@@ -8059,15 +7942,12 @@
         <v>Milene Thomaz Romano Gantzel</v>
       </c>
       <c r="P38" t="str">
-        <v>22/08/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q38" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R38" t="str">
         <v>Sim</v>
       </c>
-      <c r="S38">
+      <c r="R38">
         <v>89</v>
       </c>
     </row>
@@ -8118,15 +7998,12 @@
         <v>Beatriz Santos Kroetzler</v>
       </c>
       <c r="P39" t="str">
-        <v>12/09/2026</v>
+        <v>Estrela</v>
       </c>
       <c r="Q39" t="str">
-        <v>Estrela</v>
-      </c>
-      <c r="R39" t="str">
         <v>Sim</v>
       </c>
-      <c r="S39">
+      <c r="R39">
         <v>66</v>
       </c>
     </row>
@@ -8177,15 +8054,12 @@
         <v>Terisley Ferreira</v>
       </c>
       <c r="P40" t="str">
-        <v>05/06/2026</v>
+        <v>Empregado Sólido / Responsável</v>
       </c>
       <c r="Q40" t="str">
-        <v>Empregado Sólido / Responsável</v>
-      </c>
-      <c r="R40" t="str">
         <v>Sim</v>
       </c>
-      <c r="S40">
+      <c r="R40">
         <v>54</v>
       </c>
     </row>
@@ -8236,15 +8110,12 @@
         <v/>
       </c>
       <c r="P41" t="str">
-        <v>10/09/2026</v>
+        <v>Empregado Sólido / Responsável</v>
       </c>
       <c r="Q41" t="str">
-        <v>Empregado Sólido / Responsável</v>
-      </c>
-      <c r="R41" t="str">
         <v>Sim</v>
       </c>
-      <c r="S41">
+      <c r="R41">
         <v>39</v>
       </c>
     </row>
@@ -8295,15 +8166,12 @@
         <v/>
       </c>
       <c r="P42" t="str">
-        <v>29/06/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q42" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R42" t="str">
         <v>Sim</v>
       </c>
-      <c r="S42">
+      <c r="R42">
         <v>7</v>
       </c>
     </row>
@@ -8354,15 +8222,12 @@
         <v>Terisley Rodrigues Ferreira</v>
       </c>
       <c r="P43" t="str">
-        <v>14/09/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q43" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R43" t="str">
         <v>Sim</v>
       </c>
-      <c r="S43">
+      <c r="R43">
         <v>39</v>
       </c>
     </row>
@@ -8413,15 +8278,12 @@
         <v/>
       </c>
       <c r="P44" t="str">
-        <v>06/06/2026</v>
+        <v>Estrela</v>
       </c>
       <c r="Q44" t="str">
-        <v>Estrela</v>
-      </c>
-      <c r="R44" t="str">
         <v>Sim</v>
       </c>
-      <c r="S44">
+      <c r="R44">
         <v>36</v>
       </c>
     </row>
@@ -8472,15 +8334,12 @@
         <v/>
       </c>
       <c r="P45" t="str">
-        <v>07/07/2026</v>
+        <v>Empregado Sólido / Responsável</v>
       </c>
       <c r="Q45" t="str">
-        <v>Empregado Sólido / Responsável</v>
-      </c>
-      <c r="R45" t="str">
         <v>Sim</v>
       </c>
-      <c r="S45">
+      <c r="R45">
         <v>43</v>
       </c>
     </row>
@@ -8531,15 +8390,12 @@
         <v>Leandro Ferreira Paim Mendes</v>
       </c>
       <c r="P46" t="str">
-        <v>16/08/2026</v>
+        <v>Empregado Sólido / Responsável</v>
       </c>
       <c r="Q46" t="str">
-        <v>Empregado Sólido / Responsável</v>
-      </c>
-      <c r="R46" t="str">
         <v>Sim</v>
       </c>
-      <c r="S46">
+      <c r="R46">
         <v>36</v>
       </c>
     </row>
@@ -8590,15 +8446,12 @@
         <v>Guilherme Caetano Gelamos</v>
       </c>
       <c r="P47" t="str">
-        <v>09/06/2026</v>
+        <v>Bom Executor / Especialista</v>
       </c>
       <c r="Q47" t="str">
-        <v>Bom Executor / Especialista</v>
-      </c>
-      <c r="R47" t="str">
         <v>Sim</v>
       </c>
-      <c r="S47">
+      <c r="R47">
         <v>64</v>
       </c>
     </row>
@@ -8649,15 +8502,12 @@
         <v/>
       </c>
       <c r="P48" t="str">
-        <v>15/06/2026</v>
+        <v>Empregado Sólido / Responsável</v>
       </c>
       <c r="Q48" t="str">
-        <v>Empregado Sólido / Responsável</v>
-      </c>
-      <c r="R48" t="str">
         <v>Sim</v>
       </c>
-      <c r="S48">
+      <c r="R48">
         <v>35</v>
       </c>
     </row>
@@ -8708,15 +8558,12 @@
         <v>Bruno Martins, Odimar Antonio de Oliveira</v>
       </c>
       <c r="P49" t="str">
-        <v>18/09/2026</v>
+        <v>Risco / Baixo Desempenho</v>
       </c>
       <c r="Q49" t="str">
-        <v>Risco / Baixo Desempenho</v>
-      </c>
-      <c r="R49" t="str">
         <v>Sim</v>
       </c>
-      <c r="S49">
+      <c r="R49">
         <v>48</v>
       </c>
     </row>
@@ -8767,15 +8614,12 @@
         <v/>
       </c>
       <c r="P50" t="str">
-        <v>12/07/2026</v>
+        <v>Empregado Sólido / Responsável</v>
       </c>
       <c r="Q50" t="str">
-        <v>Empregado Sólido / Responsável</v>
-      </c>
-      <c r="R50" t="str">
         <v>Sim</v>
       </c>
-      <c r="S50">
+      <c r="R50">
         <v>64</v>
       </c>
     </row>
@@ -8826,15 +8670,12 @@
         <v>Max Antunes Cavalheiro</v>
       </c>
       <c r="P51" t="str">
-        <v>10/07/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q51" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R51" t="str">
         <v>Sim</v>
       </c>
-      <c r="S51">
+      <c r="R51">
         <v>42</v>
       </c>
     </row>
@@ -8885,15 +8726,12 @@
         <v/>
       </c>
       <c r="P52" t="str">
-        <v>11/08/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q52" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R52" t="str">
         <v>Sim</v>
       </c>
-      <c r="S52">
+      <c r="R52">
         <v>22</v>
       </c>
     </row>
@@ -8944,15 +8782,12 @@
         <v>Beatriz Santos Kroetzler</v>
       </c>
       <c r="P53" t="str">
-        <v>19/07/2026</v>
+        <v>Enigma / Questionável</v>
       </c>
       <c r="Q53" t="str">
-        <v>Enigma / Questionável</v>
-      </c>
-      <c r="R53" t="str">
         <v>Sim</v>
       </c>
-      <c r="S53">
+      <c r="R53">
         <v>77</v>
       </c>
     </row>
@@ -9003,15 +8838,12 @@
         <v/>
       </c>
       <c r="P54" t="str">
-        <v>09/09/2026</v>
+        <v>Empregado Sólido / Responsável</v>
       </c>
       <c r="Q54" t="str">
-        <v>Empregado Sólido / Responsável</v>
-      </c>
-      <c r="R54" t="str">
         <v>Sim</v>
       </c>
-      <c r="S54">
+      <c r="R54">
         <v>23</v>
       </c>
     </row>
@@ -9062,15 +8894,12 @@
         <v/>
       </c>
       <c r="P55" t="str">
-        <v>02/09/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q55" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R55" t="str">
         <v>Sim</v>
       </c>
-      <c r="S55">
+      <c r="R55">
         <v>69</v>
       </c>
     </row>
@@ -9121,15 +8950,12 @@
         <v>Teilo de Jesus Santana, Beatriz Santos Kroetzler</v>
       </c>
       <c r="P56" t="str">
-        <v>01/07/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q56" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R56" t="str">
         <v>Sim</v>
       </c>
-      <c r="S56">
+      <c r="R56">
         <v>83</v>
       </c>
     </row>
@@ -9180,15 +9006,12 @@
         <v>Teilo de Jesus Santana</v>
       </c>
       <c r="P57" t="str">
-        <v>29/08/2026</v>
+        <v>Empregado Sólido / Responsável</v>
       </c>
       <c r="Q57" t="str">
-        <v>Empregado Sólido / Responsável</v>
-      </c>
-      <c r="R57" t="str">
         <v>Sim</v>
       </c>
-      <c r="S57">
+      <c r="R57">
         <v>14</v>
       </c>
     </row>
@@ -9239,15 +9062,12 @@
         <v/>
       </c>
       <c r="P58" t="str">
-        <v>06/07/2026</v>
+        <v>Alto Potencial</v>
       </c>
       <c r="Q58" t="str">
-        <v>Alto Potencial</v>
-      </c>
-      <c r="R58" t="str">
         <v>Sim</v>
       </c>
-      <c r="S58">
+      <c r="R58">
         <v>74</v>
       </c>
     </row>
@@ -9298,15 +9118,12 @@
         <v>Beatriz Kroetzler, Max Antunes Cavalheiro</v>
       </c>
       <c r="P59" t="str">
-        <v>01/06/2026</v>
+        <v>Estrela</v>
       </c>
       <c r="Q59" t="str">
-        <v>Estrela</v>
-      </c>
-      <c r="R59" t="str">
         <v>Sim</v>
       </c>
-      <c r="S59">
+      <c r="R59">
         <v>75</v>
       </c>
     </row>
@@ -9357,15 +9174,12 @@
         <v>Beatriz Santos Kroetzler</v>
       </c>
       <c r="P60" t="str">
-        <v>10/07/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q60" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R60" t="str">
         <v>Sim</v>
       </c>
-      <c r="S60">
+      <c r="R60">
         <v>38</v>
       </c>
     </row>
@@ -9416,15 +9230,12 @@
         <v>Rogelio Vargas, Neusa Maria Kaiser</v>
       </c>
       <c r="P61" t="str">
-        <v>13/06/2026</v>
+        <v>Estrela</v>
       </c>
       <c r="Q61" t="str">
-        <v>Estrela</v>
-      </c>
-      <c r="R61" t="str">
         <v>Sim</v>
       </c>
-      <c r="S61">
+      <c r="R61">
         <v>39</v>
       </c>
     </row>
@@ -9475,15 +9286,12 @@
         <v/>
       </c>
       <c r="P62" t="str">
-        <v>22/06/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q62" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R62" t="str">
         <v>Sim</v>
       </c>
-      <c r="S62">
+      <c r="R62">
         <v>45</v>
       </c>
     </row>
@@ -9534,15 +9342,12 @@
         <v>Raquel Cristina Vidotto Ramos</v>
       </c>
       <c r="P63" t="str">
-        <v>29/08/2026</v>
+        <v>Bom Executor / Especialista</v>
       </c>
       <c r="Q63" t="str">
-        <v>Bom Executor / Especialista</v>
-      </c>
-      <c r="R63" t="str">
         <v>Sim</v>
       </c>
-      <c r="S63">
+      <c r="R63">
         <v>59</v>
       </c>
     </row>
@@ -9593,15 +9398,12 @@
         <v/>
       </c>
       <c r="P64" t="str">
-        <v>05/08/2026</v>
+        <v>Empregado Sólido / Responsável</v>
       </c>
       <c r="Q64" t="str">
-        <v>Empregado Sólido / Responsável</v>
-      </c>
-      <c r="R64" t="str">
         <v>Sim</v>
       </c>
-      <c r="S64">
+      <c r="R64">
         <v>77</v>
       </c>
     </row>
@@ -9652,15 +9454,12 @@
         <v>Jordy Alesson Souza Monteiro</v>
       </c>
       <c r="P65" t="str">
-        <v>02/08/2026</v>
+        <v>Estrela</v>
       </c>
       <c r="Q65" t="str">
-        <v>Estrela</v>
-      </c>
-      <c r="R65" t="str">
         <v>Sim</v>
       </c>
-      <c r="S65">
+      <c r="R65">
         <v>90</v>
       </c>
     </row>
@@ -9711,15 +9510,12 @@
         <v>Jordy Alesson Souza Monteiro</v>
       </c>
       <c r="P66" t="str">
-        <v>19/07/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q66" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R66" t="str">
         <v>Sim</v>
       </c>
-      <c r="S66">
+      <c r="R66">
         <v>52</v>
       </c>
     </row>
@@ -9770,15 +9566,12 @@
         <v/>
       </c>
       <c r="P67" t="str">
-        <v>15/06/2026</v>
+        <v>Bom Executor / Especialista</v>
       </c>
       <c r="Q67" t="str">
-        <v>Bom Executor / Especialista</v>
-      </c>
-      <c r="R67" t="str">
         <v>Sim</v>
       </c>
-      <c r="S67">
+      <c r="R67">
         <v>45</v>
       </c>
     </row>
@@ -9829,15 +9622,12 @@
         <v/>
       </c>
       <c r="P68" t="str">
-        <v>16/06/2026</v>
+        <v>Enigma / Questionável</v>
       </c>
       <c r="Q68" t="str">
-        <v>Enigma / Questionável</v>
-      </c>
-      <c r="R68" t="str">
         <v>Sim</v>
       </c>
-      <c r="S68">
+      <c r="R68">
         <v>97</v>
       </c>
     </row>
@@ -9888,15 +9678,12 @@
         <v>Murilo Zanella Valadares, Jordy Alesson Souza Monteiro</v>
       </c>
       <c r="P69" t="str">
-        <v>05/07/2026</v>
+        <v>Empregado Sólido / Responsável</v>
       </c>
       <c r="Q69" t="str">
-        <v>Empregado Sólido / Responsável</v>
-      </c>
-      <c r="R69" t="str">
         <v>Sim</v>
       </c>
-      <c r="S69">
+      <c r="R69">
         <v>87</v>
       </c>
     </row>
@@ -9947,15 +9734,12 @@
         <v>Bruna Pacheco Valadares, Neiva Cristiane Bortolato Goncalves</v>
       </c>
       <c r="P70" t="str">
-        <v>01/09/2026</v>
+        <v>Estrela</v>
       </c>
       <c r="Q70" t="str">
-        <v>Estrela</v>
-      </c>
-      <c r="R70" t="str">
         <v>Sim</v>
       </c>
-      <c r="S70">
+      <c r="R70">
         <v>96</v>
       </c>
     </row>
@@ -10006,15 +9790,12 @@
         <v/>
       </c>
       <c r="P71" t="str">
-        <v>21/08/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q71" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R71" t="str">
         <v>Sim</v>
       </c>
-      <c r="S71">
+      <c r="R71">
         <v>98</v>
       </c>
     </row>
@@ -10065,15 +9846,12 @@
         <v>Jordy Alesson Souza Monteiro</v>
       </c>
       <c r="P72" t="str">
-        <v>30/06/2026</v>
+        <v>Risco / Baixo Desempenho</v>
       </c>
       <c r="Q72" t="str">
-        <v>Risco / Baixo Desempenho</v>
-      </c>
-      <c r="R72" t="str">
         <v>Sim</v>
       </c>
-      <c r="S72">
+      <c r="R72">
         <v>46</v>
       </c>
     </row>
@@ -10124,15 +9902,12 @@
         <v>Bruno Rodrigues Martins</v>
       </c>
       <c r="P73" t="str">
-        <v>22/07/2026</v>
+        <v/>
       </c>
       <c r="Q73" t="str">
-        <v/>
-      </c>
-      <c r="R73" t="str">
         <v>Sim</v>
       </c>
-      <c r="S73">
+      <c r="R73">
         <v>77</v>
       </c>
     </row>
@@ -10183,15 +9958,12 @@
         <v>Robson Rodrigues Jacinto</v>
       </c>
       <c r="P74" t="str">
-        <v>07/08/2026</v>
+        <v>Risco / Baixo Desempenho</v>
       </c>
       <c r="Q74" t="str">
-        <v>Risco / Baixo Desempenho</v>
-      </c>
-      <c r="R74" t="str">
         <v>Sim</v>
       </c>
-      <c r="S74">
+      <c r="R74">
         <v>45</v>
       </c>
     </row>
@@ -10242,15 +10014,12 @@
         <v>Bruna Pacheco Valadares, Murilo Zanella Valadares</v>
       </c>
       <c r="P75" t="str">
-        <v>29/08/2026</v>
+        <v>Empregado Sólido / Responsável</v>
       </c>
       <c r="Q75" t="str">
-        <v>Empregado Sólido / Responsável</v>
-      </c>
-      <c r="R75" t="str">
         <v>Sim</v>
       </c>
-      <c r="S75">
+      <c r="R75">
         <v>53</v>
       </c>
     </row>
@@ -10301,15 +10070,12 @@
         <v>Neiva Cristiane Bortolato Goncalves</v>
       </c>
       <c r="P76" t="str">
-        <v>15/09/2026</v>
+        <v>Bom Executor / Especialista</v>
       </c>
       <c r="Q76" t="str">
-        <v>Bom Executor / Especialista</v>
-      </c>
-      <c r="R76" t="str">
         <v>Sim</v>
       </c>
-      <c r="S76">
+      <c r="R76">
         <v>56</v>
       </c>
     </row>
@@ -10360,15 +10126,12 @@
         <v/>
       </c>
       <c r="P77" t="str">
-        <v>07/08/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q77" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R77" t="str">
         <v>Sim</v>
       </c>
-      <c r="S77">
+      <c r="R77">
         <v>40</v>
       </c>
     </row>
@@ -10419,15 +10182,12 @@
         <v/>
       </c>
       <c r="P78" t="str">
-        <v>19/06/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q78" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R78" t="str">
         <v>Sim</v>
       </c>
-      <c r="S78">
+      <c r="R78">
         <v>54</v>
       </c>
     </row>
@@ -10478,15 +10238,12 @@
         <v>Beatriz Kroetzler, Bruno Rodrigues Martins</v>
       </c>
       <c r="P79" t="str">
-        <v>08/07/2026</v>
+        <v>Alto Potencial</v>
       </c>
       <c r="Q79" t="str">
-        <v>Alto Potencial</v>
-      </c>
-      <c r="R79" t="str">
         <v>Sim</v>
       </c>
-      <c r="S79">
+      <c r="R79">
         <v>72</v>
       </c>
     </row>
@@ -10537,15 +10294,12 @@
         <v/>
       </c>
       <c r="P80" t="str">
-        <v>20/07/2026</v>
+        <v>Bom Executor / Especialista</v>
       </c>
       <c r="Q80" t="str">
-        <v>Bom Executor / Especialista</v>
-      </c>
-      <c r="R80" t="str">
         <v>Sim</v>
       </c>
-      <c r="S80">
+      <c r="R80">
         <v>45</v>
       </c>
     </row>
@@ -10596,15 +10350,12 @@
         <v/>
       </c>
       <c r="P81" t="str">
-        <v>04/07/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q81" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R81" t="str">
         <v>Sim</v>
       </c>
-      <c r="S81">
+      <c r="R81">
         <v>58</v>
       </c>
     </row>
@@ -10655,15 +10406,12 @@
         <v>Neiva Cristiane Bortolato Goncalves, Edwagner Oliveira</v>
       </c>
       <c r="P82" t="str">
-        <v>09/06/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q82" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R82" t="str">
         <v>Sim</v>
       </c>
-      <c r="S82">
+      <c r="R82">
         <v>74</v>
       </c>
     </row>
@@ -10714,15 +10462,12 @@
         <v>Samuel Santana Barreto</v>
       </c>
       <c r="P83" t="str">
-        <v>12/08/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q83" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R83" t="str">
         <v>Sim</v>
       </c>
-      <c r="S83">
+      <c r="R83">
         <v>70</v>
       </c>
     </row>
@@ -10773,15 +10518,12 @@
         <v/>
       </c>
       <c r="P84" t="str">
-        <v>21/06/2026</v>
+        <v>Alto Potencial</v>
       </c>
       <c r="Q84" t="str">
-        <v>Alto Potencial</v>
-      </c>
-      <c r="R84" t="str">
         <v>Sim</v>
       </c>
-      <c r="S84">
+      <c r="R84">
         <v>26</v>
       </c>
     </row>
@@ -10832,15 +10574,12 @@
         <v>Murilo Zanella Albuquerque</v>
       </c>
       <c r="P85" t="str">
-        <v>04/07/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q85" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R85" t="str">
         <v>Sim</v>
       </c>
-      <c r="S85">
+      <c r="R85">
         <v>73</v>
       </c>
     </row>
@@ -10891,15 +10630,12 @@
         <v/>
       </c>
       <c r="P86" t="str">
-        <v>16/09/2026</v>
+        <v>Alto Potencial</v>
       </c>
       <c r="Q86" t="str">
-        <v>Alto Potencial</v>
-      </c>
-      <c r="R86" t="str">
         <v>Sim</v>
       </c>
-      <c r="S86">
+      <c r="R86">
         <v>53</v>
       </c>
     </row>
@@ -10950,15 +10686,12 @@
         <v/>
       </c>
       <c r="P87" t="str">
-        <v>13/09/2026</v>
+        <v>Empregado Sólido / Responsável</v>
       </c>
       <c r="Q87" t="str">
-        <v>Empregado Sólido / Responsável</v>
-      </c>
-      <c r="R87" t="str">
         <v>Sim</v>
       </c>
-      <c r="S87">
+      <c r="R87">
         <v>50</v>
       </c>
     </row>
@@ -11009,15 +10742,12 @@
         <v/>
       </c>
       <c r="P88" t="str">
-        <v>18/08/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q88" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R88" t="str">
         <v>Sim</v>
       </c>
-      <c r="S88">
+      <c r="R88">
         <v>53</v>
       </c>
     </row>
@@ -11068,15 +10798,12 @@
         <v/>
       </c>
       <c r="P89" t="str">
-        <v>24/06/2026</v>
+        <v>Empregado Sólido / Responsável</v>
       </c>
       <c r="Q89" t="str">
-        <v>Empregado Sólido / Responsável</v>
-      </c>
-      <c r="R89" t="str">
         <v>Sim</v>
       </c>
-      <c r="S89">
+      <c r="R89">
         <v>84</v>
       </c>
     </row>
@@ -11127,15 +10854,12 @@
         <v/>
       </c>
       <c r="P90" t="str">
-        <v>27/08/2026</v>
+        <v>Alto Potencial</v>
       </c>
       <c r="Q90" t="str">
-        <v>Alto Potencial</v>
-      </c>
-      <c r="R90" t="str">
         <v>Sim</v>
       </c>
-      <c r="S90">
+      <c r="R90">
         <v>73</v>
       </c>
     </row>
@@ -11186,15 +10910,12 @@
         <v>Rodrigo da Veiga Lima, Thiago Carvalho Ferreira</v>
       </c>
       <c r="P91" t="str">
-        <v>17/09/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q91" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R91" t="str">
         <v>Sim</v>
       </c>
-      <c r="S91">
+      <c r="R91">
         <v>55</v>
       </c>
     </row>
@@ -11245,15 +10966,12 @@
         <v/>
       </c>
       <c r="P92" t="str">
-        <v>30/08/2026</v>
+        <v>Bom Executor / Especialista</v>
       </c>
       <c r="Q92" t="str">
-        <v>Bom Executor / Especialista</v>
-      </c>
-      <c r="R92" t="str">
         <v>Sim</v>
       </c>
-      <c r="S92">
+      <c r="R92">
         <v>73</v>
       </c>
     </row>
@@ -11304,15 +11022,12 @@
         <v/>
       </c>
       <c r="P93" t="str">
-        <v>11/06/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q93" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R93" t="str">
         <v>Sim</v>
       </c>
-      <c r="S93">
+      <c r="R93">
         <v>3</v>
       </c>
     </row>
@@ -11363,15 +11078,12 @@
         <v>Vitor Guimarães Valadares, Otávio Rezende Jardim</v>
       </c>
       <c r="P94" t="str">
-        <v>19/08/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q94" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R94" t="str">
         <v>Sim</v>
       </c>
-      <c r="S94">
+      <c r="R94">
         <v>42</v>
       </c>
     </row>
@@ -11422,15 +11134,12 @@
         <v>Gabriela Valadares Siqueira</v>
       </c>
       <c r="P95" t="str">
-        <v>06/07/2026</v>
+        <v>Estrela</v>
       </c>
       <c r="Q95" t="str">
-        <v>Estrela</v>
-      </c>
-      <c r="R95" t="str">
         <v>Sim</v>
       </c>
-      <c r="S95">
+      <c r="R95">
         <v>58</v>
       </c>
     </row>
@@ -11481,15 +11190,12 @@
         <v/>
       </c>
       <c r="P96" t="str">
-        <v>12/06/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q96" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R96" t="str">
         <v>Sim</v>
       </c>
-      <c r="S96">
+      <c r="R96">
         <v>47</v>
       </c>
     </row>
@@ -11540,15 +11246,12 @@
         <v>Vitor Guimarães Valadares, Samuel Figueiredo Pacheco</v>
       </c>
       <c r="P97" t="str">
-        <v>16/07/2026</v>
+        <v>Empregado Sólido / Responsável</v>
       </c>
       <c r="Q97" t="str">
-        <v>Empregado Sólido / Responsável</v>
-      </c>
-      <c r="R97" t="str">
         <v>Sim</v>
       </c>
-      <c r="S97">
+      <c r="R97">
         <v>98</v>
       </c>
     </row>
@@ -11599,15 +11302,12 @@
         <v>Rafaela Esteves</v>
       </c>
       <c r="P98" t="str">
-        <v>09/09/2026</v>
+        <v>Estrela</v>
       </c>
       <c r="Q98" t="str">
-        <v>Estrela</v>
-      </c>
-      <c r="R98" t="str">
         <v>Sim</v>
       </c>
-      <c r="S98">
+      <c r="R98">
         <v>98</v>
       </c>
     </row>
@@ -11658,15 +11358,12 @@
         <v>Rafaela Guimarães Esteves, Otávio Rezende Jardim</v>
       </c>
       <c r="P99" t="str">
-        <v>27/06/2026</v>
+        <v>Empregado Sólido / Responsável</v>
       </c>
       <c r="Q99" t="str">
-        <v>Empregado Sólido / Responsável</v>
-      </c>
-      <c r="R99" t="str">
         <v>Sim</v>
       </c>
-      <c r="S99">
+      <c r="R99">
         <v>63</v>
       </c>
     </row>
@@ -11717,15 +11414,12 @@
         <v/>
       </c>
       <c r="P100" t="str">
-        <v>18/08/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q100" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R100" t="str">
         <v>Sim</v>
       </c>
-      <c r="S100">
+      <c r="R100">
         <v>43</v>
       </c>
     </row>
@@ -11776,15 +11470,12 @@
         <v/>
       </c>
       <c r="P101" t="str">
-        <v>06/07/2026</v>
+        <v>Estrela</v>
       </c>
       <c r="Q101" t="str">
-        <v>Estrela</v>
-      </c>
-      <c r="R101" t="str">
         <v>Sim</v>
       </c>
-      <c r="S101">
+      <c r="R101">
         <v>56</v>
       </c>
     </row>
@@ -11835,15 +11526,12 @@
         <v/>
       </c>
       <c r="P102" t="str">
-        <v>11/08/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q102" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R102" t="str">
         <v>Sim</v>
       </c>
-      <c r="S102">
+      <c r="R102">
         <v>96</v>
       </c>
     </row>
@@ -11894,15 +11582,12 @@
         <v>Mauricio Souza</v>
       </c>
       <c r="P103" t="str">
-        <v>06/08/2026</v>
+        <v>Alto Potencial</v>
       </c>
       <c r="Q103" t="str">
-        <v>Alto Potencial</v>
-      </c>
-      <c r="R103" t="str">
         <v>Sim</v>
       </c>
-      <c r="S103">
+      <c r="R103">
         <v>89</v>
       </c>
     </row>
@@ -11953,15 +11638,12 @@
         <v/>
       </c>
       <c r="P104" t="str">
-        <v>04/08/2026</v>
+        <v>Estrela</v>
       </c>
       <c r="Q104" t="str">
-        <v>Estrela</v>
-      </c>
-      <c r="R104" t="str">
         <v>Sim</v>
       </c>
-      <c r="S104">
+      <c r="R104">
         <v>40</v>
       </c>
     </row>
@@ -12012,15 +11694,12 @@
         <v/>
       </c>
       <c r="P105" t="str">
-        <v>20/07/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q105" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R105" t="str">
         <v>Sim</v>
       </c>
-      <c r="S105">
+      <c r="R105">
         <v>65</v>
       </c>
     </row>
@@ -12071,15 +11750,12 @@
         <v>Rogelio dos Santos Vargas</v>
       </c>
       <c r="P106" t="str">
-        <v>30/06/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q106" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R106" t="str">
         <v>Sim</v>
       </c>
-      <c r="S106">
+      <c r="R106">
         <v>32</v>
       </c>
     </row>
@@ -12130,15 +11806,12 @@
         <v/>
       </c>
       <c r="P107" t="str">
-        <v>04/08/2026</v>
+        <v>Empregado Sólido / Responsável</v>
       </c>
       <c r="Q107" t="str">
-        <v>Empregado Sólido / Responsável</v>
-      </c>
-      <c r="R107" t="str">
         <v>Sim</v>
       </c>
-      <c r="S107">
+      <c r="R107">
         <v>62</v>
       </c>
     </row>
@@ -12189,15 +11862,12 @@
         <v>Edson Guedes de Sousa, Milene Thomaz Romano Gantzel</v>
       </c>
       <c r="P108" t="str">
-        <v>05/06/2026</v>
+        <v>Enigma / Questionável</v>
       </c>
       <c r="Q108" t="str">
-        <v>Enigma / Questionável</v>
-      </c>
-      <c r="R108" t="str">
         <v>Sim</v>
       </c>
-      <c r="S108">
+      <c r="R108">
         <v>66</v>
       </c>
     </row>
@@ -12248,15 +11918,12 @@
         <v/>
       </c>
       <c r="P109" t="str">
-        <v>13/08/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q109" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R109" t="str">
         <v>Sim</v>
       </c>
-      <c r="S109">
+      <c r="R109">
         <v>77</v>
       </c>
     </row>
@@ -12307,15 +11974,12 @@
         <v>Raimundo Nonato Silva Amaral</v>
       </c>
       <c r="P110" t="str">
-        <v>09/06/2026</v>
+        <v>Bom Executor / Especialista</v>
       </c>
       <c r="Q110" t="str">
-        <v>Bom Executor / Especialista</v>
-      </c>
-      <c r="R110" t="str">
         <v>Sim</v>
       </c>
-      <c r="S110">
+      <c r="R110">
         <v>2</v>
       </c>
     </row>
@@ -12366,15 +12030,12 @@
         <v>Rogelio Vargas, Fernando da Silva Dias</v>
       </c>
       <c r="P111" t="str">
-        <v>03/09/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q111" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R111" t="str">
         <v>Sim</v>
       </c>
-      <c r="S111">
+      <c r="R111">
         <v>98</v>
       </c>
     </row>
@@ -12425,15 +12086,12 @@
         <v>Fabielly Garcia de Souza Costa</v>
       </c>
       <c r="P112" t="str">
-        <v>17/07/2026</v>
+        <v>Alto Potencial</v>
       </c>
       <c r="Q112" t="str">
-        <v>Alto Potencial</v>
-      </c>
-      <c r="R112" t="str">
         <v>Sim</v>
       </c>
-      <c r="S112">
+      <c r="R112">
         <v>54</v>
       </c>
     </row>
@@ -12484,15 +12142,12 @@
         <v/>
       </c>
       <c r="P113" t="str">
-        <v>27/07/2026</v>
+        <v>Risco / Baixo Desempenho</v>
       </c>
       <c r="Q113" t="str">
-        <v>Risco / Baixo Desempenho</v>
-      </c>
-      <c r="R113" t="str">
         <v>Sim</v>
       </c>
-      <c r="S113">
+      <c r="R113">
         <v>39</v>
       </c>
     </row>
@@ -12543,15 +12198,12 @@
         <v>Willian Fernando Cruz Alves, Edson Sousa</v>
       </c>
       <c r="P114" t="str">
-        <v>13/08/2026</v>
+        <v>Bom Executor / Especialista</v>
       </c>
       <c r="Q114" t="str">
-        <v>Bom Executor / Especialista</v>
-      </c>
-      <c r="R114" t="str">
         <v>Sim</v>
       </c>
-      <c r="S114">
+      <c r="R114">
         <v>35</v>
       </c>
     </row>
@@ -12602,15 +12254,12 @@
         <v>Franciele Fritsch da Silva, Willian Fernando Cruz Alves</v>
       </c>
       <c r="P115" t="str">
-        <v>18/07/2026</v>
+        <v>Estrela</v>
       </c>
       <c r="Q115" t="str">
-        <v>Estrela</v>
-      </c>
-      <c r="R115" t="str">
         <v>Sim</v>
       </c>
-      <c r="S115">
+      <c r="R115">
         <v>31</v>
       </c>
     </row>
@@ -12661,15 +12310,12 @@
         <v>Elisandra Martines dos Santos</v>
       </c>
       <c r="P116" t="str">
-        <v>06/06/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q116" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R116" t="str">
         <v>Sim</v>
       </c>
-      <c r="S116">
+      <c r="R116">
         <v>41</v>
       </c>
     </row>
@@ -12720,15 +12366,12 @@
         <v/>
       </c>
       <c r="P117" t="str">
-        <v>02/06/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q117" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R117" t="str">
         <v>Sim</v>
       </c>
-      <c r="S117">
+      <c r="R117">
         <v>4</v>
       </c>
     </row>
@@ -12779,15 +12422,12 @@
         <v>Raquel Cristina Vidotto Ramos</v>
       </c>
       <c r="P118" t="str">
-        <v>28/07/2026</v>
+        <v>Estrela</v>
       </c>
       <c r="Q118" t="str">
-        <v>Estrela</v>
-      </c>
-      <c r="R118" t="str">
         <v>Sim</v>
       </c>
-      <c r="S118">
+      <c r="R118">
         <v>50</v>
       </c>
     </row>
@@ -12838,15 +12478,12 @@
         <v/>
       </c>
       <c r="P119" t="str">
-        <v>13/09/2026</v>
+        <v>Enigma / Questionável</v>
       </c>
       <c r="Q119" t="str">
-        <v>Enigma / Questionável</v>
-      </c>
-      <c r="R119" t="str">
         <v>Sim</v>
       </c>
-      <c r="S119">
+      <c r="R119">
         <v>23</v>
       </c>
     </row>
@@ -12897,15 +12534,12 @@
         <v/>
       </c>
       <c r="P120" t="str">
-        <v>08/06/2026</v>
+        <v>Bom Executor / Especialista</v>
       </c>
       <c r="Q120" t="str">
-        <v>Bom Executor / Especialista</v>
-      </c>
-      <c r="R120" t="str">
         <v>Sim</v>
       </c>
-      <c r="S120">
+      <c r="R120">
         <v>30</v>
       </c>
     </row>
@@ -12956,15 +12590,12 @@
         <v/>
       </c>
       <c r="P121" t="str">
-        <v>01/08/2026</v>
+        <v>Alto Potencial</v>
       </c>
       <c r="Q121" t="str">
-        <v>Alto Potencial</v>
-      </c>
-      <c r="R121" t="str">
         <v>Sim</v>
       </c>
-      <c r="S121">
+      <c r="R121">
         <v>20</v>
       </c>
     </row>
@@ -13015,15 +12646,12 @@
         <v>Caio Jardim</v>
       </c>
       <c r="P122" t="str">
-        <v>20/08/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q122" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R122" t="str">
         <v>Sim</v>
       </c>
-      <c r="S122">
+      <c r="R122">
         <v>84</v>
       </c>
     </row>
@@ -13074,15 +12702,12 @@
         <v/>
       </c>
       <c r="P123" t="str">
-        <v>25/07/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q123" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R123" t="str">
         <v>Sim</v>
       </c>
-      <c r="S123">
+      <c r="R123">
         <v>98</v>
       </c>
     </row>
@@ -13133,15 +12758,12 @@
         <v>Letícia Tavares Xavier</v>
       </c>
       <c r="P124" t="str">
-        <v>21/06/2026</v>
+        <v>Estrela</v>
       </c>
       <c r="Q124" t="str">
-        <v>Estrela</v>
+        <v>Não</v>
       </c>
       <c r="R124" t="str">
-        <v>Não</v>
-      </c>
-      <c r="S124" t="str">
         <v/>
       </c>
     </row>
@@ -13192,15 +12814,12 @@
         <v>Letícia Tavares Xavier, Paulo da Silva Braz</v>
       </c>
       <c r="P125" t="str">
-        <v>05/07/2026</v>
+        <v>Estrela</v>
       </c>
       <c r="Q125" t="str">
-        <v>Estrela</v>
+        <v>Não</v>
       </c>
       <c r="R125" t="str">
-        <v>Não</v>
-      </c>
-      <c r="S125" t="str">
         <v/>
       </c>
     </row>
@@ -13251,15 +12870,12 @@
         <v>Fabner Roberto Soares, Edson Macoto Tamura Junior</v>
       </c>
       <c r="P126" t="str">
-        <v>20/06/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q126" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R126" t="str">
         <v>Sim</v>
       </c>
-      <c r="S126">
+      <c r="R126">
         <v>57</v>
       </c>
     </row>
@@ -13310,15 +12926,12 @@
         <v>Vinicios Zuse</v>
       </c>
       <c r="P127" t="str">
-        <v>08/09/2026</v>
+        <v>Enigma / Questionável</v>
       </c>
       <c r="Q127" t="str">
-        <v>Enigma / Questionável</v>
-      </c>
-      <c r="R127" t="str">
         <v>Sim</v>
       </c>
-      <c r="S127">
+      <c r="R127">
         <v>64</v>
       </c>
     </row>
@@ -13369,15 +12982,12 @@
         <v>Anderson Rodrigo Giomo</v>
       </c>
       <c r="P128" t="str">
-        <v>31/07/2026</v>
+        <v>Estrela</v>
       </c>
       <c r="Q128" t="str">
-        <v>Estrela</v>
-      </c>
-      <c r="R128" t="str">
         <v>Sim</v>
       </c>
-      <c r="S128">
+      <c r="R128">
         <v>96</v>
       </c>
     </row>
@@ -13428,15 +13038,12 @@
         <v>Anderson Rodrigo Giomo</v>
       </c>
       <c r="P129" t="str">
-        <v>07/06/2026</v>
+        <v>Alto Potencial</v>
       </c>
       <c r="Q129" t="str">
-        <v>Alto Potencial</v>
-      </c>
-      <c r="R129" t="str">
         <v>Sim</v>
       </c>
-      <c r="S129">
+      <c r="R129">
         <v>54</v>
       </c>
     </row>
@@ -13487,15 +13094,12 @@
         <v/>
       </c>
       <c r="P130" t="str">
-        <v>15/08/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q130" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R130" t="str">
         <v>Sim</v>
       </c>
-      <c r="S130">
+      <c r="R130">
         <v>98</v>
       </c>
     </row>
@@ -13546,15 +13150,12 @@
         <v>Danilo Moureira Niza da Silva</v>
       </c>
       <c r="P131" t="str">
-        <v>27/07/2026</v>
+        <v>Empregado Sólido / Responsável</v>
       </c>
       <c r="Q131" t="str">
-        <v>Empregado Sólido / Responsável</v>
-      </c>
-      <c r="R131" t="str">
         <v>Sim</v>
       </c>
-      <c r="S131">
+      <c r="R131">
         <v>44</v>
       </c>
     </row>
@@ -13605,15 +13206,12 @@
         <v/>
       </c>
       <c r="P132" t="str">
-        <v>17/08/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q132" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R132" t="str">
         <v>Sim</v>
       </c>
-      <c r="S132">
+      <c r="R132">
         <v>52</v>
       </c>
     </row>
@@ -13664,15 +13262,12 @@
         <v/>
       </c>
       <c r="P133" t="str">
-        <v>18/08/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q133" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R133" t="str">
         <v>Sim</v>
       </c>
-      <c r="S133">
+      <c r="R133">
         <v>22</v>
       </c>
     </row>
@@ -13723,15 +13318,12 @@
         <v/>
       </c>
       <c r="P134" t="str">
-        <v>04/08/2026</v>
+        <v>Empregado Sólido / Responsável</v>
       </c>
       <c r="Q134" t="str">
-        <v>Empregado Sólido / Responsável</v>
-      </c>
-      <c r="R134" t="str">
         <v>Sim</v>
       </c>
-      <c r="S134">
+      <c r="R134">
         <v>53</v>
       </c>
     </row>
@@ -13782,15 +13374,12 @@
         <v/>
       </c>
       <c r="P135" t="str">
-        <v>31/08/2026</v>
+        <v>Bom Executor / Especialista</v>
       </c>
       <c r="Q135" t="str">
-        <v>Bom Executor / Especialista</v>
-      </c>
-      <c r="R135" t="str">
         <v>Sim</v>
       </c>
-      <c r="S135">
+      <c r="R135">
         <v>61</v>
       </c>
     </row>
@@ -13841,15 +13430,12 @@
         <v>Cleiton Silva, Maykon Fernando da Costa</v>
       </c>
       <c r="P136" t="str">
-        <v>20/08/2026</v>
+        <v>Alto Potencial</v>
       </c>
       <c r="Q136" t="str">
-        <v>Alto Potencial</v>
-      </c>
-      <c r="R136" t="str">
         <v>Sim</v>
       </c>
-      <c r="S136">
+      <c r="R136">
         <v>56</v>
       </c>
     </row>
@@ -13900,15 +13486,12 @@
         <v/>
       </c>
       <c r="P137" t="str">
-        <v>02/06/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q137" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R137" t="str">
         <v>Sim</v>
       </c>
-      <c r="S137">
+      <c r="R137">
         <v>73</v>
       </c>
     </row>
@@ -13959,15 +13542,12 @@
         <v/>
       </c>
       <c r="P138" t="str">
-        <v>14/08/2026</v>
+        <v>Estrela</v>
       </c>
       <c r="Q138" t="str">
-        <v>Estrela</v>
-      </c>
-      <c r="R138" t="str">
         <v>Sim</v>
       </c>
-      <c r="S138">
+      <c r="R138">
         <v>48</v>
       </c>
     </row>
@@ -14018,15 +13598,12 @@
         <v/>
       </c>
       <c r="P139" t="str">
-        <v>29/06/2026</v>
+        <v>Risco / Baixo Desempenho</v>
       </c>
       <c r="Q139" t="str">
-        <v>Risco / Baixo Desempenho</v>
-      </c>
-      <c r="R139" t="str">
         <v>Sim</v>
       </c>
-      <c r="S139">
+      <c r="R139">
         <v>67</v>
       </c>
     </row>
@@ -14077,15 +13654,12 @@
         <v>Rodrigo Lima</v>
       </c>
       <c r="P140" t="str">
-        <v>16/07/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q140" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R140" t="str">
         <v>Sim</v>
       </c>
-      <c r="S140">
+      <c r="R140">
         <v>83</v>
       </c>
     </row>
@@ -14136,15 +13710,12 @@
         <v>Daniela Xavier</v>
       </c>
       <c r="P141" t="str">
-        <v>15/07/2026</v>
+        <v>Estrela</v>
       </c>
       <c r="Q141" t="str">
-        <v>Estrela</v>
-      </c>
-      <c r="R141" t="str">
         <v>Sim</v>
       </c>
-      <c r="S141">
+      <c r="R141">
         <v>32</v>
       </c>
     </row>
@@ -14195,15 +13766,12 @@
         <v/>
       </c>
       <c r="P142" t="str">
-        <v>21/07/2026</v>
+        <v>Estrela</v>
       </c>
       <c r="Q142" t="str">
-        <v>Estrela</v>
-      </c>
-      <c r="R142" t="str">
         <v>Sim</v>
       </c>
-      <c r="S142">
+      <c r="R142">
         <v>51</v>
       </c>
     </row>
@@ -14254,15 +13822,12 @@
         <v>Natiara Vieira</v>
       </c>
       <c r="P143" t="str">
-        <v>21/08/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q143" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R143" t="str">
         <v>Sim</v>
       </c>
-      <c r="S143">
+      <c r="R143">
         <v>68</v>
       </c>
     </row>
@@ -14313,15 +13878,12 @@
         <v/>
       </c>
       <c r="P144" t="str">
-        <v>25/07/2026</v>
+        <v>Alto Potencial</v>
       </c>
       <c r="Q144" t="str">
-        <v>Alto Potencial</v>
-      </c>
-      <c r="R144" t="str">
         <v>Sim</v>
       </c>
-      <c r="S144">
+      <c r="R144">
         <v>45</v>
       </c>
     </row>
@@ -14372,15 +13934,12 @@
         <v>Priscila Andrelina da Silva Bartolomeu</v>
       </c>
       <c r="P145" t="str">
-        <v>02/07/2026</v>
+        <v>Empregado Sólido / Responsável</v>
       </c>
       <c r="Q145" t="str">
-        <v>Empregado Sólido / Responsável</v>
-      </c>
-      <c r="R145" t="str">
         <v>Sim</v>
       </c>
-      <c r="S145">
+      <c r="R145">
         <v>98</v>
       </c>
     </row>
@@ -14431,15 +13990,12 @@
         <v>Priscila Andrelina da Silva Bartolomeu, Eduarda Jardim</v>
       </c>
       <c r="P146" t="str">
-        <v>28/07/2026</v>
+        <v>Enigma / Questionável</v>
       </c>
       <c r="Q146" t="str">
-        <v>Enigma / Questionável</v>
-      </c>
-      <c r="R146" t="str">
         <v>Sim</v>
       </c>
-      <c r="S146">
+      <c r="R146">
         <v>20</v>
       </c>
     </row>
@@ -14490,15 +14046,12 @@
         <v>Eduarda Jardim, Natiara Rodrigues dos Santos Vieira</v>
       </c>
       <c r="P147" t="str">
-        <v>02/09/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q147" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R147" t="str">
         <v>Sim</v>
       </c>
-      <c r="S147">
+      <c r="R147">
         <v>19</v>
       </c>
     </row>
@@ -14549,15 +14102,12 @@
         <v/>
       </c>
       <c r="P148" t="str">
-        <v>28/07/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q148" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R148" t="str">
         <v>Sim</v>
       </c>
-      <c r="S148">
+      <c r="R148">
         <v>96</v>
       </c>
     </row>
@@ -14608,15 +14158,12 @@
         <v>Bruna Valadares</v>
       </c>
       <c r="P149" t="str">
-        <v>13/06/2026</v>
+        <v>Enigma / Questionável</v>
       </c>
       <c r="Q149" t="str">
-        <v>Enigma / Questionável</v>
-      </c>
-      <c r="R149" t="str">
         <v>Sim</v>
       </c>
-      <c r="S149">
+      <c r="R149">
         <v>59</v>
       </c>
     </row>
@@ -14667,15 +14214,12 @@
         <v>Daniela Rezende Nogueira, Jordy Alesson Souza Monteiro</v>
       </c>
       <c r="P150" t="str">
-        <v>07/07/2026</v>
+        <v>Estrela</v>
       </c>
       <c r="Q150" t="str">
-        <v>Estrela</v>
-      </c>
-      <c r="R150" t="str">
         <v>Sim</v>
       </c>
-      <c r="S150">
+      <c r="R150">
         <v>16</v>
       </c>
     </row>
@@ -14726,15 +14270,12 @@
         <v>Jordy Monteiro</v>
       </c>
       <c r="P151" t="str">
-        <v>19/06/2026</v>
+        <v>Bom Executor / Especialista</v>
       </c>
       <c r="Q151" t="str">
-        <v>Bom Executor / Especialista</v>
-      </c>
-      <c r="R151" t="str">
         <v>Sim</v>
       </c>
-      <c r="S151">
+      <c r="R151">
         <v>36</v>
       </c>
     </row>
@@ -14785,15 +14326,12 @@
         <v>Daniela Rezende Nogueira</v>
       </c>
       <c r="P152" t="str">
-        <v>01/08/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q152" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R152" t="str">
         <v>Sim</v>
       </c>
-      <c r="S152">
+      <c r="R152">
         <v>82</v>
       </c>
     </row>
@@ -14844,15 +14382,12 @@
         <v/>
       </c>
       <c r="P153" t="str">
-        <v>13/06/2026</v>
+        <v>Empregado Sólido / Responsável</v>
       </c>
       <c r="Q153" t="str">
-        <v>Empregado Sólido / Responsável</v>
-      </c>
-      <c r="R153" t="str">
         <v>Sim</v>
       </c>
-      <c r="S153">
+      <c r="R153">
         <v>27</v>
       </c>
     </row>
@@ -14903,15 +14438,12 @@
         <v>Juliana Calvo</v>
       </c>
       <c r="P154" t="str">
-        <v>09/06/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q154" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R154" t="str">
         <v>Sim</v>
       </c>
-      <c r="S154">
+      <c r="R154">
         <v>76</v>
       </c>
     </row>
@@ -14962,15 +14494,12 @@
         <v/>
       </c>
       <c r="P155" t="str">
-        <v>13/09/2026</v>
+        <v>Risco / Baixo Desempenho</v>
       </c>
       <c r="Q155" t="str">
-        <v>Risco / Baixo Desempenho</v>
-      </c>
-      <c r="R155" t="str">
         <v>Sim</v>
       </c>
-      <c r="S155">
+      <c r="R155">
         <v>43</v>
       </c>
     </row>
@@ -15021,15 +14550,12 @@
         <v>Antonio Mendonca</v>
       </c>
       <c r="P156" t="str">
-        <v>16/09/2026</v>
+        <v>Empregado Sólido / Responsável</v>
       </c>
       <c r="Q156" t="str">
-        <v>Empregado Sólido / Responsável</v>
-      </c>
-      <c r="R156" t="str">
         <v>Sim</v>
       </c>
-      <c r="S156">
+      <c r="R156">
         <v>67</v>
       </c>
     </row>
@@ -15080,15 +14606,12 @@
         <v>Fabricio Facco, Antonio Raimundo Santos de Mendonca</v>
       </c>
       <c r="P157" t="str">
-        <v>28/07/2026</v>
+        <v>Alto Potencial</v>
       </c>
       <c r="Q157" t="str">
-        <v>Alto Potencial</v>
-      </c>
-      <c r="R157" t="str">
         <v>Sim</v>
       </c>
-      <c r="S157">
+      <c r="R157">
         <v>47</v>
       </c>
     </row>
@@ -15139,15 +14662,12 @@
         <v>Fabricio Silva Facco</v>
       </c>
       <c r="P158" t="str">
-        <v>28/07/2026</v>
+        <v>Enigma / Questionável</v>
       </c>
       <c r="Q158" t="str">
-        <v>Enigma / Questionável</v>
-      </c>
-      <c r="R158" t="str">
         <v>Sim</v>
       </c>
-      <c r="S158">
+      <c r="R158">
         <v>53</v>
       </c>
     </row>
@@ -15198,15 +14718,12 @@
         <v>Fabricio Silva Facco, Antonio Raimundo Santos de Mendonca</v>
       </c>
       <c r="P159" t="str">
-        <v>29/06/2026</v>
+        <v>Bom Executor / Especialista</v>
       </c>
       <c r="Q159" t="str">
-        <v>Bom Executor / Especialista</v>
-      </c>
-      <c r="R159" t="str">
         <v>Sim</v>
       </c>
-      <c r="S159">
+      <c r="R159">
         <v>48</v>
       </c>
     </row>
@@ -15257,15 +14774,12 @@
         <v>Antonio Mendonca</v>
       </c>
       <c r="P160" t="str">
-        <v>15/07/2026</v>
+        <v>Empregado Sólido / Responsável</v>
       </c>
       <c r="Q160" t="str">
-        <v>Empregado Sólido / Responsável</v>
-      </c>
-      <c r="R160" t="str">
         <v>Sim</v>
       </c>
-      <c r="S160">
+      <c r="R160">
         <v>46</v>
       </c>
     </row>
@@ -15316,15 +14830,12 @@
         <v>Fabricio Facco</v>
       </c>
       <c r="P161" t="str">
-        <v>15/09/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q161" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R161" t="str">
         <v>Sim</v>
       </c>
-      <c r="S161">
+      <c r="R161">
         <v>98</v>
       </c>
     </row>
@@ -15375,15 +14886,12 @@
         <v/>
       </c>
       <c r="P162" t="str">
-        <v>16/07/2026</v>
+        <v>Empregado Sólido / Responsável</v>
       </c>
       <c r="Q162" t="str">
-        <v>Empregado Sólido / Responsável</v>
-      </c>
-      <c r="R162" t="str">
         <v>Sim</v>
       </c>
-      <c r="S162">
+      <c r="R162">
         <v>73</v>
       </c>
     </row>
@@ -15434,15 +14942,12 @@
         <v>Rogerio Tsuyoshi Arida</v>
       </c>
       <c r="P163" t="str">
-        <v>09/06/2026</v>
+        <v/>
       </c>
       <c r="Q163" t="str">
-        <v/>
-      </c>
-      <c r="R163" t="str">
         <v>Sim</v>
       </c>
-      <c r="S163">
+      <c r="R163">
         <v>59</v>
       </c>
     </row>
@@ -15493,15 +14998,12 @@
         <v>Luiz Trench, Jonismar Antonio dos Santos</v>
       </c>
       <c r="P164" t="str">
-        <v>25/06/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q164" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R164" t="str">
         <v>Sim</v>
       </c>
-      <c r="S164">
+      <c r="R164">
         <v>61</v>
       </c>
     </row>
@@ -15552,15 +15054,12 @@
         <v/>
       </c>
       <c r="P165" t="str">
-        <v>18/06/2026</v>
+        <v>Estrela</v>
       </c>
       <c r="Q165" t="str">
-        <v>Estrela</v>
-      </c>
-      <c r="R165" t="str">
         <v>Sim</v>
       </c>
-      <c r="S165">
+      <c r="R165">
         <v>56</v>
       </c>
     </row>
@@ -15611,15 +15110,12 @@
         <v/>
       </c>
       <c r="P166" t="str">
-        <v>06/07/2026</v>
+        <v/>
       </c>
       <c r="Q166" t="str">
-        <v/>
-      </c>
-      <c r="R166" t="str">
         <v>Sim</v>
       </c>
-      <c r="S166">
+      <c r="R166">
         <v>43</v>
       </c>
     </row>
@@ -15670,15 +15166,12 @@
         <v/>
       </c>
       <c r="P167" t="str">
-        <v>10/08/2026</v>
+        <v>Empregado Sólido / Responsável</v>
       </c>
       <c r="Q167" t="str">
-        <v>Empregado Sólido / Responsável</v>
-      </c>
-      <c r="R167" t="str">
         <v>Sim</v>
       </c>
-      <c r="S167">
+      <c r="R167">
         <v>78</v>
       </c>
     </row>
@@ -15729,15 +15222,12 @@
         <v/>
       </c>
       <c r="P168" t="str">
-        <v>26/08/2026</v>
+        <v>Estrela</v>
       </c>
       <c r="Q168" t="str">
-        <v>Estrela</v>
-      </c>
-      <c r="R168" t="str">
         <v>Sim</v>
       </c>
-      <c r="S168">
+      <c r="R168">
         <v>20</v>
       </c>
     </row>
@@ -15788,15 +15278,12 @@
         <v>Eduardo Giacometti Xavier, Yuri Ignochevski Primao</v>
       </c>
       <c r="P169" t="str">
-        <v>15/08/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q169" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R169" t="str">
         <v>Sim</v>
       </c>
-      <c r="S169">
+      <c r="R169">
         <v>74</v>
       </c>
     </row>
@@ -15847,15 +15334,12 @@
         <v/>
       </c>
       <c r="P170" t="str">
-        <v>29/06/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q170" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R170" t="str">
         <v>Sim</v>
       </c>
-      <c r="S170">
+      <c r="R170">
         <v>68</v>
       </c>
     </row>
@@ -15906,15 +15390,12 @@
         <v/>
       </c>
       <c r="P171" t="str">
-        <v>08/08/2026</v>
+        <v>Empregado Sólido / Responsável</v>
       </c>
       <c r="Q171" t="str">
-        <v>Empregado Sólido / Responsável</v>
-      </c>
-      <c r="R171" t="str">
         <v>Sim</v>
       </c>
-      <c r="S171">
+      <c r="R171">
         <v>98</v>
       </c>
     </row>
@@ -15965,15 +15446,12 @@
         <v/>
       </c>
       <c r="P172" t="str">
-        <v>16/08/2026</v>
+        <v>Bom Executor / Especialista</v>
       </c>
       <c r="Q172" t="str">
-        <v>Bom Executor / Especialista</v>
-      </c>
-      <c r="R172" t="str">
         <v>Sim</v>
       </c>
-      <c r="S172">
+      <c r="R172">
         <v>25</v>
       </c>
     </row>
@@ -16024,15 +15502,12 @@
         <v/>
       </c>
       <c r="P173" t="str">
-        <v>05/09/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q173" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R173" t="str">
         <v>Sim</v>
       </c>
-      <c r="S173">
+      <c r="R173">
         <v>62</v>
       </c>
     </row>
@@ -16083,15 +15558,12 @@
         <v/>
       </c>
       <c r="P174" t="str">
-        <v>12/06/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q174" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R174" t="str">
         <v>Sim</v>
       </c>
-      <c r="S174">
+      <c r="R174">
         <v>80</v>
       </c>
     </row>
@@ -16142,15 +15614,12 @@
         <v>Rosana Queiroz da Silva</v>
       </c>
       <c r="P175" t="str">
-        <v>14/06/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q175" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R175" t="str">
         <v>Sim</v>
       </c>
-      <c r="S175">
+      <c r="R175">
         <v>33</v>
       </c>
     </row>
@@ -16201,15 +15670,12 @@
         <v/>
       </c>
       <c r="P176" t="str">
-        <v>25/08/2026</v>
+        <v>Enigma / Questionável</v>
       </c>
       <c r="Q176" t="str">
-        <v>Enigma / Questionável</v>
-      </c>
-      <c r="R176" t="str">
         <v>Sim</v>
       </c>
-      <c r="S176">
+      <c r="R176">
         <v>98</v>
       </c>
     </row>
@@ -16260,15 +15726,12 @@
         <v/>
       </c>
       <c r="P177" t="str">
-        <v>08/08/2026</v>
+        <v>Bom Executor / Especialista</v>
       </c>
       <c r="Q177" t="str">
-        <v>Bom Executor / Especialista</v>
-      </c>
-      <c r="R177" t="str">
         <v>Sim</v>
       </c>
-      <c r="S177">
+      <c r="R177">
         <v>64</v>
       </c>
     </row>
@@ -16319,15 +15782,12 @@
         <v/>
       </c>
       <c r="P178" t="str">
-        <v>08/07/2026</v>
+        <v>Empregado Sólido / Responsável</v>
       </c>
       <c r="Q178" t="str">
-        <v>Empregado Sólido / Responsável</v>
-      </c>
-      <c r="R178" t="str">
         <v>Sim</v>
       </c>
-      <c r="S178">
+      <c r="R178">
         <v>22</v>
       </c>
     </row>
@@ -16378,15 +15838,12 @@
         <v/>
       </c>
       <c r="P179" t="str">
-        <v>25/07/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q179" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R179" t="str">
         <v>Sim</v>
       </c>
-      <c r="S179">
+      <c r="R179">
         <v>78</v>
       </c>
     </row>
@@ -16422,12 +15879,9 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="P180" t="str">
-        <v>22/06/2026</v>
+        <v>Enigma / Questionável</v>
       </c>
       <c r="Q180" t="str">
-        <v>Enigma / Questionável</v>
-      </c>
-      <c r="R180" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -16463,12 +15917,9 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="P181" t="str">
-        <v>07/07/2026</v>
+        <v>Estrela</v>
       </c>
       <c r="Q181" t="str">
-        <v>Estrela</v>
-      </c>
-      <c r="R181" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -16495,12 +15946,9 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="P182" t="str">
-        <v>01/08/2026</v>
+        <v>Alto Potencial</v>
       </c>
       <c r="Q182" t="str">
-        <v>Alto Potencial</v>
-      </c>
-      <c r="R182" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -16536,12 +15984,9 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="P183" t="str">
-        <v>19/06/2026</v>
+        <v>Enigma / Questionável</v>
       </c>
       <c r="Q183" t="str">
-        <v>Enigma / Questionável</v>
-      </c>
-      <c r="R183" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -16586,12 +16031,9 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="P184" t="str">
-        <v>08/09/2026</v>
+        <v>Empregado Sólido / Responsável</v>
       </c>
       <c r="Q184" t="str">
-        <v>Empregado Sólido / Responsável</v>
-      </c>
-      <c r="R184" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -16636,12 +16078,9 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="P185" t="str">
-        <v>07/07/2026</v>
+        <v>Empregado Sólido / Responsável</v>
       </c>
       <c r="Q185" t="str">
-        <v>Empregado Sólido / Responsável</v>
-      </c>
-      <c r="R185" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -16668,12 +16107,9 @@
         <v>Não</v>
       </c>
       <c r="P186" t="str">
-        <v>09/09/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q186" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R186" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -16709,12 +16145,9 @@
         <v>Não</v>
       </c>
       <c r="P187" t="str">
-        <v>13/08/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q187" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R187" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -16759,12 +16192,9 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="P188" t="str">
-        <v>10/09/2026</v>
+        <v>Risco / Baixo Desempenho</v>
       </c>
       <c r="Q188" t="str">
-        <v>Risco / Baixo Desempenho</v>
-      </c>
-      <c r="R188" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -16809,12 +16239,9 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="P189" t="str">
-        <v>01/09/2026</v>
+        <v>Enigma / Questionável</v>
       </c>
       <c r="Q189" t="str">
-        <v>Enigma / Questionável</v>
-      </c>
-      <c r="R189" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -16849,10 +16276,7 @@
       <c r="M190" t="str">
         <v>Conversado, sem plano formal</v>
       </c>
-      <c r="P190" t="str">
-        <v>02/08/2026</v>
-      </c>
-      <c r="R190" t="str">
+      <c r="Q190" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -16897,12 +16321,9 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="P191" t="str">
-        <v>21/08/2026</v>
+        <v>Alto Potencial</v>
       </c>
       <c r="Q191" t="str">
-        <v>Alto Potencial</v>
-      </c>
-      <c r="R191" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -16947,12 +16368,9 @@
         <v>Não</v>
       </c>
       <c r="P192" t="str">
-        <v>12/07/2026</v>
+        <v>Alto Potencial</v>
       </c>
       <c r="Q192" t="str">
-        <v>Alto Potencial</v>
-      </c>
-      <c r="R192" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -16988,12 +16406,9 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="P193" t="str">
-        <v>06/07/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q193" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R193" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -17029,12 +16444,9 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="P194" t="str">
-        <v>23/06/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q194" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R194" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -17070,12 +16482,9 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="P195" t="str">
-        <v>21/07/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q195" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R195" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -17102,12 +16511,9 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="P196" t="str">
-        <v>08/07/2026</v>
+        <v>Bom Executor / Especialista</v>
       </c>
       <c r="Q196" t="str">
-        <v>Bom Executor / Especialista</v>
-      </c>
-      <c r="R196" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -17143,12 +16549,9 @@
         <v>Não</v>
       </c>
       <c r="P197" t="str">
-        <v>18/07/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q197" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R197" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -17193,12 +16596,9 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="P198" t="str">
-        <v>24/07/2026</v>
+        <v>Bom Executor / Especialista</v>
       </c>
       <c r="Q198" t="str">
-        <v>Bom Executor / Especialista</v>
-      </c>
-      <c r="R198" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -17243,12 +16643,9 @@
         <v>Não</v>
       </c>
       <c r="P199" t="str">
-        <v>14/08/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q199" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R199" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -17284,12 +16681,9 @@
         <v>Não</v>
       </c>
       <c r="P200" t="str">
-        <v>30/06/2026</v>
+        <v>Estrela</v>
       </c>
       <c r="Q200" t="str">
-        <v>Estrela</v>
-      </c>
-      <c r="R200" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -17316,12 +16710,9 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="P201" t="str">
-        <v>01/08/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q201" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R201" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -17357,12 +16748,9 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="P202" t="str">
-        <v>28/08/2026</v>
+        <v>Bom Executor / Especialista</v>
       </c>
       <c r="Q202" t="str">
-        <v>Bom Executor / Especialista</v>
-      </c>
-      <c r="R202" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -17407,12 +16795,9 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="P203" t="str">
-        <v>08/07/2026</v>
+        <v>Enigma / Questionável</v>
       </c>
       <c r="Q203" t="str">
-        <v>Enigma / Questionável</v>
-      </c>
-      <c r="R203" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -17448,12 +16833,9 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="P204" t="str">
-        <v>30/06/2026</v>
+        <v>Enigma / Questionável</v>
       </c>
       <c r="Q204" t="str">
-        <v>Enigma / Questionável</v>
-      </c>
-      <c r="R204" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -17489,12 +16871,9 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="P205" t="str">
-        <v>02/08/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q205" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R205" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -17521,12 +16900,9 @@
         <v>Não</v>
       </c>
       <c r="P206" t="str">
-        <v>08/08/2026</v>
+        <v>Alto Desempenho</v>
       </c>
       <c r="Q206" t="str">
-        <v>Alto Desempenho</v>
-      </c>
-      <c r="R206" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -17562,12 +16938,9 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="P207" t="str">
-        <v>22/06/2026</v>
+        <v>Empregado Eficaz</v>
       </c>
       <c r="Q207" t="str">
-        <v>Empregado Eficaz</v>
-      </c>
-      <c r="R207" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -17603,12 +16976,9 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="P208" t="str">
-        <v>09/07/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q208" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R208" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -17644,12 +17014,9 @@
         <v>Não</v>
       </c>
       <c r="P209" t="str">
-        <v>17/06/2026</v>
+        <v>Bom Executor / Especialista</v>
       </c>
       <c r="Q209" t="str">
-        <v>Bom Executor / Especialista</v>
-      </c>
-      <c r="R209" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -17685,12 +17052,9 @@
         <v>Não</v>
       </c>
       <c r="P210" t="str">
-        <v>29/06/2026</v>
+        <v>Bom Executor / Especialista</v>
       </c>
       <c r="Q210" t="str">
-        <v>Bom Executor / Especialista</v>
-      </c>
-      <c r="R210" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -17735,12 +17099,9 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="P211" t="str">
-        <v>31/07/2026</v>
+        <v>Bom Executor / Especialista</v>
       </c>
       <c r="Q211" t="str">
-        <v>Bom Executor / Especialista</v>
-      </c>
-      <c r="R211" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -17776,12 +17137,9 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="P212" t="str">
-        <v>21/08/2026</v>
+        <v>Estrela</v>
       </c>
       <c r="Q212" t="str">
-        <v>Estrela</v>
-      </c>
-      <c r="R212" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -17817,12 +17175,9 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="P213" t="str">
-        <v>03/07/2026</v>
+        <v>Empregado Sólido / Responsável</v>
       </c>
       <c r="Q213" t="str">
-        <v>Empregado Sólido / Responsável</v>
-      </c>
-      <c r="R213" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -17867,12 +17222,9 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="P214" t="str">
-        <v>20/06/2026</v>
+        <v>Empregado Comprometido</v>
       </c>
       <c r="Q214" t="str">
-        <v>Empregado Comprometido</v>
-      </c>
-      <c r="R214" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -17908,12 +17260,9 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="P215" t="str">
-        <v>09/06/2026</v>
+        <v>Bom Executor / Especialista</v>
       </c>
       <c r="Q215" t="str">
-        <v>Bom Executor / Especialista</v>
-      </c>
-      <c r="R215" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -17958,12 +17307,9 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="P216" t="str">
-        <v>12/06/2026</v>
+        <v>Empregado Sólido / Responsável</v>
       </c>
       <c r="Q216" t="str">
-        <v>Empregado Sólido / Responsável</v>
-      </c>
-      <c r="R216" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -18008,12 +17354,9 @@
         <v>Não</v>
       </c>
       <c r="P217" t="str">
-        <v>10/07/2026</v>
+        <v>Estrela</v>
       </c>
       <c r="Q217" t="str">
-        <v>Estrela</v>
-      </c>
-      <c r="R217" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -18040,12 +17383,9 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="P218" t="str">
-        <v>01/06/2026</v>
+        <v>Alto Potencial</v>
       </c>
       <c r="Q218" t="str">
-        <v>Alto Potencial</v>
-      </c>
-      <c r="R218" t="str">
         <v>Não</v>
       </c>
     </row>
@@ -18072,18 +17412,15 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="P219" t="str">
-        <v>14/06/2026</v>
+        <v>Enigma / Questionável</v>
       </c>
       <c r="Q219" t="str">
-        <v>Enigma / Questionável</v>
-      </c>
-      <c r="R219" t="str">
         <v>Não</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S219"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R219"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Pesquisa de clima como resultado percentual, sem e-NPS
O critério de clima passa a usar o resultado da pesquisa de clima 2026
da área em % (0 a 100), com as mesmas faixas e pontos do material.
Campo, coluna da planilha, validação, telas de metodologia e cartão do
candidato atualizados; planilha de exemplo regerada. Versão da base
local para 5.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E5WdJkUTyiNFgco3uhd6x7
</commit_message>
<xml_diff>
--- a/exemplos/Gazin_Mapa_Sucessorio_EXEMPLO_FICTICIO.xlsx
+++ b/exemplos/Gazin_Mapa_Sucessorio_EXEMPLO_FICTICIO.xlsx
@@ -513,7 +513,7 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>e-NPS da área 2026: número de -100 a 100, só para quem lidera equipe.</v>
+        <v>Pesquisa de clima 2026 (%): resultado da área de 0 a 100 (pode ser 82 ou 82%), só para quem lidera equipe.</v>
       </c>
     </row>
     <row r="23">
@@ -5820,7 +5820,7 @@
     <col min="15" max="15" width="50.83203125" customWidth="1"/>
     <col min="16" max="16" width="39.83203125" customWidth="1"/>
     <col min="17" max="17" width="15.83203125" customWidth="1"/>
-    <col min="18" max="18" width="20.83203125" customWidth="1"/>
+    <col min="18" max="18" width="28.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5876,7 +5876,7 @@
         <v>Lidera equipe</v>
       </c>
       <c r="R1" t="str">
-        <v>e-NPS da área 2026</v>
+        <v>Pesquisa de clima 2026 (%)</v>
       </c>
     </row>
     <row r="2">
@@ -7556,7 +7556,7 @@
         <v>Sim</v>
       </c>
       <c r="R31">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="32">
@@ -7612,7 +7612,7 @@
         <v>Sim</v>
       </c>
       <c r="R32">
-        <v>-10</v>
+        <v>18</v>
       </c>
     </row>
     <row r="33">
@@ -8172,7 +8172,7 @@
         <v>Sim</v>
       </c>
       <c r="R42">
-        <v>7</v>
+        <v>18</v>
       </c>
     </row>
     <row r="43">
@@ -9012,7 +9012,7 @@
         <v>Sim</v>
       </c>
       <c r="R57">
-        <v>14</v>
+        <v>18</v>
       </c>
     </row>
     <row r="58">
@@ -11028,7 +11028,7 @@
         <v>Sim</v>
       </c>
       <c r="R93">
-        <v>3</v>
+        <v>18</v>
       </c>
     </row>
     <row r="94">
@@ -11980,7 +11980,7 @@
         <v>Sim</v>
       </c>
       <c r="R110">
-        <v>2</v>
+        <v>18</v>
       </c>
     </row>
     <row r="111">
@@ -12372,7 +12372,7 @@
         <v>Sim</v>
       </c>
       <c r="R117">
-        <v>4</v>
+        <v>18</v>
       </c>
     </row>
     <row r="118">
@@ -14220,7 +14220,7 @@
         <v>Sim</v>
       </c>
       <c r="R150">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="151">

</xml_diff>

<commit_message>
Inclui a posição Gerente geral de recursos humanos
Ocupada por Alessandra Guerra de Souza, ligada direto à Presidência
(Gerência Executiva). Entra por POSICOES_ADICIONAIS no script da base,
no fim da lista, sem renumerar posições existentes. Planilha de exemplo
regerada; versão da base local para 6.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E5WdJkUTyiNFgco3uhd6x7
</commit_message>
<xml_diff>
--- a/exemplos/Gazin_Mapa_Sucessorio_EXEMPLO_FICTICIO.xlsx
+++ b/exemplos/Gazin_Mapa_Sucessorio_EXEMPLO_FICTICIO.xlsx
@@ -530,7 +530,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I181"/>
+  <dimension ref="A1:I182"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="50.83203125" customWidth="1"/>
@@ -592,7 +592,7 @@
         <v/>
       </c>
       <c r="G2">
-        <v>1.8</v>
+        <v>5.8</v>
       </c>
       <c r="H2" t="str">
         <v>Gilmar Alves de Oliveira</v>
@@ -621,7 +621,7 @@
         <v>Francieli Bessa Silva Tavares</v>
       </c>
       <c r="G3">
-        <v>23</v>
+        <v>5.9</v>
       </c>
       <c r="H3" t="str">
         <v>Cleiton Cesar Silva</v>
@@ -650,7 +650,7 @@
         <v>Luiz Fernando Bandeira</v>
       </c>
       <c r="G4">
-        <v>6.7</v>
+        <v>16.3</v>
       </c>
       <c r="H4" t="str">
         <v>Cleiton Cesar Silva</v>
@@ -679,7 +679,7 @@
         <v>Cleiton Cesar Silva</v>
       </c>
       <c r="G5">
-        <v>24.5</v>
+        <v>24.6</v>
       </c>
       <c r="H5" t="str">
         <v>Fernando Sanches Graci</v>
@@ -708,7 +708,7 @@
         <v>Diego Henrique Garcia Soriani</v>
       </c>
       <c r="G6">
-        <v>13.9</v>
+        <v>24.9</v>
       </c>
       <c r="H6" t="str">
         <v>Fernando Sanches Graci</v>
@@ -766,7 +766,7 @@
         <v>Leandro Tonhi Mingote</v>
       </c>
       <c r="G8">
-        <v>5.8</v>
+        <v>8.9</v>
       </c>
       <c r="H8" t="str">
         <v>Cleiton Cesar Silva</v>
@@ -795,7 +795,7 @@
         <v>Jaciane Pestana Souza</v>
       </c>
       <c r="G9">
-        <v>5.9</v>
+        <v>16</v>
       </c>
       <c r="H9" t="str">
         <v>Cleiton Cesar Silva</v>
@@ -824,7 +824,7 @@
         <v>Vinicius Ramos da Silva</v>
       </c>
       <c r="G10">
-        <v>16.3</v>
+        <v>14.4</v>
       </c>
       <c r="H10" t="str">
         <v>Cleiton Fabio Bianchini da Silva</v>
@@ -853,7 +853,7 @@
         <v>Renato Aparecido Andrade</v>
       </c>
       <c r="G11">
-        <v>24.6</v>
+        <v>7.5</v>
       </c>
       <c r="H11" t="str">
         <v>Renan da Silva Medeiros</v>
@@ -882,7 +882,7 @@
         <v>Jeferson Duarte Goncalves</v>
       </c>
       <c r="G12">
-        <v>24.9</v>
+        <v>19.1</v>
       </c>
       <c r="H12" t="str">
         <v>Cleiton Berger</v>
@@ -911,7 +911,7 @@
         <v>Thais Tarcia de Araujo Oliveira</v>
       </c>
       <c r="G13">
-        <v>23.2</v>
+        <v>17.1</v>
       </c>
       <c r="H13" t="str">
         <v>Renan da Silva Medeiros</v>
@@ -940,7 +940,7 @@
         <v>Renan da Silva Medeiros</v>
       </c>
       <c r="G14">
-        <v>8.9</v>
+        <v>21.1</v>
       </c>
       <c r="H14" t="str">
         <v>Cleiton Berger</v>
@@ -969,7 +969,7 @@
         <v>Peter Luiz Cruz Pregidio</v>
       </c>
       <c r="G15">
-        <v>16</v>
+        <v>4.2</v>
       </c>
       <c r="H15" t="str">
         <v>Cleiton Berger</v>
@@ -998,7 +998,7 @@
         <v>Cleiton Fabio Bianchini da Silva</v>
       </c>
       <c r="G16">
-        <v>14.4</v>
+        <v>17.8</v>
       </c>
       <c r="H16" t="str">
         <v>Cleiton Berger</v>
@@ -1027,7 +1027,7 @@
         <v>Leyffor Augusto de Carvalho Gastaldin</v>
       </c>
       <c r="G17">
-        <v>7.5</v>
+        <v>18.6</v>
       </c>
       <c r="H17" t="str">
         <v>Cleiton Berger</v>
@@ -1056,7 +1056,7 @@
         <v>Joel Borato</v>
       </c>
       <c r="G18">
-        <v>19.1</v>
+        <v>10.7</v>
       </c>
       <c r="H18" t="str">
         <v>Leyffor Augusto de Carvalho Gastaldin</v>
@@ -1085,7 +1085,7 @@
         <v>Juliano Silva Vicentini</v>
       </c>
       <c r="G19">
-        <v>17.1</v>
+        <v>22.9</v>
       </c>
       <c r="H19" t="str">
         <v>Leyffor Augusto de Carvalho Gastaldin</v>
@@ -1114,7 +1114,7 @@
         <v>Mateus de Azevedo Volttani</v>
       </c>
       <c r="G20">
-        <v>21.1</v>
+        <v>13.3</v>
       </c>
       <c r="H20" t="str">
         <v>Leyffor Augusto de Carvalho Gastaldin</v>
@@ -1143,7 +1143,7 @@
         <v>Patricia Giroto</v>
       </c>
       <c r="G21">
-        <v>4.2</v>
+        <v>19.8</v>
       </c>
       <c r="H21" t="str">
         <v>Peter Luiz Cruz Pregidio</v>
@@ -1172,7 +1172,7 @@
         <v>Janaina Braga Pires Kashiwaya</v>
       </c>
       <c r="G22">
-        <v>17.8</v>
+        <v>17.4</v>
       </c>
       <c r="H22" t="str">
         <v>Cleiton Berger</v>
@@ -1201,7 +1201,7 @@
         <v>Daiane Domingues dos Santos</v>
       </c>
       <c r="G23">
-        <v>18.6</v>
+        <v>16.9</v>
       </c>
       <c r="H23" t="str">
         <v>Renan da Silva Medeiros</v>
@@ -1230,7 +1230,7 @@
         <v>Fabielly Garcia de Souza Costa</v>
       </c>
       <c r="G24">
-        <v>10.7</v>
+        <v>20.7</v>
       </c>
       <c r="H24" t="str">
         <v>Renato Aparecido Andrade</v>
@@ -1259,7 +1259,7 @@
         <v>Raquel Cristina Vidotto Ramos</v>
       </c>
       <c r="G25">
-        <v>22.9</v>
+        <v>18</v>
       </c>
       <c r="H25" t="str">
         <v>Renato Aparecido Andrade</v>
@@ -1288,7 +1288,7 @@
         <v>Marcelo de Souza Rodrigues</v>
       </c>
       <c r="G26">
-        <v>13.3</v>
+        <v>20.5</v>
       </c>
       <c r="H26" t="str">
         <v>Leyffor Augusto de Carvalho Gastaldin</v>
@@ -1317,7 +1317,7 @@
         <v>Duberlei de Castro da Silva</v>
       </c>
       <c r="G27">
-        <v>19.8</v>
+        <v>20.7</v>
       </c>
       <c r="H27" t="str">
         <v>Julio Cezar da Silva</v>
@@ -1346,7 +1346,7 @@
         <v>Robson Rodrigues Jacinto</v>
       </c>
       <c r="G28">
-        <v>17.4</v>
+        <v>4.9</v>
       </c>
       <c r="H28" t="str">
         <v>Aparecido Benedito dos Santos</v>
@@ -1375,7 +1375,7 @@
         <v>Luiz Paulo da Silva Santos</v>
       </c>
       <c r="G29">
-        <v>16.9</v>
+        <v>8.5</v>
       </c>
       <c r="H29" t="str">
         <v>Robiano Eloir Pereira</v>
@@ -1404,7 +1404,7 @@
         <v>Julio Cezar da Silva</v>
       </c>
       <c r="G30">
-        <v>20.7</v>
+        <v>18.7</v>
       </c>
       <c r="H30" t="str">
         <v>Gilmar Alves de Oliveira</v>
@@ -1433,7 +1433,7 @@
         <v>Wesley Dionisio da Silva</v>
       </c>
       <c r="G31">
-        <v>18</v>
+        <v>16.1</v>
       </c>
       <c r="H31" t="str">
         <v>Julio Cezar da Silva</v>
@@ -1462,7 +1462,7 @@
         <v/>
       </c>
       <c r="G32">
-        <v>20.5</v>
+        <v>23.7</v>
       </c>
       <c r="H32" t="str">
         <v/>
@@ -1491,7 +1491,7 @@
         <v>Rosana Queiroz da Silva</v>
       </c>
       <c r="G33">
-        <v>20.7</v>
+        <v>21.5</v>
       </c>
       <c r="H33" t="str">
         <v>Luanna Geraldo Borges</v>
@@ -1520,7 +1520,7 @@
         <v>Orlando Rodrigues Neto</v>
       </c>
       <c r="G34">
-        <v>4.9</v>
+        <v>13.6</v>
       </c>
       <c r="H34" t="str">
         <v>Frank Soares do Nascimento</v>
@@ -1549,7 +1549,7 @@
         <v>Aparecido Benedito dos Santos</v>
       </c>
       <c r="G35">
-        <v>8.5</v>
+        <v>24.3</v>
       </c>
       <c r="H35" t="str">
         <v>Julio Cezar da Silva</v>
@@ -1578,7 +1578,7 @@
         <v>Thiago Dias Tavares</v>
       </c>
       <c r="G36">
-        <v>18.7</v>
+        <v>8.5</v>
       </c>
       <c r="H36" t="str">
         <v>Julio Cezar da Silva</v>
@@ -1607,7 +1607,7 @@
         <v>Paulo Jose da Silva</v>
       </c>
       <c r="G37">
-        <v>16.1</v>
+        <v>8.3</v>
       </c>
       <c r="H37" t="str">
         <v>Julio Cezar da Silva</v>
@@ -1636,7 +1636,7 @@
         <v>Leandro Santiago Afonso</v>
       </c>
       <c r="G38">
-        <v>23.7</v>
+        <v>21.5</v>
       </c>
       <c r="H38" t="str">
         <v>Paulo Sergio dos Santos</v>
@@ -1665,7 +1665,7 @@
         <v>Valdenei Vargas de Almeida</v>
       </c>
       <c r="G39">
-        <v>21.5</v>
+        <v>13.2</v>
       </c>
       <c r="H39" t="str">
         <v>Paulo Sergio dos Santos</v>
@@ -1694,7 +1694,7 @@
         <v>Andre Schafer Pasinato</v>
       </c>
       <c r="G40">
-        <v>13.6</v>
+        <v>20.8</v>
       </c>
       <c r="H40" t="str">
         <v>Julio Cezar da Silva</v>
@@ -1723,7 +1723,7 @@
         <v>Niccolas Daniel Curvelo</v>
       </c>
       <c r="G41">
-        <v>24.3</v>
+        <v>6</v>
       </c>
       <c r="H41" t="str">
         <v>Andre Schafer Pasinato</v>
@@ -1752,7 +1752,7 @@
         <v>Wesley Diniz Alves</v>
       </c>
       <c r="G42">
-        <v>8.5</v>
+        <v>9.6</v>
       </c>
       <c r="H42" t="str">
         <v>Julio Cezar da Silva</v>
@@ -1781,7 +1781,7 @@
         <v>Cidclei Reck</v>
       </c>
       <c r="G43">
-        <v>8.3</v>
+        <v>3.7</v>
       </c>
       <c r="H43" t="str">
         <v>Frank Soares do Nascimento</v>
@@ -1810,7 +1810,7 @@
         <v>Juliano Donizete de Sousa</v>
       </c>
       <c r="G44">
-        <v>21.5</v>
+        <v>8</v>
       </c>
       <c r="H44" t="str">
         <v>Frank Soares do Nascimento</v>
@@ -1839,7 +1839,7 @@
         <v>Marcio Adriano Leme</v>
       </c>
       <c r="G45">
-        <v>13.2</v>
+        <v>17.6</v>
       </c>
       <c r="H45" t="str">
         <v>Frank Soares do Nascimento</v>
@@ -1868,7 +1868,7 @@
         <v>Natan Henrique Goncalves</v>
       </c>
       <c r="G46">
-        <v>20.8</v>
+        <v>19.9</v>
       </c>
       <c r="H46" t="str">
         <v>Frank Soares do Nascimento</v>
@@ -1897,7 +1897,7 @@
         <v>Juliana Calvo</v>
       </c>
       <c r="G47">
-        <v>6</v>
+        <v>14.3</v>
       </c>
       <c r="H47" t="str">
         <v>Julio Cezar da Silva</v>
@@ -1926,7 +1926,7 @@
         <v>Frank Soares do Nascimento</v>
       </c>
       <c r="G48">
-        <v>9.6</v>
+        <v>21.8</v>
       </c>
       <c r="H48" t="str">
         <v>Julio Cezar da Silva</v>
@@ -1955,7 +1955,7 @@
         <v>Paulo Sergio dos Santos</v>
       </c>
       <c r="G49">
-        <v>3.7</v>
+        <v>4.1</v>
       </c>
       <c r="H49" t="str">
         <v>Julio Cezar da Silva</v>
@@ -1984,7 +1984,7 @@
         <v>Adson Nogueira da Silva</v>
       </c>
       <c r="G50">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="H50" t="str">
         <v>Valdenei Vargas de Almeida</v>
@@ -2013,7 +2013,7 @@
         <v>Anderson Luiz Ferreira Ricardo</v>
       </c>
       <c r="G51">
-        <v>17.6</v>
+        <v>19</v>
       </c>
       <c r="H51" t="str">
         <v>Leandro Santiago Afonso</v>
@@ -2042,7 +2042,7 @@
         <v>Arinan Moreira dos Santos</v>
       </c>
       <c r="G52">
-        <v>19.9</v>
+        <v>24.7</v>
       </c>
       <c r="H52" t="str">
         <v>Leandro Santiago Afonso</v>
@@ -2071,7 +2071,7 @@
         <v>Celso Luiz Sacramento de Souza</v>
       </c>
       <c r="G53">
-        <v>14.3</v>
+        <v>7.8</v>
       </c>
       <c r="H53" t="str">
         <v>Valdenei Vargas de Almeida</v>
@@ -2100,7 +2100,7 @@
         <v>Djalma Almeida Andrade</v>
       </c>
       <c r="G54">
-        <v>21.8</v>
+        <v>10.9</v>
       </c>
       <c r="H54" t="str">
         <v>Valdenei Vargas de Almeida</v>
@@ -2129,7 +2129,7 @@
         <v>Erlon Cesar Cruz Almeida</v>
       </c>
       <c r="G55">
-        <v>4.1</v>
+        <v>9.3</v>
       </c>
       <c r="H55" t="str">
         <v>Leandro Santiago Afonso</v>
@@ -2158,7 +2158,7 @@
         <v>Guilherme Caetano Gelamos</v>
       </c>
       <c r="G56">
-        <v>25</v>
+        <v>2.6</v>
       </c>
       <c r="H56" t="str">
         <v>Valdenei Vargas de Almeida</v>
@@ -2187,7 +2187,7 @@
         <v>Jadiel Ribeiro Durço</v>
       </c>
       <c r="G57">
-        <v>19</v>
+        <v>8.8</v>
       </c>
       <c r="H57" t="str">
         <v>Valdenei Vargas de Almeida</v>
@@ -2216,7 +2216,7 @@
         <v>Jean Medrado dos Santos</v>
       </c>
       <c r="G58">
-        <v>24.7</v>
+        <v>17.2</v>
       </c>
       <c r="H58" t="str">
         <v>Valdenei Vargas de Almeida</v>
@@ -2245,7 +2245,7 @@
         <v>Juliano de Albuquerque Silva</v>
       </c>
       <c r="G59">
-        <v>7.8</v>
+        <v>4.8</v>
       </c>
       <c r="H59" t="str">
         <v>Valdenei Vargas de Almeida</v>
@@ -2274,7 +2274,7 @@
         <v>Luis Carlos Alves de Melo</v>
       </c>
       <c r="G60">
-        <v>10.9</v>
+        <v>22.1</v>
       </c>
       <c r="H60" t="str">
         <v>Leandro Santiago Afonso</v>
@@ -2303,7 +2303,7 @@
         <v>Nicareli Neves</v>
       </c>
       <c r="G61">
-        <v>9.3</v>
+        <v>23.4</v>
       </c>
       <c r="H61" t="str">
         <v>Leandro Santiago Afonso</v>
@@ -2332,7 +2332,7 @@
         <v>Odimar Antonio de Oliveira</v>
       </c>
       <c r="G62">
-        <v>2.6</v>
+        <v>19.6</v>
       </c>
       <c r="H62" t="str">
         <v>Leandro Santiago Afonso</v>
@@ -2361,7 +2361,7 @@
         <v>Ricardo Rodrigues</v>
       </c>
       <c r="G63">
-        <v>8.8</v>
+        <v>23.1</v>
       </c>
       <c r="H63" t="str">
         <v>Leandro Santiago Afonso</v>
@@ -2390,7 +2390,7 @@
         <v>Leandro Ferreira Paim Mendes</v>
       </c>
       <c r="G64">
-        <v>17.2</v>
+        <v>21.5</v>
       </c>
       <c r="H64" t="str">
         <v>Leandro Santiago Afonso</v>
@@ -2419,7 +2419,7 @@
         <v>Gustavo Paixao dos Santos</v>
       </c>
       <c r="G65">
-        <v>4.8</v>
+        <v>3.6</v>
       </c>
       <c r="H65" t="str">
         <v>Frank Soares do Nascimento</v>
@@ -2448,7 +2448,7 @@
         <v>Bruno Rodrigues Martins</v>
       </c>
       <c r="G66">
-        <v>22.1</v>
+        <v>20.8</v>
       </c>
       <c r="H66" t="str">
         <v>Paulo Sergio dos Santos</v>
@@ -2477,7 +2477,7 @@
         <v>Aline Portela dos Santos</v>
       </c>
       <c r="G67">
-        <v>23.4</v>
+        <v>24.5</v>
       </c>
       <c r="H67" t="str">
         <v>Thais Tarcia de Araujo Oliveira</v>
@@ -2506,7 +2506,7 @@
         <v>Andreza Miranda da Silva</v>
       </c>
       <c r="G68">
-        <v>19.6</v>
+        <v>13</v>
       </c>
       <c r="H68" t="str">
         <v>Thais Tarcia de Araujo Oliveira</v>
@@ -2535,7 +2535,7 @@
         <v>Beatriz Santos Kroetzler</v>
       </c>
       <c r="G69">
-        <v>23.1</v>
+        <v>20.1</v>
       </c>
       <c r="H69" t="str">
         <v>Thais Tarcia de Araujo Oliveira</v>
@@ -2564,7 +2564,7 @@
         <v>Elisandra Martines dos Santos</v>
       </c>
       <c r="G70">
-        <v>21.5</v>
+        <v>24.1</v>
       </c>
       <c r="H70" t="str">
         <v>Thais Tarcia de Araujo Oliveira</v>
@@ -2593,7 +2593,7 @@
         <v>Hagatha Leticia Zuchinalli Nogueira</v>
       </c>
       <c r="G71">
-        <v>3.6</v>
+        <v>14.4</v>
       </c>
       <c r="H71" t="str">
         <v>Thais Tarcia de Araujo Oliveira</v>
@@ -2622,7 +2622,7 @@
         <v>Jeovanir Castro de Souza</v>
       </c>
       <c r="G72">
-        <v>20.8</v>
+        <v>12.9</v>
       </c>
       <c r="H72" t="str">
         <v>Thais Tarcia de Araujo Oliveira</v>
@@ -2651,7 +2651,7 @@
         <v>Juliana Rodriguez Ferro</v>
       </c>
       <c r="G73">
-        <v>24.5</v>
+        <v>7</v>
       </c>
       <c r="H73" t="str">
         <v>Thais Tarcia de Araujo Oliveira</v>
@@ -2680,7 +2680,7 @@
         <v>Keila da Silva Sena Leao</v>
       </c>
       <c r="G74">
-        <v>13</v>
+        <v>12.7</v>
       </c>
       <c r="H74" t="str">
         <v>Thais Tarcia de Araujo Oliveira</v>
@@ -2709,7 +2709,7 @@
         <v>Lidia dos Santos</v>
       </c>
       <c r="G75">
-        <v>20.1</v>
+        <v>23.8</v>
       </c>
       <c r="H75" t="str">
         <v>Thais Tarcia de Araujo Oliveira</v>
@@ -2738,7 +2738,7 @@
         <v>Maria Cleide Araujo</v>
       </c>
       <c r="G76">
-        <v>24.1</v>
+        <v>15.8</v>
       </c>
       <c r="H76" t="str">
         <v>Thais Tarcia de Araujo Oliveira</v>
@@ -2767,7 +2767,7 @@
         <v>Maria das Neves Nascimento Galdino</v>
       </c>
       <c r="G77">
-        <v>14.4</v>
+        <v>3.1</v>
       </c>
       <c r="H77" t="str">
         <v>Thais Tarcia de Araujo Oliveira</v>
@@ -2796,7 +2796,7 @@
         <v>Marileide Porto Fontana</v>
       </c>
       <c r="G78">
-        <v>12.9</v>
+        <v>13.9</v>
       </c>
       <c r="H78" t="str">
         <v>Thais Tarcia de Araujo Oliveira</v>
@@ -2825,7 +2825,7 @@
         <v>Neiva Cristiane Bortolato Goncalves</v>
       </c>
       <c r="G79">
-        <v>7</v>
+        <v>19.9</v>
       </c>
       <c r="H79" t="str">
         <v>Thais Tarcia de Araujo Oliveira</v>
@@ -2854,7 +2854,7 @@
         <v>Neusa Maria Kaiser</v>
       </c>
       <c r="G80">
-        <v>12.7</v>
+        <v>11.1</v>
       </c>
       <c r="H80" t="str">
         <v>Thais Tarcia de Araujo Oliveira</v>
@@ -2883,7 +2883,7 @@
         <v>Terisley Rodrigues Ferreira</v>
       </c>
       <c r="G81">
-        <v>23.8</v>
+        <v>21.9</v>
       </c>
       <c r="H81" t="str">
         <v>Thais Tarcia de Araujo Oliveira</v>
@@ -2912,7 +2912,7 @@
         <v>Samuel Santana Barreto</v>
       </c>
       <c r="G82">
-        <v>15.8</v>
+        <v>5.2</v>
       </c>
       <c r="H82" t="str">
         <v>Frank Soares do Nascimento</v>
@@ -2941,7 +2941,7 @@
         <v>Lincoln Eduardo Nunes</v>
       </c>
       <c r="G83">
-        <v>3.1</v>
+        <v>4.6</v>
       </c>
       <c r="H83" t="str">
         <v>Edson Oleksyw</v>
@@ -2970,7 +2970,7 @@
         <v>Max Antunes Cavalheiro</v>
       </c>
       <c r="G84">
-        <v>13.9</v>
+        <v>9.7</v>
       </c>
       <c r="H84" t="str">
         <v>Julio Cezar da Silva</v>
@@ -2999,7 +2999,7 @@
         <v>Edwagner Tourinho de Oliveira</v>
       </c>
       <c r="G85">
-        <v>19.9</v>
+        <v>10.5</v>
       </c>
       <c r="H85" t="str">
         <v>Cidclei Reck</v>
@@ -3028,7 +3028,7 @@
         <v>Guilherme Misak Vivian</v>
       </c>
       <c r="G86">
-        <v>11.1</v>
+        <v>15.1</v>
       </c>
       <c r="H86" t="str">
         <v>Orlando Rodrigues Neto</v>
@@ -3057,7 +3057,7 @@
         <v>Rodrigo da Veiga Lima</v>
       </c>
       <c r="G87">
-        <v>21.9</v>
+        <v>21.2</v>
       </c>
       <c r="H87" t="str">
         <v>Viviane Thomaz</v>
@@ -3086,7 +3086,7 @@
         <v>Michely Larissa Tonhi de O. Buzinhani</v>
       </c>
       <c r="G88">
-        <v>5.2</v>
+        <v>19.9</v>
       </c>
       <c r="H88" t="str">
         <v>Viviane Thomaz</v>
@@ -3115,7 +3115,7 @@
         <v>Thiago Carvalho Ferreira</v>
       </c>
       <c r="G89">
-        <v>4.6</v>
+        <v>4.4</v>
       </c>
       <c r="H89" t="str">
         <v>Viviane Thomaz</v>
@@ -3144,7 +3144,7 @@
         <v>Priscila Giomo</v>
       </c>
       <c r="G90">
-        <v>9.7</v>
+        <v>5.9</v>
       </c>
       <c r="H90" t="str">
         <v>Viviane Thomaz</v>
@@ -3173,7 +3173,7 @@
         <v>Viviane Thomaz</v>
       </c>
       <c r="G91">
-        <v>10.5</v>
+        <v>4.2</v>
       </c>
       <c r="H91" t="str">
         <v>Gilmar Alves de Oliveira</v>
@@ -3202,7 +3202,7 @@
         <v>Milene Thomaz Romano Gantzel</v>
       </c>
       <c r="G92">
-        <v>15.1</v>
+        <v>15.7</v>
       </c>
       <c r="H92" t="str">
         <v>Viviane Thomaz</v>
@@ -3231,7 +3231,7 @@
         <v>Celso Nobuyuki Yokota</v>
       </c>
       <c r="G93">
-        <v>21.2</v>
+        <v>5.9</v>
       </c>
       <c r="H93" t="str">
         <v>Viviane Thomaz</v>
@@ -3260,7 +3260,7 @@
         <v>Ana Paula Franco Prodoscimo Sarti</v>
       </c>
       <c r="G94">
-        <v>19.9</v>
+        <v>9.2</v>
       </c>
       <c r="H94" t="str">
         <v>Viviane Thomaz</v>
@@ -3289,7 +3289,7 @@
         <v>Maria Aparecida Canella</v>
       </c>
       <c r="G95">
-        <v>4.4</v>
+        <v>22.4</v>
       </c>
       <c r="H95" t="str">
         <v>Celio Roberto Cantuarios</v>
@@ -3318,7 +3318,7 @@
         <v>Edson Guedes de Sousa</v>
       </c>
       <c r="G96">
-        <v>5.9</v>
+        <v>14.5</v>
       </c>
       <c r="H96" t="str">
         <v>Celio Roberto Cantuarios</v>
@@ -3347,7 +3347,7 @@
         <v>Franciele Fritsch da Silva</v>
       </c>
       <c r="G97">
-        <v>4.2</v>
+        <v>9.1</v>
       </c>
       <c r="H97" t="str">
         <v>Celio Roberto Cantuarios</v>
@@ -3376,7 +3376,7 @@
         <v>Heitor Henrique Bataiero</v>
       </c>
       <c r="G98">
-        <v>15.7</v>
+        <v>13.3</v>
       </c>
       <c r="H98" t="str">
         <v>Celio Roberto Cantuarios</v>
@@ -3405,7 +3405,7 @@
         <v>Rafael Marques da Silva</v>
       </c>
       <c r="G99">
-        <v>5.9</v>
+        <v>23.7</v>
       </c>
       <c r="H99" t="str">
         <v>Celio Roberto Cantuarios</v>
@@ -3434,7 +3434,7 @@
         <v>Renan Gomes Casagrande</v>
       </c>
       <c r="G100">
-        <v>9.2</v>
+        <v>20.5</v>
       </c>
       <c r="H100" t="str">
         <v>Celio Roberto Cantuarios</v>
@@ -3463,7 +3463,7 @@
         <v>Rogelio dos Santos Vargas</v>
       </c>
       <c r="G101">
-        <v>22.4</v>
+        <v>10.3</v>
       </c>
       <c r="H101" t="str">
         <v>Celio Roberto Cantuarios</v>
@@ -3492,7 +3492,7 @@
         <v>Teilo de Jesus Santana</v>
       </c>
       <c r="G102">
-        <v>14.5</v>
+        <v>3.3</v>
       </c>
       <c r="H102" t="str">
         <v>Celio Roberto Cantuarios</v>
@@ -3521,7 +3521,7 @@
         <v>Willian Fernando Cruz Alves</v>
       </c>
       <c r="G103">
-        <v>9.1</v>
+        <v>2.5</v>
       </c>
       <c r="H103" t="str">
         <v>Celio Roberto Cantuarios</v>
@@ -3550,7 +3550,7 @@
         <v>Marcos Antonio Utsunomiya</v>
       </c>
       <c r="G104">
-        <v>13.3</v>
+        <v>20.8</v>
       </c>
       <c r="H104" t="str">
         <v>Gilmar Alves de Oliveira</v>
@@ -3579,7 +3579,7 @@
         <v>Celio Roberto Cantuarios</v>
       </c>
       <c r="G105">
-        <v>23.7</v>
+        <v>23.1</v>
       </c>
       <c r="H105" t="str">
         <v>Marcos Antonio Utsunomiya</v>
@@ -3608,7 +3608,7 @@
         <v>Luis Carlos da Costa Junior</v>
       </c>
       <c r="G106">
-        <v>20.5</v>
+        <v>12.9</v>
       </c>
       <c r="H106" t="str">
         <v>Marcos Antonio Utsunomiya</v>
@@ -3637,7 +3637,7 @@
         <v>Acleilton de Souza Lima</v>
       </c>
       <c r="G107">
-        <v>10.3</v>
+        <v>3.5</v>
       </c>
       <c r="H107" t="str">
         <v>Luis Carlos da Costa Junior</v>
@@ -3666,7 +3666,7 @@
         <v>Benjamin Dene de Carvalho Junior</v>
       </c>
       <c r="G108">
-        <v>3.3</v>
+        <v>16.6</v>
       </c>
       <c r="H108" t="str">
         <v>Luis Carlos da Costa Junior</v>
@@ -3695,7 +3695,7 @@
         <v>Diego Alisson de Lima Borges</v>
       </c>
       <c r="G109">
-        <v>2.5</v>
+        <v>17.6</v>
       </c>
       <c r="H109" t="str">
         <v>Luis Carlos da Costa Junior</v>
@@ -3724,7 +3724,7 @@
         <v>Eduardo Roberto da Silva</v>
       </c>
       <c r="G110">
-        <v>20.8</v>
+        <v>14.5</v>
       </c>
       <c r="H110" t="str">
         <v>Luis Carlos da Costa Junior</v>
@@ -3753,7 +3753,7 @@
         <v>Gabriel Pereira Fontaneli</v>
       </c>
       <c r="G111">
-        <v>23.1</v>
+        <v>4.1</v>
       </c>
       <c r="H111" t="str">
         <v>Luis Carlos da Costa Junior</v>
@@ -3782,7 +3782,7 @@
         <v>Juliano Bueno da Silva Oliveira</v>
       </c>
       <c r="G112">
-        <v>12.9</v>
+        <v>18.4</v>
       </c>
       <c r="H112" t="str">
         <v>Luis Carlos da Costa Junior</v>
@@ -3811,7 +3811,7 @@
         <v>Mauricio Barboza de Souza</v>
       </c>
       <c r="G113">
-        <v>3.5</v>
+        <v>18.9</v>
       </c>
       <c r="H113" t="str">
         <v>Luis Carlos da Costa Junior</v>
@@ -3840,7 +3840,7 @@
         <v>Raimundo Nonato Silva Amaral</v>
       </c>
       <c r="G114">
-        <v>16.6</v>
+        <v>8.8</v>
       </c>
       <c r="H114" t="str">
         <v>Luis Carlos da Costa Junior</v>
@@ -3869,7 +3869,7 @@
         <v>Renato da Silva Oliveira</v>
       </c>
       <c r="G115">
-        <v>17.6</v>
+        <v>25</v>
       </c>
       <c r="H115" t="str">
         <v>Luis Carlos da Costa Junior</v>
@@ -3898,7 +3898,7 @@
         <v>Sidnei Francisco da Silva</v>
       </c>
       <c r="G116">
-        <v>14.5</v>
+        <v>19.4</v>
       </c>
       <c r="H116" t="str">
         <v>Luis Carlos da Costa Junior</v>
@@ -3927,7 +3927,7 @@
         <v>Donizete Denilson Giomo</v>
       </c>
       <c r="G117">
-        <v>4.1</v>
+        <v>18.7</v>
       </c>
       <c r="H117" t="str">
         <v>Celio Roberto Cantuarios</v>
@@ -3956,7 +3956,7 @@
         <v>Vanderlei de Souza Gonçalo</v>
       </c>
       <c r="G118">
-        <v>18.4</v>
+        <v>1.3</v>
       </c>
       <c r="H118" t="str">
         <v>Marcos Antonio Utsunomiya</v>
@@ -3985,7 +3985,7 @@
         <v>Elessandro Alves da Silva</v>
       </c>
       <c r="G119">
-        <v>18.9</v>
+        <v>18.1</v>
       </c>
       <c r="H119" t="str">
         <v>Celio Roberto Cantuarios</v>
@@ -4014,7 +4014,7 @@
         <v>Jonismar Antonio dos Santos</v>
       </c>
       <c r="G120">
-        <v>8.8</v>
+        <v>19.6</v>
       </c>
       <c r="H120" t="str">
         <v>Celio Roberto Cantuarios</v>
@@ -4043,7 +4043,7 @@
         <v>Robson Muniz de Morais</v>
       </c>
       <c r="G121">
-        <v>25</v>
+        <v>23.2</v>
       </c>
       <c r="H121" t="str">
         <v>Celio Roberto Cantuarios</v>
@@ -4072,7 +4072,7 @@
         <v>Alexsandro Bataieiro</v>
       </c>
       <c r="G122">
-        <v>19.4</v>
+        <v>23.3</v>
       </c>
       <c r="H122" t="str">
         <v>Marcos Antonio Utsunomiya</v>
@@ -4101,7 +4101,7 @@
         <v>Edson Oleksyw</v>
       </c>
       <c r="G123">
-        <v>18.7</v>
+        <v>18.2</v>
       </c>
       <c r="H123" t="str">
         <v>Gilmar Alves de Oliveira</v>
@@ -4130,7 +4130,7 @@
         <v>Evaldo Barbosa Cavalcante</v>
       </c>
       <c r="G124">
-        <v>1.3</v>
+        <v>9.1</v>
       </c>
       <c r="H124" t="str">
         <v>Edson Oleksyw</v>
@@ -4159,7 +4159,7 @@
         <v>Francisco de Paula Junior</v>
       </c>
       <c r="G125">
-        <v>18.1</v>
+        <v>4.5</v>
       </c>
       <c r="H125" t="str">
         <v>Alex Coronado dos Santos</v>
@@ -4188,7 +4188,7 @@
         <v>Fabner Roberto Soares</v>
       </c>
       <c r="G126">
-        <v>19.6</v>
+        <v>14.2</v>
       </c>
       <c r="H126" t="str">
         <v>Alex Coronado dos Santos</v>
@@ -4217,7 +4217,7 @@
         <v>Junior Gil Custodio</v>
       </c>
       <c r="G127">
-        <v>23.2</v>
+        <v>20.5</v>
       </c>
       <c r="H127" t="str">
         <v>Alex Coronado dos Santos</v>
@@ -4246,7 +4246,7 @@
         <v>Danilo Mulizine Stochi</v>
       </c>
       <c r="G128">
-        <v>23.3</v>
+        <v>19.5</v>
       </c>
       <c r="H128" t="str">
         <v>Alex Coronado dos Santos</v>
@@ -4275,7 +4275,7 @@
         <v>Ricardo Brito Soares</v>
       </c>
       <c r="G129">
-        <v>18.2</v>
+        <v>9.4</v>
       </c>
       <c r="H129" t="str">
         <v>Gilmar Alves de Oliveira</v>
@@ -4304,7 +4304,7 @@
         <v>Alex Coronado dos Santos</v>
       </c>
       <c r="G130">
-        <v>9.1</v>
+        <v>10.8</v>
       </c>
       <c r="H130" t="str">
         <v>Ricardo Brito Soares</v>
@@ -4333,7 +4333,7 @@
         <v>Kleverson Ricardo de Melo</v>
       </c>
       <c r="G131">
-        <v>4.5</v>
+        <v>8.7</v>
       </c>
       <c r="H131" t="str">
         <v>Alex Coronado dos Santos</v>
@@ -4362,7 +4362,7 @@
         <v>Rogerio Tsuyoshi Arida</v>
       </c>
       <c r="G132">
-        <v>14.2</v>
+        <v>23.6</v>
       </c>
       <c r="H132" t="str">
         <v>Alex Coronado dos Santos</v>
@@ -4391,7 +4391,7 @@
         <v>Joel Correia Junior</v>
       </c>
       <c r="G133">
-        <v>20.5</v>
+        <v>1.3</v>
       </c>
       <c r="H133" t="str">
         <v>Alex Coronado dos Santos</v>
@@ -4420,7 +4420,7 @@
         <v>Anderson Rodrigo Giomo</v>
       </c>
       <c r="G134">
-        <v>19.5</v>
+        <v>16.9</v>
       </c>
       <c r="H134" t="str">
         <v>Alex Coronado dos Santos</v>
@@ -4449,7 +4449,7 @@
         <v>Rodrigo Romano Gantzel</v>
       </c>
       <c r="G135">
-        <v>9.4</v>
+        <v>13.1</v>
       </c>
       <c r="H135" t="str">
         <v>Alex Coronado dos Santos</v>
@@ -4478,7 +4478,7 @@
         <v>Cadmiel Cristiano de Grande</v>
       </c>
       <c r="G136">
-        <v>10.8</v>
+        <v>17.1</v>
       </c>
       <c r="H136" t="str">
         <v>Rodrigo Romano Gantzel</v>
@@ -4507,7 +4507,7 @@
         <v>Edson Macoto Tamura Junior</v>
       </c>
       <c r="G137">
-        <v>8.7</v>
+        <v>14.8</v>
       </c>
       <c r="H137" t="str">
         <v>Alex Coronado dos Santos</v>
@@ -4536,7 +4536,7 @@
         <v>Fernando Sanches Graci</v>
       </c>
       <c r="G138">
-        <v>23.6</v>
+        <v>1.6</v>
       </c>
       <c r="H138" t="str">
         <v>Gilmar Alves de Oliveira</v>
@@ -4565,7 +4565,7 @@
         <v>Joao Everton Ramos</v>
       </c>
       <c r="G139">
-        <v>1.3</v>
+        <v>9.1</v>
       </c>
       <c r="H139" t="str">
         <v>Maykon Fernando da Costa</v>
@@ -4594,7 +4594,7 @@
         <v>Ademar Alencar Jardim Junior</v>
       </c>
       <c r="G140">
-        <v>16.9</v>
+        <v>8</v>
       </c>
       <c r="H140" t="str">
         <v>Maykon Fernando da Costa</v>
@@ -4623,7 +4623,7 @@
         <v>Anderson Izidoro da Silva</v>
       </c>
       <c r="G141">
-        <v>13.1</v>
+        <v>10.8</v>
       </c>
       <c r="H141" t="str">
         <v>Fernando Sanches Graci</v>
@@ -4652,7 +4652,7 @@
         <v>Natanael Estevao Chagas Moraes</v>
       </c>
       <c r="G142">
-        <v>17.1</v>
+        <v>20.5</v>
       </c>
       <c r="H142" t="str">
         <v>Fernando Sanches Graci</v>
@@ -4681,7 +4681,7 @@
         <v>Celia Xavier Novo</v>
       </c>
       <c r="G143">
-        <v>14.8</v>
+        <v>24.3</v>
       </c>
       <c r="H143" t="str">
         <v>Fernando Sanches Graci</v>
@@ -4710,7 +4710,7 @@
         <v>Maykon Fernando da Costa</v>
       </c>
       <c r="G144">
-        <v>1.6</v>
+        <v>24.5</v>
       </c>
       <c r="H144" t="str">
         <v>Fernando Sanches Graci</v>
@@ -4739,7 +4739,7 @@
         <v>Jessica Fonzar da Silva</v>
       </c>
       <c r="G145">
-        <v>9.1</v>
+        <v>20.7</v>
       </c>
       <c r="H145" t="str">
         <v>Ademar Alencar Jardim Junior</v>
@@ -4768,7 +4768,7 @@
         <v>Maiara Cristine de Jesus Vieira</v>
       </c>
       <c r="G146">
-        <v>8</v>
+        <v>21.4</v>
       </c>
       <c r="H146" t="str">
         <v>Ademar Alencar Jardim Junior</v>
@@ -4797,7 +4797,7 @@
         <v>Maria Eduarda Matos Medeiros</v>
       </c>
       <c r="G147">
-        <v>10.8</v>
+        <v>13.1</v>
       </c>
       <c r="H147" t="str">
         <v>Ademar Alencar Jardim Junior</v>
@@ -4826,7 +4826,7 @@
         <v>Natiara Rodrigues dos Santos Vieira</v>
       </c>
       <c r="G148">
-        <v>20.5</v>
+        <v>16.5</v>
       </c>
       <c r="H148" t="str">
         <v>Ademar Alencar Jardim Junior</v>
@@ -4855,7 +4855,7 @@
         <v>Priscila Andrelina da Silva Bartolomeu</v>
       </c>
       <c r="G149">
-        <v>24.3</v>
+        <v>1.1</v>
       </c>
       <c r="H149" t="str">
         <v>Ademar Alencar Jardim Junior</v>
@@ -4884,7 +4884,7 @@
         <v>Thomas Jefesson Soares de Souza</v>
       </c>
       <c r="G150">
-        <v>24.5</v>
+        <v>20.2</v>
       </c>
       <c r="H150" t="str">
         <v>Ademar Alencar Jardim Junior</v>
@@ -4913,7 +4913,7 @@
         <v>Antonio Raimundo Santos de Mendonca</v>
       </c>
       <c r="G151">
-        <v>20.7</v>
+        <v>6.3</v>
       </c>
       <c r="H151" t="str">
         <v>Ademar Alencar Jardim Junior</v>
@@ -4942,7 +4942,7 @@
         <v>Fernando da Silva Dias</v>
       </c>
       <c r="G152">
-        <v>21.4</v>
+        <v>20.2</v>
       </c>
       <c r="H152" t="str">
         <v>Ademar Alencar Jardim Junior</v>
@@ -4971,7 +4971,7 @@
         <v>Iuri Barroso Pinheiro</v>
       </c>
       <c r="G153">
-        <v>13.1</v>
+        <v>18.3</v>
       </c>
       <c r="H153" t="str">
         <v>Ademar Alencar Jardim Junior</v>
@@ -5000,7 +5000,7 @@
         <v>Jordy Alesson Souza Monteiro</v>
       </c>
       <c r="G154">
-        <v>16.5</v>
+        <v>1.9</v>
       </c>
       <c r="H154" t="str">
         <v>Ademar Alencar Jardim Junior</v>
@@ -5029,7 +5029,7 @@
         <v>Danilo Moureira Niza da Silva</v>
       </c>
       <c r="G155">
-        <v>1.1</v>
+        <v>23.3</v>
       </c>
       <c r="H155" t="str">
         <v>Edgar Zaleski</v>
@@ -5058,7 +5058,7 @@
         <v>Maicon Aurelio Trovo</v>
       </c>
       <c r="G156">
-        <v>20.2</v>
+        <v>18.7</v>
       </c>
       <c r="H156" t="str">
         <v>Gilmar Alves de Oliveira</v>
@@ -5087,7 +5087,7 @@
         <v>Rodrigo de Oliveira Novo</v>
       </c>
       <c r="G157">
-        <v>6.3</v>
+        <v>18.9</v>
       </c>
       <c r="H157" t="str">
         <v>Maicon Aurelio Trovo</v>
@@ -5116,7 +5116,7 @@
         <v>Francisca Marisangela de Jesus Sousa</v>
       </c>
       <c r="G158">
-        <v>20.2</v>
+        <v>15.6</v>
       </c>
       <c r="H158" t="str">
         <v>Everson Oliveira Lima</v>
@@ -5145,7 +5145,7 @@
         <v>Jefson Henrique de Jesus Santos</v>
       </c>
       <c r="G159">
-        <v>18.3</v>
+        <v>12.2</v>
       </c>
       <c r="H159" t="str">
         <v>Rafael Tomaz Mariano</v>
@@ -5174,7 +5174,7 @@
         <v>Luan Gabriel Schroeder</v>
       </c>
       <c r="G160">
-        <v>1.9</v>
+        <v>6.8</v>
       </c>
       <c r="H160" t="str">
         <v>Vinicios Zuse</v>
@@ -5203,7 +5203,7 @@
         <v>Luiz Henrique Martins Trench</v>
       </c>
       <c r="G161">
-        <v>23.3</v>
+        <v>7.6</v>
       </c>
       <c r="H161" t="str">
         <v>Marcos de Oliveira Souza</v>
@@ -5232,7 +5232,7 @@
         <v>Ricardo Poteriko Sobrinho</v>
       </c>
       <c r="G162">
-        <v>18.7</v>
+        <v>20.7</v>
       </c>
       <c r="H162" t="str">
         <v>Edgar Zaleski</v>
@@ -5261,7 +5261,7 @@
         <v>Roberto Ricardo Buth</v>
       </c>
       <c r="G163">
-        <v>18.9</v>
+        <v>16.5</v>
       </c>
       <c r="H163" t="str">
         <v>Anderson Furlan Karnopp</v>
@@ -5290,7 +5290,7 @@
         <v>Yuri Ignochevski Primao</v>
       </c>
       <c r="G164">
-        <v>15.6</v>
+        <v>19.6</v>
       </c>
       <c r="H164" t="str">
         <v>Caio Henrique Macedo Garcia</v>
@@ -5319,7 +5319,7 @@
         <v>Anderson Furlan Karnopp</v>
       </c>
       <c r="G165">
-        <v>12.2</v>
+        <v>13.5</v>
       </c>
       <c r="H165" t="str">
         <v>Maicon Aurélio Trovo</v>
@@ -5348,7 +5348,7 @@
         <v>Caio Henrique Macedo Garcia</v>
       </c>
       <c r="G166">
-        <v>6.8</v>
+        <v>3.6</v>
       </c>
       <c r="H166" t="str">
         <v>Maicon Aurélio Trovo</v>
@@ -5377,7 +5377,7 @@
         <v>Edgar Zaleski</v>
       </c>
       <c r="G167">
-        <v>7.6</v>
+        <v>12.3</v>
       </c>
       <c r="H167" t="str">
         <v>Maicon Aurélio Trovo</v>
@@ -5406,7 +5406,7 @@
         <v>Everson Oliveira Lima</v>
       </c>
       <c r="G168">
-        <v>20.7</v>
+        <v>14.6</v>
       </c>
       <c r="H168" t="str">
         <v>Maicon Aurélio Trovo</v>
@@ -5435,7 +5435,7 @@
         <v>Juliana Severo Arantes</v>
       </c>
       <c r="G169">
-        <v>16.5</v>
+        <v>3.8</v>
       </c>
       <c r="H169" t="str">
         <v>Maicon Aurélio Trovo</v>
@@ -5464,7 +5464,7 @@
         <v>Marcos de Oliveira Souza</v>
       </c>
       <c r="G170">
-        <v>19.6</v>
+        <v>20.5</v>
       </c>
       <c r="H170" t="str">
         <v>Maicon Aurélio Trovo</v>
@@ -5493,7 +5493,7 @@
         <v>Rafael Tomaz Mariano</v>
       </c>
       <c r="G171">
-        <v>13.5</v>
+        <v>14</v>
       </c>
       <c r="H171" t="str">
         <v>Maicon Aurélio Trovo</v>
@@ -5522,7 +5522,7 @@
         <v>Vinicios Zuse</v>
       </c>
       <c r="G172">
-        <v>3.6</v>
+        <v>4.2</v>
       </c>
       <c r="H172" t="str">
         <v>Maicon Aurélio Trovo</v>
@@ -5551,7 +5551,7 @@
         <v>Marcus Vinicius Cabeça Pereira</v>
       </c>
       <c r="G173">
-        <v>12.3</v>
+        <v>17.8</v>
       </c>
       <c r="H173" t="str">
         <v>Maicon Aurélio Trovo</v>
@@ -5580,7 +5580,7 @@
         <v>Eduardo Giacometti Xavier</v>
       </c>
       <c r="G174">
-        <v>14.6</v>
+        <v>11.2</v>
       </c>
       <c r="H174" t="str">
         <v>Maicon Aurélio Trovo</v>
@@ -5609,7 +5609,7 @@
         <v>Iago Fernando Luiz</v>
       </c>
       <c r="G175">
-        <v>3.8</v>
+        <v>9.3</v>
       </c>
       <c r="H175" t="str">
         <v>Maicon Aurélio Trovo</v>
@@ -5638,7 +5638,7 @@
         <v>Denise Avelino da Silva Fattore</v>
       </c>
       <c r="G176">
-        <v>20.5</v>
+        <v>16.1</v>
       </c>
       <c r="H176" t="str">
         <v>Gilmar Alves de Oliveira</v>
@@ -5667,7 +5667,7 @@
         <v>Keno Carlos Pratis de Oliveira</v>
       </c>
       <c r="G177">
-        <v>14</v>
+        <v>17.3</v>
       </c>
       <c r="H177" t="str">
         <v>Gilmar Alves de Oliveira</v>
@@ -5696,7 +5696,7 @@
         <v>Marcos Henrique Sabec</v>
       </c>
       <c r="G178">
-        <v>4.2</v>
+        <v>17.9</v>
       </c>
       <c r="H178" t="str">
         <v>Gilmar Alves de Oliveira</v>
@@ -5725,7 +5725,7 @@
         <v>Carla Francieli Fernandes dos Anjos</v>
       </c>
       <c r="G179">
-        <v>17.8</v>
+        <v>4.6</v>
       </c>
       <c r="H179" t="str">
         <v>Alessandra Guerra de Souza</v>
@@ -5754,7 +5754,7 @@
         <v>Paulo da Silva Braz</v>
       </c>
       <c r="G180">
-        <v>11.2</v>
+        <v>10.1</v>
       </c>
       <c r="H180" t="str">
         <v>Alessandra Guerra de Souza</v>
@@ -5783,7 +5783,7 @@
         <v>Elton Fernando Hoshino</v>
       </c>
       <c r="G181">
-        <v>9.3</v>
+        <v>3.2</v>
       </c>
       <c r="H181" t="str">
         <v>Alessandra Guerra de Souza</v>
@@ -5792,16 +5792,45 @@
         <v>Gerente geral de recursos humanos</v>
       </c>
     </row>
+    <row r="182">
+      <c r="A182" t="str">
+        <v>c181</v>
+      </c>
+      <c r="B182" t="str">
+        <v>Gerente geral de recursos humanos</v>
+      </c>
+      <c r="C182" t="str">
+        <v>Gerência Executiva</v>
+      </c>
+      <c r="D182" t="str">
+        <v>Gerente geral de recursos humanos</v>
+      </c>
+      <c r="E182" t="str">
+        <v>Douradina/PR</v>
+      </c>
+      <c r="F182" t="str">
+        <v>Alessandra Guerra de Souza</v>
+      </c>
+      <c r="G182">
+        <v>9.5</v>
+      </c>
+      <c r="H182" t="str">
+        <v>Gilmar Alves de Oliveira</v>
+      </c>
+      <c r="I182" t="str">
+        <v>Presidente</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I181"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I182"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R219"/>
+  <dimension ref="A1:R220"/>
   <cols>
     <col min="1" max="1" width="40.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -5920,10 +5949,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N2" t="str">
-        <v>Alguém assume com suporte</v>
+        <v>Não identifico sucessor</v>
       </c>
       <c r="O2" t="str">
-        <v>João Pedro Cardoso Jardim</v>
+        <v/>
       </c>
       <c r="P2" t="str">
         <v>Alto Desempenho</v>
@@ -6315,7 +6344,7 @@
         <v>Alguém assume com suporte</v>
       </c>
       <c r="O9" t="str">
-        <v>Bruna Guimarães Queiroz</v>
+        <v>Daniela Queiroz Xavier</v>
       </c>
       <c r="P9" t="str">
         <v>Empregado Sólido / Responsável</v>
@@ -7211,7 +7240,7 @@
         <v>Alguém assume imediatamente</v>
       </c>
       <c r="O25" t="str">
-        <v>Daiane Domingues dos Santos, Raquel Cristina Vidotto Ramos</v>
+        <v>Letícia Zanella Damasceno</v>
       </c>
       <c r="P25" t="str">
         <v>Empregado Comprometido</v>
@@ -7264,7 +7293,7 @@
         <v>Não</v>
       </c>
       <c r="N26" t="str">
-        <v>Sem elementos para avaliar</v>
+        <v>Não identifico sucessor</v>
       </c>
       <c r="O26" t="str">
         <v/>
@@ -7320,10 +7349,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N27" t="str">
-        <v>Alguém assume com suporte</v>
+        <v>Sem elementos para avaliar</v>
       </c>
       <c r="O27" t="str">
-        <v>Lincoln Eduardo Nunes, Eduarda Meireles</v>
+        <v/>
       </c>
       <c r="P27" t="str">
         <v>Alto Desempenho</v>
@@ -7364,7 +7393,7 @@
         <v>Visão financeira do negócio (DRE, orçamento)</v>
       </c>
       <c r="J28" t="str">
-        <v>Gerente administrativo de logística</v>
+        <v>Gerente de assistência</v>
       </c>
       <c r="K28" t="str">
         <v>Mais de 3 até 5 anos</v>
@@ -7376,10 +7405,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N28" t="str">
-        <v>Não identifico sucessor</v>
+        <v>Alguém assume imediatamente</v>
       </c>
       <c r="O28" t="str">
-        <v/>
+        <v>Daniela Guimarães Valadares</v>
       </c>
       <c r="P28" t="str">
         <v>Estrela</v>
@@ -7432,10 +7461,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N29" t="str">
-        <v>Não identifico sucessor</v>
+        <v>Alguém assume com suporte</v>
       </c>
       <c r="O29" t="str">
-        <v/>
+        <v>Frank Soares do Nascimento, Adson Nogueira da Silva</v>
       </c>
       <c r="P29" t="str">
         <v>Empregado Eficaz</v>
@@ -7488,10 +7517,10 @@
         <v>Não</v>
       </c>
       <c r="N30" t="str">
-        <v>Não identifico sucessor</v>
+        <v>Alguém assume com suporte</v>
       </c>
       <c r="O30" t="str">
-        <v/>
+        <v>Beatriz Kroetzler</v>
       </c>
       <c r="P30" t="str">
         <v>Empregado Eficaz</v>
@@ -7523,7 +7552,7 @@
         <v>Total (qualquer unidade)</v>
       </c>
       <c r="G31" t="str">
-        <v>Gerente de auditoria</v>
+        <v>Gerente geral agropecuária</v>
       </c>
       <c r="H31" t="str">
         <v>Mais de 5 anos</v>
@@ -7544,10 +7573,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N31" t="str">
-        <v>Alguém assume imediatamente</v>
+        <v>Não identifico sucessor</v>
       </c>
       <c r="O31" t="str">
-        <v>Andreza Miranda da Silva</v>
+        <v/>
       </c>
       <c r="P31" t="str">
         <v>Empregado Comprometido</v>
@@ -7635,7 +7664,7 @@
         <v>Matriz (Douradina/PR)</v>
       </c>
       <c r="G33" t="str">
-        <v>Gerente geral</v>
+        <v>Gerente administrativo da indústria</v>
       </c>
       <c r="H33" t="str">
         <v>Imediato</v>
@@ -7656,7 +7685,7 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="N33" t="str">
-        <v>Alguém assume com suporte</v>
+        <v>Alguém assume imediatamente</v>
       </c>
       <c r="O33" t="str">
         <v>Elton Fernando Hoshino</v>
@@ -7768,10 +7797,10 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="N35" t="str">
-        <v>Não identifico sucessor</v>
+        <v>Alguém assume com suporte</v>
       </c>
       <c r="O35" t="str">
-        <v/>
+        <v>Neiva Goncalves</v>
       </c>
       <c r="P35" t="str">
         <v>Alto Desempenho</v>
@@ -7824,10 +7853,10 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="N36" t="str">
-        <v>Alguém assume com suporte</v>
+        <v>Não identifico sucessor</v>
       </c>
       <c r="O36" t="str">
-        <v>Nicareli Neves</v>
+        <v/>
       </c>
       <c r="P36" t="str">
         <v>Risco / Baixo Desempenho</v>
@@ -7880,10 +7909,10 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="N37" t="str">
-        <v>Não identifico sucessor</v>
+        <v>Alguém assume com suporte</v>
       </c>
       <c r="O37" t="str">
-        <v/>
+        <v>Juliano de Albuquerque Silva</v>
       </c>
       <c r="P37" t="str">
         <v>Empregado Comprometido</v>
@@ -7936,10 +7965,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N38" t="str">
-        <v>Alguém assume com suporte</v>
+        <v>Alguém assume imediatamente</v>
       </c>
       <c r="O38" t="str">
-        <v>Milene Thomaz Romano Gantzel</v>
+        <v>Marcio Adriano Leme</v>
       </c>
       <c r="P38" t="str">
         <v>Empregado Comprometido</v>
@@ -7992,10 +8021,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N39" t="str">
-        <v>Alguém assume imediatamente</v>
+        <v>Alguém assume com suporte</v>
       </c>
       <c r="O39" t="str">
-        <v>Beatriz Santos Kroetzler</v>
+        <v>Elisandra Santos</v>
       </c>
       <c r="P39" t="str">
         <v>Estrela</v>
@@ -8048,10 +8077,10 @@
         <v>Não</v>
       </c>
       <c r="N40" t="str">
-        <v>Alguém assume com suporte</v>
+        <v>Não identifico sucessor</v>
       </c>
       <c r="O40" t="str">
-        <v>Terisley Ferreira</v>
+        <v/>
       </c>
       <c r="P40" t="str">
         <v>Empregado Sólido / Responsável</v>
@@ -8160,10 +8189,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N42" t="str">
-        <v>Não identifico sucessor</v>
+        <v>Alguém assume com suporte</v>
       </c>
       <c r="O42" t="str">
-        <v/>
+        <v>Terisley Rodrigues Ferreira</v>
       </c>
       <c r="P42" t="str">
         <v>Empregado Comprometido</v>
@@ -8216,10 +8245,10 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="N43" t="str">
-        <v>Alguém assume com suporte</v>
+        <v>Sem elementos para avaliar</v>
       </c>
       <c r="O43" t="str">
-        <v>Terisley Rodrigues Ferreira</v>
+        <v/>
       </c>
       <c r="P43" t="str">
         <v>Empregado Comprometido</v>
@@ -8272,7 +8301,7 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N44" t="str">
-        <v>Sem elementos para avaliar</v>
+        <v>Não identifico sucessor</v>
       </c>
       <c r="O44" t="str">
         <v/>
@@ -8307,7 +8336,7 @@
         <v>Local atual</v>
       </c>
       <c r="G45" t="str">
-        <v>Gerente administrativo da indústria</v>
+        <v>Gerente de indústria</v>
       </c>
       <c r="H45" t="str">
         <v>Até 3 anos</v>
@@ -8328,10 +8357,10 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="N45" t="str">
-        <v>Não identifico sucessor</v>
+        <v>Alguém assume imediatamente</v>
       </c>
       <c r="O45" t="str">
-        <v/>
+        <v>Priscila Giomo</v>
       </c>
       <c r="P45" t="str">
         <v>Empregado Sólido / Responsável</v>
@@ -8440,10 +8469,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N47" t="str">
-        <v>Alguém assume imediatamente</v>
+        <v>Não identifico sucessor</v>
       </c>
       <c r="O47" t="str">
-        <v>Guilherme Caetano Gelamos</v>
+        <v/>
       </c>
       <c r="P47" t="str">
         <v>Bom Executor / Especialista</v>
@@ -8496,10 +8525,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N48" t="str">
-        <v>Não identifico sucessor</v>
+        <v>Alguém assume com suporte</v>
       </c>
       <c r="O48" t="str">
-        <v/>
+        <v>Bruno Martins, Odimar Antonio de Oliveira</v>
       </c>
       <c r="P48" t="str">
         <v>Empregado Sólido / Responsável</v>
@@ -8552,10 +8581,10 @@
         <v>Não</v>
       </c>
       <c r="N49" t="str">
-        <v>Alguém assume com suporte</v>
+        <v>Não identifico sucessor</v>
       </c>
       <c r="O49" t="str">
-        <v>Bruno Martins, Odimar Antonio de Oliveira</v>
+        <v/>
       </c>
       <c r="P49" t="str">
         <v>Risco / Baixo Desempenho</v>
@@ -8587,7 +8616,7 @@
         <v>Total (qualquer unidade)</v>
       </c>
       <c r="G50" t="str">
-        <v>Gerente geral</v>
+        <v>Gerente administrativo da indústria</v>
       </c>
       <c r="H50" t="str">
         <v>Até 3 anos</v>
@@ -8608,10 +8637,10 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="N50" t="str">
-        <v>Não identifico sucessor</v>
+        <v>Alguém assume com suporte</v>
       </c>
       <c r="O50" t="str">
-        <v/>
+        <v>Rogelio dos Santos Vargas</v>
       </c>
       <c r="P50" t="str">
         <v>Empregado Sólido / Responsável</v>
@@ -8664,10 +8693,10 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="N51" t="str">
-        <v>Alguém assume com suporte</v>
+        <v>Não identifico sucessor</v>
       </c>
       <c r="O51" t="str">
-        <v>Max Antunes Cavalheiro</v>
+        <v/>
       </c>
       <c r="P51" t="str">
         <v>Empregado Comprometido</v>
@@ -8720,10 +8749,10 @@
         <v>Não</v>
       </c>
       <c r="N52" t="str">
-        <v>Não identifico sucessor</v>
+        <v>Alguém assume imediatamente</v>
       </c>
       <c r="O52" t="str">
-        <v/>
+        <v>Beatriz Santos Kroetzler</v>
       </c>
       <c r="P52" t="str">
         <v>Empregado Comprometido</v>
@@ -8776,10 +8805,10 @@
         <v>Não</v>
       </c>
       <c r="N53" t="str">
-        <v>Alguém assume imediatamente</v>
+        <v>Não identifico sucessor</v>
       </c>
       <c r="O53" t="str">
-        <v>Beatriz Santos Kroetzler</v>
+        <v/>
       </c>
       <c r="P53" t="str">
         <v>Enigma / Questionável</v>
@@ -8888,10 +8917,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N55" t="str">
-        <v>Não identifico sucessor</v>
+        <v>Alguém assume imediatamente</v>
       </c>
       <c r="O55" t="str">
-        <v/>
+        <v>Lucas Cardoso Jardim, Elisandra Martines dos Santos</v>
       </c>
       <c r="P55" t="str">
         <v>Empregado Comprometido</v>
@@ -8944,10 +8973,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N56" t="str">
-        <v>Alguém assume imediatamente</v>
+        <v>Alguém assume com suporte</v>
       </c>
       <c r="O56" t="str">
-        <v>Teilo de Jesus Santana, Beatriz Santos Kroetzler</v>
+        <v>Lucas Cardoso Jardim</v>
       </c>
       <c r="P56" t="str">
         <v>Empregado Comprometido</v>
@@ -9000,10 +9029,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N57" t="str">
-        <v>Alguém assume com suporte</v>
+        <v>Sem elementos para avaliar</v>
       </c>
       <c r="O57" t="str">
-        <v>Teilo de Jesus Santana</v>
+        <v/>
       </c>
       <c r="P57" t="str">
         <v>Empregado Sólido / Responsável</v>
@@ -9056,10 +9085,10 @@
         <v>Não</v>
       </c>
       <c r="N58" t="str">
-        <v>Sem elementos para avaliar</v>
+        <v>Alguém assume imediatamente</v>
       </c>
       <c r="O58" t="str">
-        <v/>
+        <v>Beatriz Kroetzler, Rogelio dos Santos Vargas</v>
       </c>
       <c r="P58" t="str">
         <v>Alto Potencial</v>
@@ -9112,10 +9141,10 @@
         <v>Não</v>
       </c>
       <c r="N59" t="str">
-        <v>Alguém assume imediatamente</v>
+        <v>Alguém assume com suporte</v>
       </c>
       <c r="O59" t="str">
-        <v>Beatriz Kroetzler, Max Antunes Cavalheiro</v>
+        <v>Bruno Rodrigues Martins</v>
       </c>
       <c r="P59" t="str">
         <v>Estrela</v>
@@ -9171,7 +9200,7 @@
         <v>Alguém assume com suporte</v>
       </c>
       <c r="O60" t="str">
-        <v>Beatriz Santos Kroetzler</v>
+        <v>Teilo Santana, Lincoln Eduardo Nunes</v>
       </c>
       <c r="P60" t="str">
         <v>Alto Desempenho</v>
@@ -9224,10 +9253,10 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="N61" t="str">
-        <v>Alguém assume com suporte</v>
+        <v>Não identifico sucessor</v>
       </c>
       <c r="O61" t="str">
-        <v>Rogelio Vargas, Neusa Maria Kaiser</v>
+        <v/>
       </c>
       <c r="P61" t="str">
         <v>Estrela</v>
@@ -9280,10 +9309,10 @@
         <v>Não</v>
       </c>
       <c r="N62" t="str">
-        <v>Não identifico sucessor</v>
+        <v>Alguém assume com suporte</v>
       </c>
       <c r="O62" t="str">
-        <v/>
+        <v>Odimar Antonio de Oliveira</v>
       </c>
       <c r="P62" t="str">
         <v>Empregado Comprometido</v>
@@ -9336,10 +9365,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N63" t="str">
-        <v>Alguém assume com suporte</v>
+        <v>Sem elementos para avaliar</v>
       </c>
       <c r="O63" t="str">
-        <v>Raquel Cristina Vidotto Ramos</v>
+        <v/>
       </c>
       <c r="P63" t="str">
         <v>Bom Executor / Especialista</v>
@@ -9392,10 +9421,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N64" t="str">
-        <v>Sem elementos para avaliar</v>
+        <v>Alguém assume com suporte</v>
       </c>
       <c r="O64" t="str">
-        <v/>
+        <v>Mariana Holanda Siqueira</v>
       </c>
       <c r="P64" t="str">
         <v>Empregado Sólido / Responsável</v>
@@ -9504,10 +9533,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N66" t="str">
-        <v>Alguém assume com suporte</v>
+        <v>Sem elementos para avaliar</v>
       </c>
       <c r="O66" t="str">
-        <v>Jordy Alesson Souza Monteiro</v>
+        <v/>
       </c>
       <c r="P66" t="str">
         <v>Alto Desempenho</v>
@@ -9616,10 +9645,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N68" t="str">
-        <v>Sem elementos para avaliar</v>
+        <v>Alguém assume com suporte</v>
       </c>
       <c r="O68" t="str">
-        <v/>
+        <v>Mariana Meireles Esteves, Samuel Santana Barreto</v>
       </c>
       <c r="P68" t="str">
         <v>Enigma / Questionável</v>
@@ -9675,7 +9704,7 @@
         <v>Alguém assume com suporte</v>
       </c>
       <c r="O69" t="str">
-        <v>Murilo Zanella Valadares, Jordy Alesson Souza Monteiro</v>
+        <v>Jordy Alesson Souza Monteiro, Neiva Cristiane Bortolato Goncalves</v>
       </c>
       <c r="P69" t="str">
         <v>Empregado Sólido / Responsável</v>
@@ -9728,10 +9757,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N70" t="str">
-        <v>Alguém assume com suporte</v>
+        <v>Sem elementos para avaliar</v>
       </c>
       <c r="O70" t="str">
-        <v>Bruna Pacheco Valadares, Neiva Cristiane Bortolato Goncalves</v>
+        <v/>
       </c>
       <c r="P70" t="str">
         <v>Estrela</v>
@@ -9784,10 +9813,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N71" t="str">
-        <v>Sem elementos para avaliar</v>
+        <v>Alguém assume imediatamente</v>
       </c>
       <c r="O71" t="str">
-        <v/>
+        <v>Samuel Santana Barreto</v>
       </c>
       <c r="P71" t="str">
         <v>Empregado Comprometido</v>
@@ -9840,10 +9869,10 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="N72" t="str">
-        <v>Alguém assume imediatamente</v>
+        <v>Alguém assume com suporte</v>
       </c>
       <c r="O72" t="str">
-        <v>Jordy Alesson Souza Monteiro</v>
+        <v>Bruno Rodrigues Martins</v>
       </c>
       <c r="P72" t="str">
         <v>Risco / Baixo Desempenho</v>
@@ -9896,10 +9925,10 @@
         <v>Não</v>
       </c>
       <c r="N73" t="str">
-        <v>Alguém assume com suporte</v>
+        <v>Alguém assume imediatamente</v>
       </c>
       <c r="O73" t="str">
-        <v>Bruno Rodrigues Martins</v>
+        <v>Robson Rodrigues Jacinto</v>
       </c>
       <c r="P73" t="str">
         <v/>
@@ -9955,7 +9984,7 @@
         <v>Alguém assume imediatamente</v>
       </c>
       <c r="O74" t="str">
-        <v>Robson Rodrigues Jacinto</v>
+        <v>Jordy Alesson Souza Monteiro, Mariana Meireles Esteves</v>
       </c>
       <c r="P74" t="str">
         <v>Risco / Baixo Desempenho</v>
@@ -10008,10 +10037,10 @@
         <v>Não</v>
       </c>
       <c r="N75" t="str">
-        <v>Alguém assume imediatamente</v>
+        <v>Alguém assume com suporte</v>
       </c>
       <c r="O75" t="str">
-        <v>Bruna Pacheco Valadares, Murilo Zanella Valadares</v>
+        <v>Marileide Porto Fontana</v>
       </c>
       <c r="P75" t="str">
         <v>Empregado Sólido / Responsável</v>
@@ -10064,10 +10093,10 @@
         <v>Não</v>
       </c>
       <c r="N76" t="str">
-        <v>Alguém assume com suporte</v>
+        <v>Sem elementos para avaliar</v>
       </c>
       <c r="O76" t="str">
-        <v>Neiva Cristiane Bortolato Goncalves</v>
+        <v/>
       </c>
       <c r="P76" t="str">
         <v>Bom Executor / Especialista</v>
@@ -10120,7 +10149,7 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="N77" t="str">
-        <v>Sem elementos para avaliar</v>
+        <v>Não identifico sucessor</v>
       </c>
       <c r="O77" t="str">
         <v/>
@@ -10176,10 +10205,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N78" t="str">
-        <v>Não identifico sucessor</v>
+        <v>Alguém assume com suporte</v>
       </c>
       <c r="O78" t="str">
-        <v/>
+        <v>Beatriz Kroetzler, Bruno Rodrigues Martins</v>
       </c>
       <c r="P78" t="str">
         <v>Empregado Comprometido</v>
@@ -10232,10 +10261,10 @@
         <v>Não</v>
       </c>
       <c r="N79" t="str">
-        <v>Alguém assume com suporte</v>
+        <v>Não identifico sucessor</v>
       </c>
       <c r="O79" t="str">
-        <v>Beatriz Kroetzler, Bruno Rodrigues Martins</v>
+        <v/>
       </c>
       <c r="P79" t="str">
         <v>Alto Potencial</v>
@@ -10344,10 +10373,10 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="N81" t="str">
-        <v>Não identifico sucessor</v>
+        <v>Alguém assume imediatamente</v>
       </c>
       <c r="O81" t="str">
-        <v/>
+        <v>Heitor Jardim Valadares</v>
       </c>
       <c r="P81" t="str">
         <v>Empregado Comprometido</v>
@@ -10400,10 +10429,10 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="N82" t="str">
-        <v>Alguém assume com suporte</v>
+        <v>Alguém assume imediatamente</v>
       </c>
       <c r="O82" t="str">
-        <v>Neiva Cristiane Bortolato Goncalves, Edwagner Oliveira</v>
+        <v>Edwagner Oliveira</v>
       </c>
       <c r="P82" t="str">
         <v>Alto Desempenho</v>
@@ -10456,7 +10485,7 @@
         <v>Não</v>
       </c>
       <c r="N83" t="str">
-        <v>Alguém assume com suporte</v>
+        <v>Alguém assume imediatamente</v>
       </c>
       <c r="O83" t="str">
         <v>Samuel Santana Barreto</v>
@@ -10512,10 +10541,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N84" t="str">
-        <v>Não identifico sucessor</v>
+        <v>Alguém assume com suporte</v>
       </c>
       <c r="O84" t="str">
-        <v/>
+        <v>Samuel Santana Barreto</v>
       </c>
       <c r="P84" t="str">
         <v>Alto Potencial</v>
@@ -10568,10 +10597,10 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="N85" t="str">
-        <v>Alguém assume com suporte</v>
+        <v>Não identifico sucessor</v>
       </c>
       <c r="O85" t="str">
-        <v>Murilo Zanella Albuquerque</v>
+        <v/>
       </c>
       <c r="P85" t="str">
         <v>Empregado Comprometido</v>
@@ -10624,7 +10653,7 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N86" t="str">
-        <v>Não identifico sucessor</v>
+        <v>Sem elementos para avaliar</v>
       </c>
       <c r="O86" t="str">
         <v/>
@@ -10792,7 +10821,7 @@
         <v>Não</v>
       </c>
       <c r="N89" t="str">
-        <v>Não identifico sucessor</v>
+        <v>Sem elementos para avaliar</v>
       </c>
       <c r="O89" t="str">
         <v/>
@@ -10848,10 +10877,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N90" t="str">
-        <v>Não identifico sucessor</v>
+        <v>Alguém assume imediatamente</v>
       </c>
       <c r="O90" t="str">
-        <v/>
+        <v>Ana Paula Franco Prodoscimo Sarti</v>
       </c>
       <c r="P90" t="str">
         <v>Alto Potencial</v>
@@ -10883,7 +10912,7 @@
         <v>Total (qualquer unidade)</v>
       </c>
       <c r="G91" t="str">
-        <v>Gerente de assistência</v>
+        <v>Gerente de banco de dados</v>
       </c>
       <c r="H91" t="str">
         <v>Mais de 3 até 5 anos</v>
@@ -10907,7 +10936,7 @@
         <v>Alguém assume com suporte</v>
       </c>
       <c r="O91" t="str">
-        <v>Rodrigo da Veiga Lima, Thiago Carvalho Ferreira</v>
+        <v>Ana Paula Franco Prodoscimo Sarti</v>
       </c>
       <c r="P91" t="str">
         <v>Alto Desempenho</v>
@@ -10960,7 +10989,7 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N92" t="str">
-        <v>Sem elementos para avaliar</v>
+        <v>Não identifico sucessor</v>
       </c>
       <c r="O92" t="str">
         <v/>
@@ -11016,10 +11045,10 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="N93" t="str">
-        <v>Sem elementos para avaliar</v>
+        <v>Alguém assume imediatamente</v>
       </c>
       <c r="O93" t="str">
-        <v/>
+        <v>Willian Fernando Cruz Alves, Heitor Henrique Bataiero</v>
       </c>
       <c r="P93" t="str">
         <v>Alto Desempenho</v>
@@ -11072,10 +11101,10 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="N94" t="str">
-        <v>Alguém assume imediatamente</v>
+        <v>Alguém assume com suporte</v>
       </c>
       <c r="O94" t="str">
-        <v>Vitor Guimarães Valadares, Otávio Rezende Jardim</v>
+        <v>Paula Albuquerque Meireles</v>
       </c>
       <c r="P94" t="str">
         <v>Alto Desempenho</v>
@@ -11128,10 +11157,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N95" t="str">
-        <v>Alguém assume com suporte</v>
+        <v>Sem elementos para avaliar</v>
       </c>
       <c r="O95" t="str">
-        <v>Gabriela Valadares Siqueira</v>
+        <v/>
       </c>
       <c r="P95" t="str">
         <v>Estrela</v>
@@ -11184,10 +11213,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N96" t="str">
-        <v>Sem elementos para avaliar</v>
+        <v>Alguém assume com suporte</v>
       </c>
       <c r="O96" t="str">
-        <v/>
+        <v>Vitor Guimarães Valadares, Paula Cardoso Barreto</v>
       </c>
       <c r="P96" t="str">
         <v>Empregado Comprometido</v>
@@ -11240,10 +11269,10 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="N97" t="str">
-        <v>Alguém assume com suporte</v>
+        <v>Alguém assume imediatamente</v>
       </c>
       <c r="O97" t="str">
-        <v>Vitor Guimarães Valadares, Samuel Figueiredo Pacheco</v>
+        <v>Paula Barreto</v>
       </c>
       <c r="P97" t="str">
         <v>Empregado Sólido / Responsável</v>
@@ -11299,7 +11328,7 @@
         <v>Alguém assume imediatamente</v>
       </c>
       <c r="O98" t="str">
-        <v>Rafaela Esteves</v>
+        <v>Paula Cardoso Barreto, Paula Albuquerque Meireles</v>
       </c>
       <c r="P98" t="str">
         <v>Estrela</v>
@@ -11352,10 +11381,10 @@
         <v>Não</v>
       </c>
       <c r="N99" t="str">
-        <v>Alguém assume imediatamente</v>
+        <v>Não identifico sucessor</v>
       </c>
       <c r="O99" t="str">
-        <v>Rafaela Guimarães Esteves, Otávio Rezende Jardim</v>
+        <v/>
       </c>
       <c r="P99" t="str">
         <v>Empregado Sólido / Responsável</v>
@@ -11579,7 +11608,7 @@
         <v>Alguém assume com suporte</v>
       </c>
       <c r="O103" t="str">
-        <v>Mauricio Souza</v>
+        <v>Rodrigo de Oliveira Novo</v>
       </c>
       <c r="P103" t="str">
         <v>Alto Potencial</v>
@@ -11632,10 +11661,10 @@
         <v>Não</v>
       </c>
       <c r="N104" t="str">
-        <v>Não identifico sucessor</v>
+        <v>Alguém assume com suporte</v>
       </c>
       <c r="O104" t="str">
-        <v/>
+        <v>Danilo Moureira Niza da Silva, Fabielly Garcia de Souza Costa</v>
       </c>
       <c r="P104" t="str">
         <v>Estrela</v>
@@ -11688,10 +11717,10 @@
         <v>Não</v>
       </c>
       <c r="N105" t="str">
-        <v>Sem elementos para avaliar</v>
+        <v>Alguém assume imediatamente</v>
       </c>
       <c r="O105" t="str">
-        <v/>
+        <v>Luiz Paulo da Silva Santos</v>
       </c>
       <c r="P105" t="str">
         <v>Empregado Comprometido</v>
@@ -11744,10 +11773,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N106" t="str">
-        <v>Alguém assume imediatamente</v>
+        <v>Não identifico sucessor</v>
       </c>
       <c r="O106" t="str">
-        <v>Rogelio dos Santos Vargas</v>
+        <v/>
       </c>
       <c r="P106" t="str">
         <v>Empregado Comprometido</v>
@@ -11800,10 +11829,10 @@
         <v>Não</v>
       </c>
       <c r="N107" t="str">
-        <v>Não identifico sucessor</v>
+        <v>Alguém assume imediatamente</v>
       </c>
       <c r="O107" t="str">
-        <v/>
+        <v>Fabielly Garcia de Souza Costa, Danilo Moureira Niza da Silva</v>
       </c>
       <c r="P107" t="str">
         <v>Empregado Sólido / Responsável</v>
@@ -11856,10 +11885,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N108" t="str">
-        <v>Alguém assume imediatamente</v>
+        <v>Não identifico sucessor</v>
       </c>
       <c r="O108" t="str">
-        <v>Edson Guedes de Sousa, Milene Thomaz Romano Gantzel</v>
+        <v/>
       </c>
       <c r="P108" t="str">
         <v>Enigma / Questionável</v>
@@ -11968,10 +11997,10 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="N110" t="str">
-        <v>Alguém assume com suporte</v>
+        <v>Não identifico sucessor</v>
       </c>
       <c r="O110" t="str">
-        <v>Raimundo Nonato Silva Amaral</v>
+        <v/>
       </c>
       <c r="P110" t="str">
         <v>Bom Executor / Especialista</v>
@@ -12027,7 +12056,7 @@
         <v>Alguém assume imediatamente</v>
       </c>
       <c r="O111" t="str">
-        <v>Rogelio Vargas, Fernando da Silva Dias</v>
+        <v>Willian Fernando Cruz Alves, Fabielly Garcia de Souza Costa</v>
       </c>
       <c r="P111" t="str">
         <v>Alto Desempenho</v>
@@ -12080,10 +12109,10 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="N112" t="str">
-        <v>Alguém assume imediatamente</v>
+        <v>Não identifico sucessor</v>
       </c>
       <c r="O112" t="str">
-        <v>Fabielly Garcia de Souza Costa</v>
+        <v/>
       </c>
       <c r="P112" t="str">
         <v>Alto Potencial</v>
@@ -12227,7 +12256,7 @@
         <v>Dentro do Estado</v>
       </c>
       <c r="G115" t="str">
-        <v>Gerente de indústria</v>
+        <v>Gerente de atendimento ao cliente</v>
       </c>
       <c r="H115" t="str">
         <v>Imediato</v>
@@ -12236,7 +12265,7 @@
         <v>Conhecimento da operação de outras unidades</v>
       </c>
       <c r="J115" t="str">
-        <v>Gerente geral agropecuária</v>
+        <v>Gerente geral de recursos humanos</v>
       </c>
       <c r="K115" t="str">
         <v>Até 3 anos</v>
@@ -12416,10 +12445,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N118" t="str">
-        <v>Alguém assume com suporte</v>
+        <v>Alguém assume imediatamente</v>
       </c>
       <c r="O118" t="str">
-        <v>Raquel Cristina Vidotto Ramos</v>
+        <v>Raquel Cristina Vidotto Ramos, Yasmin Valadares</v>
       </c>
       <c r="P118" t="str">
         <v>Estrela</v>
@@ -12472,10 +12501,10 @@
         <v>Não</v>
       </c>
       <c r="N119" t="str">
-        <v>Não identifico sucessor</v>
+        <v>Alguém assume com suporte</v>
       </c>
       <c r="O119" t="str">
-        <v/>
+        <v>Raquel Ramos</v>
       </c>
       <c r="P119" t="str">
         <v>Enigma / Questionável</v>
@@ -12584,7 +12613,7 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N121" t="str">
-        <v>Não identifico sucessor</v>
+        <v>Sem elementos para avaliar</v>
       </c>
       <c r="O121" t="str">
         <v/>
@@ -12640,10 +12669,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N122" t="str">
-        <v>Alguém assume com suporte</v>
+        <v>Não identifico sucessor</v>
       </c>
       <c r="O122" t="str">
-        <v>Caio Jardim</v>
+        <v/>
       </c>
       <c r="P122" t="str">
         <v>Alto Desempenho</v>
@@ -12696,10 +12725,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N123" t="str">
-        <v>Não identifico sucessor</v>
+        <v>Alguém assume imediatamente</v>
       </c>
       <c r="O123" t="str">
-        <v/>
+        <v>Cadmiel Cristiano de Grande</v>
       </c>
       <c r="P123" t="str">
         <v>Alto Desempenho</v>
@@ -12752,10 +12781,10 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="N124" t="str">
-        <v>Alguém assume imediatamente</v>
+        <v>Alguém assume com suporte</v>
       </c>
       <c r="O124" t="str">
-        <v>Letícia Tavares Xavier</v>
+        <v>Gabriela Valadares Siqueira, Bruna Cardoso Damasceno</v>
       </c>
       <c r="P124" t="str">
         <v>Estrela</v>
@@ -12808,10 +12837,10 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="N125" t="str">
-        <v>Alguém assume com suporte</v>
+        <v>Alguém assume imediatamente</v>
       </c>
       <c r="O125" t="str">
-        <v>Letícia Tavares Xavier, Paulo da Silva Braz</v>
+        <v>Gabriela Valadares Siqueira, Bruna Cardoso Damasceno</v>
       </c>
       <c r="P125" t="str">
         <v>Estrela</v>
@@ -12867,7 +12896,7 @@
         <v>Alguém assume imediatamente</v>
       </c>
       <c r="O126" t="str">
-        <v>Fabner Roberto Soares, Edson Macoto Tamura Junior</v>
+        <v>Edson Junior</v>
       </c>
       <c r="P126" t="str">
         <v>Empregado Comprometido</v>
@@ -12979,7 +13008,7 @@
         <v>Alguém assume imediatamente</v>
       </c>
       <c r="O128" t="str">
-        <v>Anderson Rodrigo Giomo</v>
+        <v>Yuri Ignochevski Primao</v>
       </c>
       <c r="P128" t="str">
         <v>Estrela</v>
@@ -13011,7 +13040,7 @@
         <v>Matriz (Douradina/PR)</v>
       </c>
       <c r="G129" t="str">
-        <v>Gerente de indústria</v>
+        <v>Gerente de atendimento ao cliente</v>
       </c>
       <c r="H129" t="str">
         <v>Mais de 3 até 5 anos</v>
@@ -13032,10 +13061,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N129" t="str">
-        <v>Alguém assume imediatamente</v>
+        <v>Não identifico sucessor</v>
       </c>
       <c r="O129" t="str">
-        <v>Anderson Rodrigo Giomo</v>
+        <v/>
       </c>
       <c r="P129" t="str">
         <v>Alto Potencial</v>
@@ -13076,7 +13105,7 @@
         <v>Visão financeira do negócio (DRE, orçamento)</v>
       </c>
       <c r="J130" t="str">
-        <v>Gerente administrativo da indústria</v>
+        <v>Gerente de atendimento ao cliente</v>
       </c>
       <c r="K130" t="str">
         <v>Até 3 anos</v>
@@ -13088,10 +13117,10 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="N130" t="str">
-        <v>Não identifico sucessor</v>
+        <v>Alguém assume com suporte</v>
       </c>
       <c r="O130" t="str">
-        <v/>
+        <v>Anderson Rodrigo Giomo</v>
       </c>
       <c r="P130" t="str">
         <v>Empregado Comprometido</v>
@@ -13144,10 +13173,10 @@
         <v>Não</v>
       </c>
       <c r="N131" t="str">
-        <v>Alguém assume com suporte</v>
+        <v>Não identifico sucessor</v>
       </c>
       <c r="O131" t="str">
-        <v>Danilo Moureira Niza da Silva</v>
+        <v/>
       </c>
       <c r="P131" t="str">
         <v>Empregado Sólido / Responsável</v>
@@ -13200,7 +13229,7 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N132" t="str">
-        <v>Não identifico sucessor</v>
+        <v>Sem elementos para avaliar</v>
       </c>
       <c r="O132" t="str">
         <v/>
@@ -13256,7 +13285,7 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N133" t="str">
-        <v>Sem elementos para avaliar</v>
+        <v>Não identifico sucessor</v>
       </c>
       <c r="O133" t="str">
         <v/>
@@ -13368,10 +13397,10 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="N135" t="str">
-        <v>Não identifico sucessor</v>
+        <v>Alguém assume com suporte</v>
       </c>
       <c r="O135" t="str">
-        <v/>
+        <v>Mariana Holanda Siqueira</v>
       </c>
       <c r="P135" t="str">
         <v>Bom Executor / Especialista</v>
@@ -13424,7 +13453,7 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="N136" t="str">
-        <v>Alguém assume com suporte</v>
+        <v>Sem elementos para avaliar</v>
       </c>
       <c r="O136" t="str">
         <v>Cleiton Silva, Maykon Fernando da Costa</v>
@@ -13480,7 +13509,7 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N137" t="str">
-        <v>Sem elementos para avaliar</v>
+        <v>Não identifico sucessor</v>
       </c>
       <c r="O137" t="str">
         <v/>
@@ -13515,7 +13544,7 @@
         <v>Local atual</v>
       </c>
       <c r="G138" t="str">
-        <v>Gerente comercial do varejo</v>
+        <v>Gerente de compras</v>
       </c>
       <c r="H138" t="str">
         <v>Imediato</v>
@@ -13571,7 +13600,7 @@
         <v>Local atual</v>
       </c>
       <c r="G139" t="str">
-        <v>Gerente de atendimento ao cliente</v>
+        <v>Gerente de auditoria</v>
       </c>
       <c r="H139" t="str">
         <v>Mais de 3 até 5 anos</v>
@@ -13592,10 +13621,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N139" t="str">
-        <v>Sem elementos para avaliar</v>
+        <v>Alguém assume com suporte</v>
       </c>
       <c r="O139" t="str">
-        <v/>
+        <v>Maria Eduarda Matos Medeiros, Fernando da Silva Dias</v>
       </c>
       <c r="P139" t="str">
         <v>Risco / Baixo Desempenho</v>
@@ -13648,10 +13677,10 @@
         <v>Não</v>
       </c>
       <c r="N140" t="str">
-        <v>Alguém assume imediatamente</v>
+        <v>Não identifico sucessor</v>
       </c>
       <c r="O140" t="str">
-        <v>Rodrigo Lima</v>
+        <v/>
       </c>
       <c r="P140" t="str">
         <v>Alto Desempenho</v>
@@ -13704,10 +13733,10 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="N141" t="str">
-        <v>Alguém assume imediatamente</v>
+        <v>Sem elementos para avaliar</v>
       </c>
       <c r="O141" t="str">
-        <v>Daniela Xavier</v>
+        <v/>
       </c>
       <c r="P141" t="str">
         <v>Estrela</v>
@@ -13760,10 +13789,10 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="N142" t="str">
-        <v>Sem elementos para avaliar</v>
+        <v>Alguém assume imediatamente</v>
       </c>
       <c r="O142" t="str">
-        <v/>
+        <v>Natan Goncalves</v>
       </c>
       <c r="P142" t="str">
         <v>Estrela</v>
@@ -13816,10 +13845,10 @@
         <v>Não</v>
       </c>
       <c r="N143" t="str">
-        <v>Alguém assume imediatamente</v>
+        <v>Não identifico sucessor</v>
       </c>
       <c r="O143" t="str">
-        <v>Natiara Vieira</v>
+        <v/>
       </c>
       <c r="P143" t="str">
         <v>Empregado Comprometido</v>
@@ -13872,10 +13901,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N144" t="str">
-        <v>Não identifico sucessor</v>
+        <v>Alguém assume com suporte</v>
       </c>
       <c r="O144" t="str">
-        <v/>
+        <v>Priscila Andrelina da Silva Bartolomeu</v>
       </c>
       <c r="P144" t="str">
         <v>Alto Potencial</v>
@@ -13928,10 +13957,10 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="N145" t="str">
-        <v>Alguém assume com suporte</v>
+        <v>Alguém assume imediatamente</v>
       </c>
       <c r="O145" t="str">
-        <v>Priscila Andrelina da Silva Bartolomeu</v>
+        <v>Natiara Rodrigues dos Santos Vieira, Amanda Holanda</v>
       </c>
       <c r="P145" t="str">
         <v>Empregado Sólido / Responsável</v>
@@ -13984,10 +14013,10 @@
         <v>Não</v>
       </c>
       <c r="N146" t="str">
-        <v>Alguém assume imediatamente</v>
+        <v>Alguém assume com suporte</v>
       </c>
       <c r="O146" t="str">
-        <v>Priscila Andrelina da Silva Bartolomeu, Eduarda Jardim</v>
+        <v>João Queiroz, Lucas Barreto Holanda</v>
       </c>
       <c r="P146" t="str">
         <v>Enigma / Questionável</v>
@@ -14040,10 +14069,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N147" t="str">
-        <v>Alguém assume com suporte</v>
+        <v>Não identifico sucessor</v>
       </c>
       <c r="O147" t="str">
-        <v>Eduarda Jardim, Natiara Rodrigues dos Santos Vieira</v>
+        <v/>
       </c>
       <c r="P147" t="str">
         <v>Alto Desempenho</v>
@@ -14096,10 +14125,10 @@
         <v>Não</v>
       </c>
       <c r="N148" t="str">
-        <v>Não identifico sucessor</v>
+        <v>Alguém assume com suporte</v>
       </c>
       <c r="O148" t="str">
-        <v/>
+        <v>João Queiroz</v>
       </c>
       <c r="P148" t="str">
         <v>Empregado Comprometido</v>
@@ -14155,7 +14184,7 @@
         <v>Alguém assume com suporte</v>
       </c>
       <c r="O149" t="str">
-        <v>Bruna Valadares</v>
+        <v>Daniela Rezende Nogueira, Jordy Alesson Souza Monteiro</v>
       </c>
       <c r="P149" t="str">
         <v>Enigma / Questionável</v>
@@ -14196,7 +14225,7 @@
         <v>Comunicação com a diretoria</v>
       </c>
       <c r="J150" t="str">
-        <v>Gerente de atendimento ao cliente</v>
+        <v>Gerente de auditoria</v>
       </c>
       <c r="K150" t="str">
         <v>Até 3 anos</v>
@@ -14208,10 +14237,10 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="N150" t="str">
-        <v>Alguém assume com suporte</v>
+        <v>Alguém assume imediatamente</v>
       </c>
       <c r="O150" t="str">
-        <v>Daniela Rezende Nogueira, Jordy Alesson Souza Monteiro</v>
+        <v>Jordy Monteiro</v>
       </c>
       <c r="P150" t="str">
         <v>Estrela</v>
@@ -14267,7 +14296,7 @@
         <v>Alguém assume imediatamente</v>
       </c>
       <c r="O151" t="str">
-        <v>Jordy Monteiro</v>
+        <v>Daniela Rezende Nogueira</v>
       </c>
       <c r="P151" t="str">
         <v>Bom Executor / Especialista</v>
@@ -14320,10 +14349,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N152" t="str">
-        <v>Alguém assume imediatamente</v>
+        <v>Não identifico sucessor</v>
       </c>
       <c r="O152" t="str">
-        <v>Daniela Rezende Nogueira</v>
+        <v/>
       </c>
       <c r="P152" t="str">
         <v>Empregado Comprometido</v>
@@ -14376,7 +14405,7 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="N153" t="str">
-        <v>Sem elementos para avaliar</v>
+        <v>Não identifico sucessor</v>
       </c>
       <c r="O153" t="str">
         <v/>
@@ -14432,10 +14461,10 @@
         <v>Não</v>
       </c>
       <c r="N154" t="str">
-        <v>Alguém assume imediatamente</v>
+        <v>Alguém assume com suporte</v>
       </c>
       <c r="O154" t="str">
-        <v>Juliana Calvo</v>
+        <v>Arinan Moreira dos Santos</v>
       </c>
       <c r="P154" t="str">
         <v>Alto Desempenho</v>
@@ -14488,7 +14517,7 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="N155" t="str">
-        <v>Sem elementos para avaliar</v>
+        <v>Não identifico sucessor</v>
       </c>
       <c r="O155" t="str">
         <v/>
@@ -14547,7 +14576,7 @@
         <v>Alguém assume com suporte</v>
       </c>
       <c r="O156" t="str">
-        <v>Antonio Mendonca</v>
+        <v>Fabricio Silva Facco</v>
       </c>
       <c r="P156" t="str">
         <v>Empregado Sólido / Responsável</v>
@@ -14603,7 +14632,7 @@
         <v>Alguém assume imediatamente</v>
       </c>
       <c r="O157" t="str">
-        <v>Fabricio Facco, Antonio Raimundo Santos de Mendonca</v>
+        <v>Fabricio Facco</v>
       </c>
       <c r="P157" t="str">
         <v>Alto Potencial</v>
@@ -14659,7 +14688,7 @@
         <v>Alguém assume com suporte</v>
       </c>
       <c r="O158" t="str">
-        <v>Fabricio Silva Facco</v>
+        <v>Antonio Mendonca</v>
       </c>
       <c r="P158" t="str">
         <v>Enigma / Questionável</v>
@@ -14712,10 +14741,10 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="N159" t="str">
-        <v>Alguém assume com suporte</v>
+        <v>Não identifico sucessor</v>
       </c>
       <c r="O159" t="str">
-        <v>Fabricio Silva Facco, Antonio Raimundo Santos de Mendonca</v>
+        <v/>
       </c>
       <c r="P159" t="str">
         <v>Bom Executor / Especialista</v>
@@ -14771,7 +14800,7 @@
         <v>Alguém assume com suporte</v>
       </c>
       <c r="O160" t="str">
-        <v>Antonio Mendonca</v>
+        <v>Fabricio Silva Facco</v>
       </c>
       <c r="P160" t="str">
         <v>Empregado Sólido / Responsável</v>
@@ -14812,7 +14841,7 @@
         <v>Comunicação com a diretoria</v>
       </c>
       <c r="J161" t="str">
-        <v>Gerente geral</v>
+        <v>Gerente administrativo da indústria</v>
       </c>
       <c r="K161" t="str">
         <v>Até 3 anos</v>
@@ -14824,10 +14853,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N161" t="str">
-        <v>Alguém assume com suporte</v>
+        <v>Não identifico sucessor</v>
       </c>
       <c r="O161" t="str">
-        <v>Fabricio Facco</v>
+        <v/>
       </c>
       <c r="P161" t="str">
         <v>Alto Desempenho</v>
@@ -14859,7 +14888,7 @@
         <v>Total (qualquer unidade)</v>
       </c>
       <c r="G162" t="str">
-        <v>Gerente de assistência</v>
+        <v>Gerente de banco de dados</v>
       </c>
       <c r="H162" t="str">
         <v>Mais de 5 anos</v>
@@ -14880,10 +14909,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N162" t="str">
-        <v>Não identifico sucessor</v>
+        <v>Alguém assume com suporte</v>
       </c>
       <c r="O162" t="str">
-        <v/>
+        <v>Antonio Raimundo Santos de Mendonca</v>
       </c>
       <c r="P162" t="str">
         <v>Empregado Sólido / Responsável</v>
@@ -14939,7 +14968,7 @@
         <v>Alguém assume com suporte</v>
       </c>
       <c r="O163" t="str">
-        <v>Rogerio Tsuyoshi Arida</v>
+        <v>Francisca Marisangela de Jesus Sousa</v>
       </c>
       <c r="P163" t="str">
         <v/>
@@ -14992,10 +15021,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N164" t="str">
-        <v>Alguém assume com suporte</v>
+        <v>Alguém assume imediatamente</v>
       </c>
       <c r="O164" t="str">
-        <v>Luiz Trench, Jonismar Antonio dos Santos</v>
+        <v>Alexsandro Bataieiro, Celia Xavier Novo</v>
       </c>
       <c r="P164" t="str">
         <v>Empregado Comprometido</v>
@@ -15104,10 +15133,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N166" t="str">
-        <v>Não identifico sucessor</v>
+        <v>Alguém assume com suporte</v>
       </c>
       <c r="O166" t="str">
-        <v/>
+        <v>Rodrigo Romano Gantzel</v>
       </c>
       <c r="P166" t="str">
         <v/>
@@ -15160,10 +15189,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N167" t="str">
-        <v>Sem elementos para avaliar</v>
+        <v>Alguém assume com suporte</v>
       </c>
       <c r="O167" t="str">
-        <v/>
+        <v>Alexsandro Bataieiro</v>
       </c>
       <c r="P167" t="str">
         <v>Empregado Sólido / Responsável</v>
@@ -15275,7 +15304,7 @@
         <v>Alguém assume com suporte</v>
       </c>
       <c r="O169" t="str">
-        <v>Eduardo Giacometti Xavier, Yuri Ignochevski Primao</v>
+        <v>Iago Fernando Luiz, Marcus Vinicius Cabeça Pereira</v>
       </c>
       <c r="P169" t="str">
         <v>Empregado Comprometido</v>
@@ -15611,7 +15640,7 @@
         <v>Alguém assume com suporte</v>
       </c>
       <c r="O175" t="str">
-        <v>Rosana Queiroz da Silva</v>
+        <v>Fernando da Silva Dias</v>
       </c>
       <c r="P175" t="str">
         <v>Empregado Comprometido</v>
@@ -15776,7 +15805,7 @@
         <v>Conversado, sem plano formal</v>
       </c>
       <c r="N178" t="str">
-        <v>Não identifico sucessor</v>
+        <v>Sem elementos para avaliar</v>
       </c>
       <c r="O178" t="str">
         <v/>
@@ -15832,10 +15861,10 @@
         <v>Sim, em andamento</v>
       </c>
       <c r="N179" t="str">
-        <v>Não identifico sucessor</v>
+        <v>Alguém assume imediatamente</v>
       </c>
       <c r="O179" t="str">
-        <v/>
+        <v>Aline Santos</v>
       </c>
       <c r="P179" t="str">
         <v>Alto Desempenho</v>
@@ -15849,45 +15878,63 @@
     </row>
     <row r="180">
       <c r="A180" t="str">
-        <v>Paula Albuquerque Meireles</v>
+        <v>Alessandra Guerra de Souza</v>
       </c>
       <c r="B180" t="str">
-        <v>Analista / Técnico</v>
+        <v>Gerência Executiva</v>
       </c>
       <c r="C180" t="str">
-        <v>Analista de compras</v>
+        <v>Gerente geral de recursos humanos</v>
       </c>
       <c r="D180" t="str">
-        <v>Diretoria administrativa</v>
+        <v>Gerente geral de recursos humanos</v>
       </c>
       <c r="E180" t="str">
-        <v>Cuiabá/MT</v>
+        <v>Douradina/PR</v>
       </c>
       <c r="F180" t="str">
         <v>Dentro do Estado</v>
       </c>
       <c r="G180" t="str">
-        <v>Coordenador de comunicação</v>
+        <v/>
       </c>
       <c r="H180" t="str">
-        <v>Imediato</v>
+        <v/>
       </c>
       <c r="I180" t="str">
-        <v>Conhecimento da operação de outras unidades</v>
+        <v/>
+      </c>
+      <c r="J180" t="str">
+        <v/>
+      </c>
+      <c r="K180" t="str">
+        <v/>
+      </c>
+      <c r="L180" t="str">
+        <v/>
       </c>
       <c r="M180" t="str">
-        <v>Sim, em andamento</v>
+        <v>Conversado, sem plano formal</v>
+      </c>
+      <c r="N180" t="str">
+        <v>Sem elementos para avaliar</v>
+      </c>
+      <c r="O180" t="str">
+        <v/>
       </c>
       <c r="P180" t="str">
         <v>Enigma / Questionável</v>
       </c>
       <c r="Q180" t="str">
-        <v>Não</v>
+        <v>Sim</v>
+      </c>
+      <c r="R180">
+        <v>63</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="str">
-        <v>Otávio Rezende Jardim</v>
+        <v>Paula Albuquerque Meireles</v>
       </c>
       <c r="B181" t="str">
         <v>Analista / Técnico</v>
@@ -15899,7 +15946,7 @@
         <v>Diretoria administrativa</v>
       </c>
       <c r="E181" t="str">
-        <v>Douradina/PR</v>
+        <v>Cuiabá/MT</v>
       </c>
       <c r="F181" t="str">
         <v>Local atual</v>
@@ -15925,16 +15972,16 @@
     </row>
     <row r="182">
       <c r="A182" t="str">
-        <v>Lucas Cardoso Jardim</v>
+        <v>Otávio Rezende Jardim</v>
       </c>
       <c r="B182" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C182" t="str">
-        <v>Analista de crédito</v>
+        <v>Analista de compras</v>
       </c>
       <c r="D182" t="str">
-        <v>Diretoria financeira</v>
+        <v>Diretoria administrativa</v>
       </c>
       <c r="E182" t="str">
         <v>Douradina/PR</v>
@@ -15954,16 +16001,16 @@
     </row>
     <row r="183">
       <c r="A183" t="str">
-        <v>Lucas Barreto Holanda</v>
+        <v>Lucas Cardoso Jardim</v>
       </c>
       <c r="B183" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C183" t="str">
-        <v>Técnico de segurança do trabalho</v>
+        <v>Analista de crédito</v>
       </c>
       <c r="D183" t="str">
-        <v>Diretoria de governança</v>
+        <v>Diretoria financeira</v>
       </c>
       <c r="E183" t="str">
         <v>Douradina/PR</v>
@@ -15972,7 +16019,7 @@
         <v>Local atual</v>
       </c>
       <c r="G183" t="str">
-        <v>Gerente geral do varejo</v>
+        <v>Gerente regional</v>
       </c>
       <c r="H183" t="str">
         <v>Imediato</v>
@@ -15992,25 +16039,25 @@
     </row>
     <row r="184">
       <c r="A184" t="str">
-        <v>Eduarda Albuquerque Jardim</v>
+        <v>Lucas Barreto Holanda</v>
       </c>
       <c r="B184" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C184" t="str">
-        <v>Analista de logística</v>
+        <v>Técnico de segurança do trabalho</v>
       </c>
       <c r="D184" t="str">
-        <v>Diretoria de logística</v>
+        <v>Diretoria de governança</v>
       </c>
       <c r="E184" t="str">
-        <v>Cuiabá/MT</v>
+        <v>Douradina/PR</v>
       </c>
       <c r="F184" t="str">
         <v>Local atual</v>
       </c>
       <c r="G184" t="str">
-        <v>Coordenador de estoque</v>
+        <v>Coordenador central de compras</v>
       </c>
       <c r="H184" t="str">
         <v>Imediato</v>
@@ -16039,25 +16086,25 @@
     </row>
     <row r="185">
       <c r="A185" t="str">
-        <v>Eduarda Queiroz Meireles</v>
+        <v>Eduarda Albuquerque Jardim</v>
       </c>
       <c r="B185" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C185" t="str">
-        <v>Técnico de segurança do trabalho</v>
+        <v>Analista de logística</v>
       </c>
       <c r="D185" t="str">
-        <v>Diretoria de governança</v>
+        <v>Diretoria de logística</v>
       </c>
       <c r="E185" t="str">
-        <v>Douradina/PR</v>
+        <v>Cuiabá/MT</v>
       </c>
       <c r="F185" t="str">
         <v>Dentro do Estado</v>
       </c>
       <c r="G185" t="str">
-        <v>Coordenador comercial</v>
+        <v>Supervisor administrativo</v>
       </c>
       <c r="H185" t="str">
         <v>Até 3 anos</v>
@@ -16066,7 +16113,7 @@
         <v>Planejamento estratégico</v>
       </c>
       <c r="J185" t="str">
-        <v>Coordenador administrativo (governança)</v>
+        <v>Coordenador de transporte</v>
       </c>
       <c r="K185" t="str">
         <v>Até 3 anos</v>
@@ -16086,16 +16133,16 @@
     </row>
     <row r="186">
       <c r="A186" t="str">
-        <v>Samuel Lacerda Siqueira</v>
+        <v>Eduarda Queiroz Meireles</v>
       </c>
       <c r="B186" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C186" t="str">
-        <v>Analista de compras</v>
+        <v>Técnico de segurança do trabalho</v>
       </c>
       <c r="D186" t="str">
-        <v>Diretoria administrativa</v>
+        <v>Diretoria de governança</v>
       </c>
       <c r="E186" t="str">
         <v>Douradina/PR</v>
@@ -16115,16 +16162,16 @@
     </row>
     <row r="187">
       <c r="A187" t="str">
-        <v>Tatiane Damasceno Guimarães</v>
+        <v>Samuel Lacerda Siqueira</v>
       </c>
       <c r="B187" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C187" t="str">
-        <v>Analista de sistemas</v>
+        <v>Analista de compras</v>
       </c>
       <c r="D187" t="str">
-        <v>Diretoria de tecnologia da informação e inovação</v>
+        <v>Diretoria administrativa</v>
       </c>
       <c r="E187" t="str">
         <v>Douradina/PR</v>
@@ -16153,16 +16200,16 @@
     </row>
     <row r="188">
       <c r="A188" t="str">
-        <v>Daniela Rezende Nogueira</v>
+        <v>Tatiane Damasceno Guimarães</v>
       </c>
       <c r="B188" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C188" t="str">
-        <v>Analista de crédito</v>
+        <v>Analista de sistemas</v>
       </c>
       <c r="D188" t="str">
-        <v>Diretoria financeira</v>
+        <v>Diretoria de tecnologia da informação e inovação</v>
       </c>
       <c r="E188" t="str">
         <v>Douradina/PR</v>
@@ -16171,7 +16218,7 @@
         <v>Dentro do Estado</v>
       </c>
       <c r="G188" t="str">
-        <v>Supervisor regional</v>
+        <v>Supervisor de tecnologia da informação</v>
       </c>
       <c r="H188" t="str">
         <v>Até 3 anos</v>
@@ -16200,7 +16247,7 @@
     </row>
     <row r="189">
       <c r="A189" t="str">
-        <v>Bruna Pacheco Valadares</v>
+        <v>Daniela Rezende Nogueira</v>
       </c>
       <c r="B189" t="str">
         <v>Analista / Técnico</v>
@@ -16212,13 +16259,13 @@
         <v>Diretoria financeira</v>
       </c>
       <c r="E189" t="str">
-        <v>Dourados/MS</v>
+        <v>Douradina/PR</v>
       </c>
       <c r="F189" t="str">
         <v>Total (qualquer unidade)</v>
       </c>
       <c r="G189" t="str">
-        <v>Supervisor administrativo</v>
+        <v>Coordenador comercial</v>
       </c>
       <c r="H189" t="str">
         <v>Mais de 3 até 5 anos</v>
@@ -16247,16 +16294,16 @@
     </row>
     <row r="190">
       <c r="A190" t="str">
-        <v>João Pedro Guimarães Queiroz</v>
+        <v>Bruna Pacheco Valadares</v>
       </c>
       <c r="B190" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C190" t="str">
-        <v>Analista de compras</v>
+        <v>Analista de crédito</v>
       </c>
       <c r="D190" t="str">
-        <v>Diretoria administrativa</v>
+        <v>Diretoria financeira</v>
       </c>
       <c r="E190" t="str">
         <v>Dourados/MS</v>
@@ -16265,7 +16312,7 @@
         <v>Dentro do Estado</v>
       </c>
       <c r="G190" t="str">
-        <v>Gerente de riscos</v>
+        <v>Gerente de assistência</v>
       </c>
       <c r="H190" t="str">
         <v>Até 3 anos</v>
@@ -16282,25 +16329,25 @@
     </row>
     <row r="191">
       <c r="A191" t="str">
-        <v>Letícia Tavares Xavier</v>
+        <v>João Pedro Guimarães Queiroz</v>
       </c>
       <c r="B191" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C191" t="str">
-        <v>Analista administrativo</v>
+        <v>Analista de compras</v>
       </c>
       <c r="D191" t="str">
-        <v>Diretoria comercial</v>
+        <v>Diretoria administrativa</v>
       </c>
       <c r="E191" t="str">
-        <v>Douradina/PR</v>
+        <v>Dourados/MS</v>
       </c>
       <c r="F191" t="str">
         <v>Total (qualquer unidade)</v>
       </c>
       <c r="G191" t="str">
-        <v>Supervisor administrativo (despesas)</v>
+        <v>Coordenador central de compras</v>
       </c>
       <c r="H191" t="str">
         <v>Até 3 anos</v>
@@ -16309,7 +16356,7 @@
         <v>Comunicação com a diretoria</v>
       </c>
       <c r="J191" t="str">
-        <v>Administrador de redes</v>
+        <v>Supervisor comercial (Gazin Bank)</v>
       </c>
       <c r="K191" t="str">
         <v>Imediato</v>
@@ -16329,25 +16376,25 @@
     </row>
     <row r="192">
       <c r="A192" t="str">
-        <v>Yasmin Figueiredo Valadares</v>
+        <v>Letícia Tavares Xavier</v>
       </c>
       <c r="B192" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C192" t="str">
-        <v>Analista de logística</v>
+        <v>Analista administrativo</v>
       </c>
       <c r="D192" t="str">
-        <v>Diretoria de logística</v>
+        <v>Diretoria comercial</v>
       </c>
       <c r="E192" t="str">
-        <v>Dourados/MS</v>
+        <v>Douradina/PR</v>
       </c>
       <c r="F192" t="str">
         <v>Total (qualquer unidade)</v>
       </c>
       <c r="G192" t="str">
-        <v>Coordenador financeiro (financeiro)</v>
+        <v>Supervisor administrativo</v>
       </c>
       <c r="H192" t="str">
         <v>Até 3 anos</v>
@@ -16356,7 +16403,7 @@
         <v>Gestão de pessoas e feedback</v>
       </c>
       <c r="J192" t="str">
-        <v>Supervisor administrativo</v>
+        <v>Coordenador comercial</v>
       </c>
       <c r="K192" t="str">
         <v>Mais de 3 até 5 anos</v>
@@ -16376,25 +16423,25 @@
     </row>
     <row r="193">
       <c r="A193" t="str">
-        <v>Daniela Queiroz Xavier</v>
+        <v>Yasmin Figueiredo Valadares</v>
       </c>
       <c r="B193" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C193" t="str">
-        <v>Analista de crédito</v>
+        <v>Analista de logística</v>
       </c>
       <c r="D193" t="str">
-        <v>Diretoria financeira</v>
+        <v>Diretoria de logística</v>
       </c>
       <c r="E193" t="str">
-        <v>Maringá/PR</v>
+        <v>Dourados/MS</v>
       </c>
       <c r="F193" t="str">
         <v>Total (qualquer unidade)</v>
       </c>
       <c r="G193" t="str">
-        <v>Gerente financeiro</v>
+        <v>Gerente de transporte</v>
       </c>
       <c r="H193" t="str">
         <v>Mais de 3 até 5 anos</v>
@@ -16414,25 +16461,25 @@
     </row>
     <row r="194">
       <c r="A194" t="str">
-        <v>João Pedro Cardoso Jardim</v>
+        <v>Daniela Queiroz Xavier</v>
       </c>
       <c r="B194" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C194" t="str">
-        <v>Analista contábil</v>
+        <v>Analista de crédito</v>
       </c>
       <c r="D194" t="str">
-        <v>Controller</v>
+        <v>Diretoria financeira</v>
       </c>
       <c r="E194" t="str">
-        <v>Ji-Paraná/RO</v>
+        <v>Maringá/PR</v>
       </c>
       <c r="F194" t="str">
         <v>Dentro do Estado</v>
       </c>
       <c r="G194" t="str">
-        <v>Coordenador contábil/tributário</v>
+        <v>Coordenador central de compras</v>
       </c>
       <c r="H194" t="str">
         <v>Mais de 5 anos</v>
@@ -16452,25 +16499,25 @@
     </row>
     <row r="195">
       <c r="A195" t="str">
-        <v>Mariana Barreto Tavares</v>
+        <v>João Pedro Cardoso Jardim</v>
       </c>
       <c r="B195" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C195" t="str">
-        <v>Técnico de segurança do trabalho</v>
+        <v>Analista contábil</v>
       </c>
       <c r="D195" t="str">
-        <v>Diretoria de governança</v>
+        <v>Controller</v>
       </c>
       <c r="E195" t="str">
-        <v>Douradina/PR</v>
+        <v>Ji-Paraná/RO</v>
       </c>
       <c r="F195" t="str">
         <v>Total (qualquer unidade)</v>
       </c>
       <c r="G195" t="str">
-        <v>Coordenador de pessoal</v>
+        <v>Supervisor de vendas (atacado)</v>
       </c>
       <c r="H195" t="str">
         <v>Mais de 5 anos</v>
@@ -16490,16 +16537,16 @@
     </row>
     <row r="196">
       <c r="A196" t="str">
-        <v>Daniela Guimarães Valadares</v>
+        <v>Mariana Barreto Tavares</v>
       </c>
       <c r="B196" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C196" t="str">
-        <v>Analista contábil</v>
+        <v>Técnico de segurança do trabalho</v>
       </c>
       <c r="D196" t="str">
-        <v>Controller</v>
+        <v>Diretoria de governança</v>
       </c>
       <c r="E196" t="str">
         <v>Douradina/PR</v>
@@ -16519,16 +16566,16 @@
     </row>
     <row r="197">
       <c r="A197" t="str">
-        <v>Paula Meireles Guimarães</v>
+        <v>Daniela Guimarães Valadares</v>
       </c>
       <c r="B197" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C197" t="str">
-        <v>Analista administrativo</v>
+        <v>Analista contábil</v>
       </c>
       <c r="D197" t="str">
-        <v>Diretoria comercial</v>
+        <v>Controller</v>
       </c>
       <c r="E197" t="str">
         <v>Douradina/PR</v>
@@ -16537,7 +16584,7 @@
         <v>Total (qualquer unidade)</v>
       </c>
       <c r="G197" t="str">
-        <v>Supervisor administrativo</v>
+        <v>Coordenador de estoque</v>
       </c>
       <c r="H197" t="str">
         <v>Até 3 anos</v>
@@ -16557,16 +16604,16 @@
     </row>
     <row r="198">
       <c r="A198" t="str">
-        <v>Bruna Guimarães Queiroz</v>
+        <v>Paula Meireles Guimarães</v>
       </c>
       <c r="B198" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C198" t="str">
-        <v>Analista de recursos humanos</v>
+        <v>Analista administrativo</v>
       </c>
       <c r="D198" t="str">
-        <v>Gerente geral de recursos humanos</v>
+        <v>Diretoria comercial</v>
       </c>
       <c r="E198" t="str">
         <v>Douradina/PR</v>
@@ -16575,7 +16622,7 @@
         <v>Matriz (Douradina/PR)</v>
       </c>
       <c r="G198" t="str">
-        <v>Supervisor de contabilidade</v>
+        <v>Supervisor administrativo (despesas)</v>
       </c>
       <c r="H198" t="str">
         <v>Até 3 anos</v>
@@ -16584,7 +16631,7 @@
         <v>Negociação com fornecedores</v>
       </c>
       <c r="J198" t="str">
-        <v>Coordenador central de compras</v>
+        <v>Coordenador administrativo (assessoria)</v>
       </c>
       <c r="K198" t="str">
         <v>Até 3 anos</v>
@@ -16604,16 +16651,16 @@
     </row>
     <row r="199">
       <c r="A199" t="str">
-        <v>Mariana Meireles Esteves</v>
+        <v>Bruna Guimarães Queiroz</v>
       </c>
       <c r="B199" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C199" t="str">
-        <v>Técnico de segurança do trabalho</v>
+        <v>Analista de recursos humanos</v>
       </c>
       <c r="D199" t="str">
-        <v>Diretoria de governança</v>
+        <v>Gerente geral de recursos humanos</v>
       </c>
       <c r="E199" t="str">
         <v>Douradina/PR</v>
@@ -16622,7 +16669,7 @@
         <v>Dentro do Estado</v>
       </c>
       <c r="G199" t="str">
-        <v>Supervisor administrativo (administração geral)</v>
+        <v>Coordenador central de compras</v>
       </c>
       <c r="H199" t="str">
         <v>Até 3 anos</v>
@@ -16651,16 +16698,16 @@
     </row>
     <row r="200">
       <c r="A200" t="str">
-        <v>Murilo Zanella Valadares</v>
+        <v>Mariana Meireles Esteves</v>
       </c>
       <c r="B200" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C200" t="str">
-        <v>Analista administrativo</v>
+        <v>Técnico de segurança do trabalho</v>
       </c>
       <c r="D200" t="str">
-        <v>Diretoria comercial</v>
+        <v>Diretoria de governança</v>
       </c>
       <c r="E200" t="str">
         <v>Douradina/PR</v>
@@ -16689,19 +16736,19 @@
     </row>
     <row r="201">
       <c r="A201" t="str">
-        <v>Amanda Zanella Guimarães</v>
+        <v>Murilo Zanella Valadares</v>
       </c>
       <c r="B201" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C201" t="str">
-        <v>Analista de recursos humanos</v>
+        <v>Analista administrativo</v>
       </c>
       <c r="D201" t="str">
-        <v>Gerente geral de recursos humanos</v>
+        <v>Diretoria comercial</v>
       </c>
       <c r="E201" t="str">
-        <v>Maringá/PR</v>
+        <v>Douradina/PR</v>
       </c>
       <c r="F201" t="str">
         <v>Dentro do Estado</v>
@@ -16718,25 +16765,25 @@
     </row>
     <row r="202">
       <c r="A202" t="str">
-        <v>Gabriela Valadares Siqueira</v>
+        <v>Amanda Zanella Guimarães</v>
       </c>
       <c r="B202" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C202" t="str">
-        <v>Técnico de segurança do trabalho</v>
+        <v>Analista de recursos humanos</v>
       </c>
       <c r="D202" t="str">
-        <v>Diretoria de governança</v>
+        <v>Gerente geral de recursos humanos</v>
       </c>
       <c r="E202" t="str">
-        <v>Douradina/PR</v>
+        <v>Maringá/PR</v>
       </c>
       <c r="F202" t="str">
         <v>Matriz (Douradina/PR)</v>
       </c>
       <c r="G202" t="str">
-        <v>Coordenador de transporte</v>
+        <v>Supervisor regional</v>
       </c>
       <c r="H202" t="str">
         <v>Mais de 5 anos</v>
@@ -16756,16 +16803,16 @@
     </row>
     <row r="203">
       <c r="A203" t="str">
-        <v>Caio Cardoso Jardim</v>
+        <v>Gabriela Valadares Siqueira</v>
       </c>
       <c r="B203" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C203" t="str">
-        <v>Analista de logística</v>
+        <v>Técnico de segurança do trabalho</v>
       </c>
       <c r="D203" t="str">
-        <v>Diretoria de logística</v>
+        <v>Diretoria de governança</v>
       </c>
       <c r="E203" t="str">
         <v>Douradina/PR</v>
@@ -16783,7 +16830,7 @@
         <v>Planejamento estratégico</v>
       </c>
       <c r="J203" t="str">
-        <v>Supervisor de propaganda</v>
+        <v>Administrador de redes</v>
       </c>
       <c r="K203" t="str">
         <v>Mais de 3 até 5 anos</v>
@@ -16803,25 +16850,25 @@
     </row>
     <row r="204">
       <c r="A204" t="str">
-        <v>Wellington Guimarães Xavier</v>
+        <v>Caio Cardoso Jardim</v>
       </c>
       <c r="B204" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C204" t="str">
-        <v>Técnico de segurança do trabalho</v>
+        <v>Analista de logística</v>
       </c>
       <c r="D204" t="str">
-        <v>Diretoria de governança</v>
+        <v>Diretoria de logística</v>
       </c>
       <c r="E204" t="str">
-        <v>Dourados/MS</v>
+        <v>Douradina/PR</v>
       </c>
       <c r="F204" t="str">
         <v>Dentro do Estado</v>
       </c>
       <c r="G204" t="str">
-        <v>Coordenador de comunicação</v>
+        <v>Supervisor administrativo (governança)</v>
       </c>
       <c r="H204" t="str">
         <v>Mais de 5 anos</v>
@@ -16841,25 +16888,25 @@
     </row>
     <row r="205">
       <c r="A205" t="str">
-        <v>Felipe Holanda Guimarães</v>
+        <v>Wellington Guimarães Xavier</v>
       </c>
       <c r="B205" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C205" t="str">
-        <v>Analista de crédito</v>
+        <v>Técnico de segurança do trabalho</v>
       </c>
       <c r="D205" t="str">
-        <v>Diretoria financeira</v>
+        <v>Diretoria de governança</v>
       </c>
       <c r="E205" t="str">
-        <v>Douradina/PR</v>
+        <v>Dourados/MS</v>
       </c>
       <c r="F205" t="str">
         <v>Local atual</v>
       </c>
       <c r="G205" t="str">
-        <v>Supervisor de vendas (atacado)</v>
+        <v>Supervisor de licitação</v>
       </c>
       <c r="H205" t="str">
         <v>Até 3 anos</v>
@@ -16879,16 +16926,16 @@
     </row>
     <row r="206">
       <c r="A206" t="str">
-        <v>Letícia Zanella Damasceno</v>
+        <v>Felipe Holanda Guimarães</v>
       </c>
       <c r="B206" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C206" t="str">
-        <v>Analista contábil</v>
+        <v>Analista de crédito</v>
       </c>
       <c r="D206" t="str">
-        <v>Controller</v>
+        <v>Diretoria financeira</v>
       </c>
       <c r="E206" t="str">
         <v>Douradina/PR</v>
@@ -16908,16 +16955,16 @@
     </row>
     <row r="207">
       <c r="A207" t="str">
-        <v>Amanda Siqueira Holanda</v>
+        <v>Letícia Zanella Damasceno</v>
       </c>
       <c r="B207" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C207" t="str">
-        <v>Analista de crédito</v>
+        <v>Analista contábil</v>
       </c>
       <c r="D207" t="str">
-        <v>Diretoria financeira</v>
+        <v>Controller</v>
       </c>
       <c r="E207" t="str">
         <v>Douradina/PR</v>
@@ -16926,7 +16973,7 @@
         <v>Total (qualquer unidade)</v>
       </c>
       <c r="G207" t="str">
-        <v>Supervisor de licitação</v>
+        <v>Supervisor administrativo (expansão)</v>
       </c>
       <c r="H207" t="str">
         <v>Até 3 anos</v>
@@ -16946,16 +16993,16 @@
     </row>
     <row r="208">
       <c r="A208" t="str">
-        <v>Vitor Guimarães Valadares</v>
+        <v>Amanda Siqueira Holanda</v>
       </c>
       <c r="B208" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C208" t="str">
-        <v>Analista de logística</v>
+        <v>Analista de crédito</v>
       </c>
       <c r="D208" t="str">
-        <v>Diretoria de logística</v>
+        <v>Diretoria financeira</v>
       </c>
       <c r="E208" t="str">
         <v>Douradina/PR</v>
@@ -16964,7 +17011,7 @@
         <v>Local atual</v>
       </c>
       <c r="G208" t="str">
-        <v>Coordenador de transporte</v>
+        <v>Supervisor comercial (Gazin Bank)</v>
       </c>
       <c r="H208" t="str">
         <v>Mais de 3 até 5 anos</v>
@@ -16984,7 +17031,7 @@
     </row>
     <row r="209">
       <c r="A209" t="str">
-        <v>Rafaela Guimarães Esteves</v>
+        <v>Vitor Guimarães Valadares</v>
       </c>
       <c r="B209" t="str">
         <v>Analista / Técnico</v>
@@ -16996,7 +17043,7 @@
         <v>Diretoria de logística</v>
       </c>
       <c r="E209" t="str">
-        <v>Rio Branco/AC</v>
+        <v>Douradina/PR</v>
       </c>
       <c r="F209" t="str">
         <v>Matriz (Douradina/PR)</v>
@@ -17022,25 +17069,25 @@
     </row>
     <row r="210">
       <c r="A210" t="str">
-        <v>Bruna Esteves Pacheco</v>
+        <v>Rafaela Guimarães Esteves</v>
       </c>
       <c r="B210" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C210" t="str">
-        <v>Analista de recursos humanos</v>
+        <v>Analista de logística</v>
       </c>
       <c r="D210" t="str">
-        <v>Gerente geral de recursos humanos</v>
+        <v>Diretoria de logística</v>
       </c>
       <c r="E210" t="str">
-        <v>Douradina/PR</v>
+        <v>Rio Branco/AC</v>
       </c>
       <c r="F210" t="str">
         <v>Local atual</v>
       </c>
       <c r="G210" t="str">
-        <v>Supervisor de e-commerce (atacado)</v>
+        <v>Supervisor administrativo (atacado)</v>
       </c>
       <c r="H210" t="str">
         <v>Mais de 3 até 5 anos</v>
@@ -17060,7 +17107,7 @@
     </row>
     <row r="211">
       <c r="A211" t="str">
-        <v>Heitor Jardim Valadares</v>
+        <v>Bruna Esteves Pacheco</v>
       </c>
       <c r="B211" t="str">
         <v>Analista / Técnico</v>
@@ -17087,7 +17134,7 @@
         <v>Formação técnica específica da área</v>
       </c>
       <c r="J211" t="str">
-        <v>Gerente de espumação</v>
+        <v>Gerente de indústria</v>
       </c>
       <c r="K211" t="str">
         <v>Até 3 anos</v>
@@ -17107,25 +17154,25 @@
     </row>
     <row r="212">
       <c r="A212" t="str">
-        <v>Isabela Pacheco Albuquerque</v>
+        <v>Heitor Jardim Valadares</v>
       </c>
       <c r="B212" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C212" t="str">
-        <v>Analista de compras</v>
+        <v>Analista de recursos humanos</v>
       </c>
       <c r="D212" t="str">
-        <v>Diretoria administrativa</v>
+        <v>Gerente geral de recursos humanos</v>
       </c>
       <c r="E212" t="str">
-        <v>Ji-Paraná/RO</v>
+        <v>Douradina/PR</v>
       </c>
       <c r="F212" t="str">
         <v>Dentro do Estado</v>
       </c>
       <c r="G212" t="str">
-        <v>Supervisor de varejo</v>
+        <v>Supervisor administrativo (e-commerce)</v>
       </c>
       <c r="H212" t="str">
         <v>Mais de 3 até 5 anos</v>
@@ -17145,25 +17192,25 @@
     </row>
     <row r="213">
       <c r="A213" t="str">
-        <v>Paula Cardoso Barreto</v>
+        <v>Isabela Pacheco Albuquerque</v>
       </c>
       <c r="B213" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C213" t="str">
-        <v>Técnico de segurança do trabalho</v>
+        <v>Analista de compras</v>
       </c>
       <c r="D213" t="str">
-        <v>Diretoria de governança</v>
+        <v>Diretoria administrativa</v>
       </c>
       <c r="E213" t="str">
-        <v>Douradina/PR</v>
+        <v>Ji-Paraná/RO</v>
       </c>
       <c r="F213" t="str">
         <v>Dentro do Estado</v>
       </c>
       <c r="G213" t="str">
-        <v>Supervisor administrativo (e-commerce)</v>
+        <v>Coordenador administrativo (assessoria)</v>
       </c>
       <c r="H213" t="str">
         <v>Mais de 5 anos</v>
@@ -17183,19 +17230,19 @@
     </row>
     <row r="214">
       <c r="A214" t="str">
-        <v>Samuel Figueiredo Pacheco</v>
+        <v>Paula Cardoso Barreto</v>
       </c>
       <c r="B214" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C214" t="str">
-        <v>Analista contábil</v>
+        <v>Técnico de segurança do trabalho</v>
       </c>
       <c r="D214" t="str">
-        <v>Controller</v>
+        <v>Diretoria de governança</v>
       </c>
       <c r="E214" t="str">
-        <v>Goiânia/GO</v>
+        <v>Douradina/PR</v>
       </c>
       <c r="F214" t="str">
         <v>Local atual</v>
@@ -17210,7 +17257,7 @@
         <v>Gestão de indicadores e metas</v>
       </c>
       <c r="J214" t="str">
-        <v>Supervisor contábil</v>
+        <v>Supervisor de e-commerce (atacado)</v>
       </c>
       <c r="K214" t="str">
         <v>Mais de 3 até 5 anos</v>
@@ -17230,25 +17277,25 @@
     </row>
     <row r="215">
       <c r="A215" t="str">
-        <v>Bruna Cardoso Damasceno</v>
+        <v>Samuel Figueiredo Pacheco</v>
       </c>
       <c r="B215" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C215" t="str">
-        <v>Analista de recursos humanos</v>
+        <v>Analista contábil</v>
       </c>
       <c r="D215" t="str">
-        <v>Gerente geral de recursos humanos</v>
+        <v>Controller</v>
       </c>
       <c r="E215" t="str">
-        <v>Douradina/PR</v>
+        <v>Goiânia/GO</v>
       </c>
       <c r="F215" t="str">
         <v>Total (qualquer unidade)</v>
       </c>
       <c r="G215" t="str">
-        <v>Supervisor de desenvolvimento humano</v>
+        <v>Supervisor regional</v>
       </c>
       <c r="H215" t="str">
         <v>Até 3 anos</v>
@@ -17268,16 +17315,16 @@
     </row>
     <row r="216">
       <c r="A216" t="str">
-        <v>Mariana Holanda Siqueira</v>
+        <v>Bruna Cardoso Damasceno</v>
       </c>
       <c r="B216" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C216" t="str">
-        <v>Analista contábil</v>
+        <v>Analista de recursos humanos</v>
       </c>
       <c r="D216" t="str">
-        <v>Controller</v>
+        <v>Gerente geral de recursos humanos</v>
       </c>
       <c r="E216" t="str">
         <v>Douradina/PR</v>
@@ -17286,7 +17333,7 @@
         <v>Matriz (Douradina/PR)</v>
       </c>
       <c r="G216" t="str">
-        <v>Coordenador de orçamento</v>
+        <v>Supervisor de contabilidade</v>
       </c>
       <c r="H216" t="str">
         <v>Imediato</v>
@@ -17295,7 +17342,7 @@
         <v>Gestão de pessoas e feedback</v>
       </c>
       <c r="J216" t="str">
-        <v>Supervisor administrativo (governança)</v>
+        <v>Administrador de redes</v>
       </c>
       <c r="K216" t="str">
         <v>Mais de 3 até 5 anos</v>
@@ -17315,16 +17362,16 @@
     </row>
     <row r="217">
       <c r="A217" t="str">
-        <v>Murilo Zanella Albuquerque</v>
+        <v>Mariana Holanda Siqueira</v>
       </c>
       <c r="B217" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C217" t="str">
-        <v>Técnico de segurança do trabalho</v>
+        <v>Analista contábil</v>
       </c>
       <c r="D217" t="str">
-        <v>Diretoria de governança</v>
+        <v>Controller</v>
       </c>
       <c r="E217" t="str">
         <v>Douradina/PR</v>
@@ -17333,7 +17380,7 @@
         <v>Local atual</v>
       </c>
       <c r="G217" t="str">
-        <v>Coordenador administrativo (governança)</v>
+        <v>Supervisor de varejo</v>
       </c>
       <c r="H217" t="str">
         <v>Até 3 anos</v>
@@ -17362,19 +17409,19 @@
     </row>
     <row r="218">
       <c r="A218" t="str">
-        <v>João Pedro Pacheco Meireles</v>
+        <v>Murilo Zanella Albuquerque</v>
       </c>
       <c r="B218" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C218" t="str">
-        <v>Analista de sistemas</v>
+        <v>Técnico de segurança do trabalho</v>
       </c>
       <c r="D218" t="str">
-        <v>Diretoria de tecnologia da informação e inovação</v>
+        <v>Diretoria de governança</v>
       </c>
       <c r="E218" t="str">
-        <v>Maringá/PR</v>
+        <v>Douradina/PR</v>
       </c>
       <c r="F218" t="str">
         <v>Dentro do Estado</v>
@@ -17391,19 +17438,19 @@
     </row>
     <row r="219">
       <c r="A219" t="str">
-        <v>Gabriela Zanella Pacheco</v>
+        <v>João Pedro Pacheco Meireles</v>
       </c>
       <c r="B219" t="str">
         <v>Analista / Técnico</v>
       </c>
       <c r="C219" t="str">
-        <v>Analista de logística</v>
+        <v>Analista de sistemas</v>
       </c>
       <c r="D219" t="str">
-        <v>Diretoria de logística</v>
+        <v>Diretoria de tecnologia da informação e inovação</v>
       </c>
       <c r="E219" t="str">
-        <v>Douradina/PR</v>
+        <v>Maringá/PR</v>
       </c>
       <c r="F219" t="str">
         <v>Total (qualquer unidade)</v>
@@ -17418,9 +17465,38 @@
         <v>Não</v>
       </c>
     </row>
+    <row r="220">
+      <c r="A220" t="str">
+        <v>Gabriela Zanella Pacheco</v>
+      </c>
+      <c r="B220" t="str">
+        <v>Analista / Técnico</v>
+      </c>
+      <c r="C220" t="str">
+        <v>Analista de logística</v>
+      </c>
+      <c r="D220" t="str">
+        <v>Diretoria de logística</v>
+      </c>
+      <c r="E220" t="str">
+        <v>Douradina/PR</v>
+      </c>
+      <c r="F220" t="str">
+        <v>Matriz (Douradina/PR)</v>
+      </c>
+      <c r="M220" t="str">
+        <v>Conversado, sem plano formal</v>
+      </c>
+      <c r="P220" t="str">
+        <v>Empregado Sólido / Responsável</v>
+      </c>
+      <c r="Q220" t="str">
+        <v>Não</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R219"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R220"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -17594,7 +17670,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H101"/>
+  <dimension ref="A1:H102"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -19579,7 +19655,7 @@
         <v/>
       </c>
       <c r="H76" t="str">
-        <v>Gerente geral do atacado</v>
+        <v>Gerente geral de recursos humanos</v>
       </c>
     </row>
     <row r="77">
@@ -19605,7 +19681,7 @@
         <v/>
       </c>
       <c r="H77" t="str">
-        <v>Gerente geral do varejo</v>
+        <v>Gerente geral do atacado</v>
       </c>
     </row>
     <row r="78">
@@ -19631,7 +19707,7 @@
         <v/>
       </c>
       <c r="H78" t="str">
-        <v>Gerente jurídico</v>
+        <v>Gerente geral do varejo</v>
       </c>
     </row>
     <row r="79">
@@ -19657,7 +19733,7 @@
         <v/>
       </c>
       <c r="H79" t="str">
-        <v>Gerente regional</v>
+        <v>Gerente jurídico</v>
       </c>
     </row>
     <row r="80">
@@ -19683,7 +19759,7 @@
         <v/>
       </c>
       <c r="H80" t="str">
-        <v>Supervisor administrativo</v>
+        <v>Gerente regional</v>
       </c>
     </row>
     <row r="81">
@@ -19709,7 +19785,7 @@
         <v/>
       </c>
       <c r="H81" t="str">
-        <v>Supervisor administrativo (administração geral)</v>
+        <v>Supervisor administrativo</v>
       </c>
     </row>
     <row r="82">
@@ -19735,7 +19811,7 @@
         <v/>
       </c>
       <c r="H82" t="str">
-        <v>Supervisor administrativo (atacado)</v>
+        <v>Supervisor administrativo (administração geral)</v>
       </c>
     </row>
     <row r="83">
@@ -19761,7 +19837,7 @@
         <v/>
       </c>
       <c r="H83" t="str">
-        <v>Supervisor administrativo (despesas)</v>
+        <v>Supervisor administrativo (atacado)</v>
       </c>
     </row>
     <row r="84">
@@ -19787,7 +19863,7 @@
         <v/>
       </c>
       <c r="H84" t="str">
-        <v>Supervisor administrativo (e-commerce)</v>
+        <v>Supervisor administrativo (despesas)</v>
       </c>
     </row>
     <row r="85">
@@ -19813,7 +19889,7 @@
         <v/>
       </c>
       <c r="H85" t="str">
-        <v>Supervisor administrativo (expansão)</v>
+        <v>Supervisor administrativo (e-commerce)</v>
       </c>
     </row>
     <row r="86">
@@ -19839,7 +19915,7 @@
         <v/>
       </c>
       <c r="H86" t="str">
-        <v>Supervisor administrativo (gestão de pessoas)</v>
+        <v>Supervisor administrativo (expansão)</v>
       </c>
     </row>
     <row r="87">
@@ -19865,7 +19941,7 @@
         <v/>
       </c>
       <c r="H87" t="str">
-        <v>Supervisor administrativo (governança)</v>
+        <v>Supervisor administrativo (gestão de pessoas)</v>
       </c>
     </row>
     <row r="88">
@@ -19891,7 +19967,7 @@
         <v/>
       </c>
       <c r="H88" t="str">
-        <v>Supervisor comercial (Gazin Bank)</v>
+        <v>Supervisor administrativo (governança)</v>
       </c>
     </row>
     <row r="89">
@@ -19917,7 +19993,7 @@
         <v/>
       </c>
       <c r="H89" t="str">
-        <v>Supervisor contábil</v>
+        <v>Supervisor comercial (Gazin Bank)</v>
       </c>
     </row>
     <row r="90">
@@ -19943,7 +20019,7 @@
         <v/>
       </c>
       <c r="H90" t="str">
-        <v>Supervisor de contabilidade</v>
+        <v>Supervisor contábil</v>
       </c>
     </row>
     <row r="91">
@@ -19969,7 +20045,7 @@
         <v/>
       </c>
       <c r="H91" t="str">
-        <v>Supervisor de desenvolvimento humano</v>
+        <v>Supervisor de contabilidade</v>
       </c>
     </row>
     <row r="92">
@@ -19995,7 +20071,7 @@
         <v/>
       </c>
       <c r="H92" t="str">
-        <v>Supervisor de e-commerce (atacado)</v>
+        <v>Supervisor de desenvolvimento humano</v>
       </c>
     </row>
     <row r="93">
@@ -20021,7 +20097,7 @@
         <v/>
       </c>
       <c r="H93" t="str">
-        <v>Supervisor de licitação</v>
+        <v>Supervisor de e-commerce (atacado)</v>
       </c>
     </row>
     <row r="94">
@@ -20047,7 +20123,7 @@
         <v/>
       </c>
       <c r="H94" t="str">
-        <v>Supervisor de operação tributária</v>
+        <v>Supervisor de licitação</v>
       </c>
     </row>
     <row r="95">
@@ -20073,7 +20149,7 @@
         <v/>
       </c>
       <c r="H95" t="str">
-        <v>Supervisor de propaganda</v>
+        <v>Supervisor de operação tributária</v>
       </c>
     </row>
     <row r="96">
@@ -20099,7 +20175,7 @@
         <v/>
       </c>
       <c r="H96" t="str">
-        <v>Supervisor de recrutamento e seleção</v>
+        <v>Supervisor de propaganda</v>
       </c>
     </row>
     <row r="97">
@@ -20125,7 +20201,7 @@
         <v/>
       </c>
       <c r="H97" t="str">
-        <v>Supervisor de tecnologia da informação</v>
+        <v>Supervisor de recrutamento e seleção</v>
       </c>
     </row>
     <row r="98">
@@ -20151,7 +20227,7 @@
         <v/>
       </c>
       <c r="H98" t="str">
-        <v>Supervisor de varejo</v>
+        <v>Supervisor de tecnologia da informação</v>
       </c>
     </row>
     <row r="99">
@@ -20177,7 +20253,7 @@
         <v/>
       </c>
       <c r="H99" t="str">
-        <v>Supervisor de vendas (atacado)</v>
+        <v>Supervisor de varejo</v>
       </c>
     </row>
     <row r="100">
@@ -20203,7 +20279,7 @@
         <v/>
       </c>
       <c r="H100" t="str">
-        <v>Supervisor regional</v>
+        <v>Supervisor de vendas (atacado)</v>
       </c>
     </row>
     <row r="101">
@@ -20229,12 +20305,38 @@
         <v/>
       </c>
       <c r="H101" t="str">
+        <v>Supervisor regional</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v/>
+      </c>
+      <c r="B102" t="str">
+        <v/>
+      </c>
+      <c r="C102" t="str">
+        <v/>
+      </c>
+      <c r="D102" t="str">
+        <v/>
+      </c>
+      <c r="E102" t="str">
+        <v/>
+      </c>
+      <c r="F102" t="str">
+        <v/>
+      </c>
+      <c r="G102" t="str">
+        <v/>
+      </c>
+      <c r="H102" t="str">
         <v>Tech Lead</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H101"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H102"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>